<commit_message>
feat: consolidate team view into single sheet and update member stats
#VERCEL_SKIP
</commit_message>
<xml_diff>
--- a/public/Detailed Team View.xlsx
+++ b/public/Detailed Team View.xlsx
@@ -3,12 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="All Members" sheetId="1" r:id="rId1"/>
-    <sheet name="Role Summary" sheetId="2" r:id="rId2"/>
-    <sheet name="Release Summary" sheetId="3" r:id="rId3"/>
-    <sheet name="Valuestream Summary" sheetId="4" r:id="rId4"/>
-    <sheet name="FPL Members" sheetId="5" r:id="rId5"/>
-    <sheet name="Statistics" sheetId="6" r:id="rId6"/>
+    <sheet name="Team Members" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -466,6 +461,9 @@
       <c r="G2" t="str">
         <v>Program Leadership</v>
       </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
       <c r="I2" t="str">
         <v>No</v>
       </c>
@@ -492,6 +490,9 @@
       <c r="G3" t="str">
         <v>Program Leadership</v>
       </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
       <c r="I3" t="str">
         <v>No</v>
       </c>
@@ -518,6 +519,9 @@
       <c r="G4" t="str">
         <v>Program Leadership</v>
       </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
       <c r="I4" t="str">
         <v>No</v>
       </c>
@@ -544,6 +548,9 @@
       <c r="G5" t="str">
         <v>Program Leadership</v>
       </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
       <c r="I5" t="str">
         <v>No</v>
       </c>
@@ -570,6 +577,9 @@
       <c r="G6" t="str">
         <v>Architecture</v>
       </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
       <c r="I6" t="str">
         <v>No</v>
       </c>
@@ -596,6 +606,9 @@
       <c r="G7" t="str">
         <v>Architecture</v>
       </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
       <c r="I7" t="str">
         <v>No</v>
       </c>
@@ -622,6 +635,9 @@
       <c r="G8" t="str">
         <v>Architecture</v>
       </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
       <c r="I8" t="str">
         <v>No</v>
       </c>
@@ -648,6 +664,9 @@
       <c r="G9" t="str">
         <v>PMO</v>
       </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
       <c r="I9" t="str">
         <v>No</v>
       </c>
@@ -674,6 +693,9 @@
       <c r="G10" t="str">
         <v>PMO</v>
       </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
       <c r="I10" t="str">
         <v>No</v>
       </c>
@@ -700,6 +722,9 @@
       <c r="G11" t="str">
         <v>PMO</v>
       </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
       <c r="I11" t="str">
         <v>No</v>
       </c>
@@ -726,6 +751,9 @@
       <c r="G12" t="str">
         <v>Integration</v>
       </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
       <c r="I12" t="str">
         <v>No</v>
       </c>
@@ -752,6 +780,9 @@
       <c r="G13" t="str">
         <v>Integration</v>
       </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
       <c r="I13" t="str">
         <v>No</v>
       </c>
@@ -778,6 +809,9 @@
       <c r="G14" t="str">
         <v>Integration</v>
       </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
       <c r="I14" t="str">
         <v>No</v>
       </c>
@@ -804,6 +838,9 @@
       <c r="G15" t="str">
         <v>Integration</v>
       </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
       <c r="I15" t="str">
         <v>No</v>
       </c>
@@ -830,6 +867,9 @@
       <c r="G16" t="str">
         <v>DevOps</v>
       </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
       <c r="I16" t="str">
         <v>No</v>
       </c>
@@ -856,6 +896,9 @@
       <c r="G17" t="str">
         <v>DevOps</v>
       </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
       <c r="I17" t="str">
         <v>No</v>
       </c>
@@ -882,6 +925,9 @@
       <c r="G18" t="str">
         <v>DevOps</v>
       </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
       <c r="I18" t="str">
         <v>No</v>
       </c>
@@ -908,6 +954,9 @@
       <c r="G19" t="str">
         <v>DevOps</v>
       </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
       <c r="I19" t="str">
         <v>No</v>
       </c>
@@ -934,6 +983,9 @@
       <c r="G20" t="str">
         <v>DevOps</v>
       </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
       <c r="I20" t="str">
         <v>No</v>
       </c>
@@ -960,6 +1012,9 @@
       <c r="G21" t="str">
         <v>DevOps</v>
       </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
       <c r="I21" t="str">
         <v>No</v>
       </c>
@@ -986,6 +1041,9 @@
       <c r="G22" t="str">
         <v>DevOps</v>
       </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
       <c r="I22" t="str">
         <v>No</v>
       </c>
@@ -1012,6 +1070,9 @@
       <c r="G23" t="str">
         <v>Windsurf/Performance</v>
       </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
       <c r="I23" t="str">
         <v>No</v>
       </c>
@@ -1038,6 +1099,9 @@
       <c r="G24" t="str">
         <v>Windsurf/Performance</v>
       </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
       <c r="I24" t="str">
         <v>No</v>
       </c>
@@ -1064,6 +1128,9 @@
       <c r="G25" t="str">
         <v>Interactions/Search | Correspondence/360s/PEXT/Account Maintenance</v>
       </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
       <c r="I25" t="str">
         <v>No</v>
       </c>
@@ -1090,6 +1157,9 @@
       <c r="G26" t="str">
         <v>Interactions/Search</v>
       </c>
+      <c r="H26" t="str">
+        <v/>
+      </c>
       <c r="I26" t="str">
         <v>No</v>
       </c>
@@ -1116,6 +1186,9 @@
       <c r="G27" t="str">
         <v>Interactions/Search</v>
       </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
       <c r="I27" t="str">
         <v>No</v>
       </c>
@@ -1142,6 +1215,9 @@
       <c r="G28" t="str">
         <v>Move In/Move Out/Transfer</v>
       </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
       <c r="I28" t="str">
         <v>No</v>
       </c>
@@ -1168,6 +1244,9 @@
       <c r="G29" t="str">
         <v>Move In/Move Out/Transfer | Multi Move In/Transfer/Amend</v>
       </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
       <c r="I29" t="str">
         <v>No</v>
       </c>
@@ -1194,6 +1273,9 @@
       <c r="G30" t="str">
         <v>Move In/Move Out/Transfer</v>
       </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
       <c r="I30" t="str">
         <v>No</v>
       </c>
@@ -1220,6 +1302,9 @@
       <c r="G31" t="str">
         <v>Move In/Move Out/Transfer</v>
       </c>
+      <c r="H31" t="str">
+        <v/>
+      </c>
       <c r="I31" t="str">
         <v>No</v>
       </c>
@@ -1246,6 +1331,9 @@
       <c r="G32" t="str">
         <v>Account Maintenance | Customer ID &amp; Fraud</v>
       </c>
+      <c r="H32" t="str">
+        <v/>
+      </c>
       <c r="I32" t="str">
         <v>No</v>
       </c>
@@ -1272,6 +1360,9 @@
       <c r="G33" t="str">
         <v>Account Maintenance</v>
       </c>
+      <c r="H33" t="str">
+        <v/>
+      </c>
       <c r="I33" t="str">
         <v>No</v>
       </c>
@@ -1298,6 +1389,9 @@
       <c r="G34" t="str">
         <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
       <c r="I34" t="str">
         <v>No</v>
       </c>
@@ -1324,6 +1418,9 @@
       <c r="G35" t="str">
         <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
       <c r="I35" t="str">
         <v>No</v>
       </c>
@@ -1350,6 +1447,9 @@
       <c r="G36" t="str">
         <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
       <c r="I36" t="str">
         <v>No</v>
       </c>
@@ -1376,6 +1476,9 @@
       <c r="G37" t="str">
         <v>Case Management</v>
       </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
       <c r="I37" t="str">
         <v>No</v>
       </c>
@@ -1402,6 +1505,9 @@
       <c r="G38" t="str">
         <v>Case Management</v>
       </c>
+      <c r="H38" t="str">
+        <v/>
+      </c>
       <c r="I38" t="str">
         <v>No</v>
       </c>
@@ -1428,6 +1534,9 @@
       <c r="G39" t="str">
         <v>Case Management</v>
       </c>
+      <c r="H39" t="str">
+        <v/>
+      </c>
       <c r="I39" t="str">
         <v>No</v>
       </c>
@@ -1454,6 +1563,9 @@
       <c r="G40" t="str">
         <v>Case Management</v>
       </c>
+      <c r="H40" t="str">
+        <v/>
+      </c>
       <c r="I40" t="str">
         <v>No</v>
       </c>
@@ -1480,6 +1592,9 @@
       <c r="G41" t="str">
         <v>QA - All Value Streams</v>
       </c>
+      <c r="H41" t="str">
+        <v/>
+      </c>
       <c r="I41" t="str">
         <v>No</v>
       </c>
@@ -1488,6 +1603,9 @@
       <c r="A42" t="str">
         <v>Maneesha</v>
       </c>
+      <c r="B42" t="str">
+        <v/>
+      </c>
       <c r="C42" t="str">
         <v>Infosys</v>
       </c>
@@ -1502,6 +1620,9 @@
       </c>
       <c r="G42" t="str">
         <v>Move In/Move Out/Transfer</v>
+      </c>
+      <c r="H42" t="str">
+        <v/>
       </c>
       <c r="I42" t="str">
         <v>No</v>
@@ -1529,6 +1650,9 @@
       <c r="G43" t="str">
         <v>Move In/Move Out</v>
       </c>
+      <c r="H43" t="str">
+        <v/>
+      </c>
       <c r="I43" t="str">
         <v>No</v>
       </c>
@@ -1555,6 +1679,9 @@
       <c r="G44" t="str">
         <v>Move In/Transfer</v>
       </c>
+      <c r="H44" t="str">
+        <v/>
+      </c>
       <c r="I44" t="str">
         <v>No</v>
       </c>
@@ -1581,6 +1708,9 @@
       <c r="G45" t="str">
         <v>Move Out/Transfer</v>
       </c>
+      <c r="H45" t="str">
+        <v/>
+      </c>
       <c r="I45" t="str">
         <v>No</v>
       </c>
@@ -1589,6 +1719,9 @@
       <c r="A46" t="str">
         <v>Venugopal Sinde</v>
       </c>
+      <c r="B46" t="str">
+        <v/>
+      </c>
       <c r="C46" t="str">
         <v>Infosys</v>
       </c>
@@ -1603,6 +1736,9 @@
       </c>
       <c r="G46" t="str">
         <v>Move In/Move Out</v>
+      </c>
+      <c r="H46" t="str">
+        <v/>
       </c>
       <c r="I46" t="str">
         <v>No</v>
@@ -1630,6 +1766,9 @@
       <c r="G47" t="str">
         <v>Transfer</v>
       </c>
+      <c r="H47" t="str">
+        <v/>
+      </c>
       <c r="I47" t="str">
         <v>No</v>
       </c>
@@ -1656,6 +1795,9 @@
       <c r="G48" t="str">
         <v>Move In</v>
       </c>
+      <c r="H48" t="str">
+        <v/>
+      </c>
       <c r="I48" t="str">
         <v>No</v>
       </c>
@@ -1682,6 +1824,9 @@
       <c r="G49" t="str">
         <v>Move Out</v>
       </c>
+      <c r="H49" t="str">
+        <v/>
+      </c>
       <c r="I49" t="str">
         <v>No</v>
       </c>
@@ -1690,6 +1835,9 @@
       <c r="A50" t="str">
         <v>Keerthana Manjunath</v>
       </c>
+      <c r="B50" t="str">
+        <v/>
+      </c>
       <c r="C50" t="str">
         <v>Infosys</v>
       </c>
@@ -1704,6 +1852,9 @@
       </c>
       <c r="G50" t="str">
         <v>Transfer</v>
+      </c>
+      <c r="H50" t="str">
+        <v/>
       </c>
       <c r="I50" t="str">
         <v>No</v>
@@ -1731,6 +1882,9 @@
       <c r="G51" t="str">
         <v>Move In/Move Out</v>
       </c>
+      <c r="H51" t="str">
+        <v/>
+      </c>
       <c r="I51" t="str">
         <v>No</v>
       </c>
@@ -1757,6 +1911,9 @@
       <c r="G52" t="str">
         <v>Move In/Transfer</v>
       </c>
+      <c r="H52" t="str">
+        <v/>
+      </c>
       <c r="I52" t="str">
         <v>No</v>
       </c>
@@ -1765,6 +1922,9 @@
       <c r="A53" t="str">
         <v>Sanjana</v>
       </c>
+      <c r="B53" t="str">
+        <v/>
+      </c>
       <c r="C53" t="str">
         <v>Infosys</v>
       </c>
@@ -1779,6 +1939,9 @@
       </c>
       <c r="G53" t="str">
         <v>Interactions/Search</v>
+      </c>
+      <c r="H53" t="str">
+        <v/>
       </c>
       <c r="I53" t="str">
         <v>No</v>
@@ -1806,6 +1969,9 @@
       <c r="G54" t="str">
         <v>Interactions/Search</v>
       </c>
+      <c r="H54" t="str">
+        <v/>
+      </c>
       <c r="I54" t="str">
         <v>No</v>
       </c>
@@ -1814,6 +1980,9 @@
       <c r="A55" t="str">
         <v>Nilesh</v>
       </c>
+      <c r="B55" t="str">
+        <v/>
+      </c>
       <c r="C55" t="str">
         <v>Infosys</v>
       </c>
@@ -1828,6 +1997,9 @@
       </c>
       <c r="G55" t="str">
         <v>Account Maintenance</v>
+      </c>
+      <c r="H55" t="str">
+        <v/>
       </c>
       <c r="I55" t="str">
         <v>No</v>
@@ -1837,6 +2009,9 @@
       <c r="A56" t="str">
         <v>Pritam</v>
       </c>
+      <c r="B56" t="str">
+        <v/>
+      </c>
       <c r="C56" t="str">
         <v>Infosys</v>
       </c>
@@ -1851,6 +2026,9 @@
       </c>
       <c r="G56" t="str">
         <v>Account Maintenance</v>
+      </c>
+      <c r="H56" t="str">
+        <v/>
       </c>
       <c r="I56" t="str">
         <v>No</v>
@@ -1860,6 +2038,9 @@
       <c r="A57" t="str">
         <v>Smita</v>
       </c>
+      <c r="B57" t="str">
+        <v/>
+      </c>
       <c r="C57" t="str">
         <v>Infosys</v>
       </c>
@@ -1874,6 +2055,9 @@
       </c>
       <c r="G57" t="str">
         <v>Payment &amp; Payment Options/Billing Programs</v>
+      </c>
+      <c r="H57" t="str">
+        <v/>
       </c>
       <c r="I57" t="str">
         <v>No</v>
@@ -1901,6 +2085,9 @@
       <c r="G58" t="str">
         <v>Payment &amp; Payment Options</v>
       </c>
+      <c r="H58" t="str">
+        <v/>
+      </c>
       <c r="I58" t="str">
         <v>No</v>
       </c>
@@ -1927,6 +2114,9 @@
       <c r="G59" t="str">
         <v>Billing Programs</v>
       </c>
+      <c r="H59" t="str">
+        <v/>
+      </c>
       <c r="I59" t="str">
         <v>No</v>
       </c>
@@ -1935,6 +2125,9 @@
       <c r="A60" t="str">
         <v>Nikita</v>
       </c>
+      <c r="B60" t="str">
+        <v/>
+      </c>
       <c r="C60" t="str">
         <v>Infosys</v>
       </c>
@@ -1949,6 +2142,9 @@
       </c>
       <c r="G60" t="str">
         <v>Payment &amp; Payment Options</v>
+      </c>
+      <c r="H60" t="str">
+        <v/>
       </c>
       <c r="I60" t="str">
         <v>No</v>
@@ -1976,6 +2172,9 @@
       <c r="G61" t="str">
         <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
+      <c r="H61" t="str">
+        <v/>
+      </c>
       <c r="I61" t="str">
         <v>No</v>
       </c>
@@ -2002,6 +2201,9 @@
       <c r="G62" t="str">
         <v>Outage</v>
       </c>
+      <c r="H62" t="str">
+        <v/>
+      </c>
       <c r="I62" t="str">
         <v>No</v>
       </c>
@@ -2010,6 +2212,9 @@
       <c r="A63" t="str">
         <v>Jitain Mohun</v>
       </c>
+      <c r="B63" t="str">
+        <v/>
+      </c>
       <c r="C63" t="str">
         <v>Manager</v>
       </c>
@@ -2024,6 +2229,9 @@
       </c>
       <c r="G63" t="str">
         <v>Outage</v>
+      </c>
+      <c r="H63" t="str">
+        <v/>
       </c>
       <c r="I63" t="str">
         <v>No</v>
@@ -2051,6 +2259,9 @@
       <c r="G64" t="str">
         <v>Outage</v>
       </c>
+      <c r="H64" t="str">
+        <v/>
+      </c>
       <c r="I64" t="str">
         <v>No</v>
       </c>
@@ -2077,6 +2288,9 @@
       <c r="G65" t="str">
         <v>Outage</v>
       </c>
+      <c r="H65" t="str">
+        <v/>
+      </c>
       <c r="I65" t="str">
         <v>No</v>
       </c>
@@ -2085,6 +2299,9 @@
       <c r="A66" t="str">
         <v>Aakanksha</v>
       </c>
+      <c r="B66" t="str">
+        <v/>
+      </c>
       <c r="C66" t="str">
         <v>Infosys</v>
       </c>
@@ -2099,6 +2316,9 @@
       </c>
       <c r="G66" t="str">
         <v>Outage</v>
+      </c>
+      <c r="H66" t="str">
+        <v/>
       </c>
       <c r="I66" t="str">
         <v>No</v>
@@ -2108,6 +2328,9 @@
       <c r="A67" t="str">
         <v>Diksha</v>
       </c>
+      <c r="B67" t="str">
+        <v/>
+      </c>
       <c r="C67" t="str">
         <v>Infosys</v>
       </c>
@@ -2122,6 +2345,9 @@
       </c>
       <c r="G67" t="str">
         <v>Outage</v>
+      </c>
+      <c r="H67" t="str">
+        <v/>
       </c>
       <c r="I67" t="str">
         <v>No</v>
@@ -2131,6 +2357,9 @@
       <c r="A68" t="str">
         <v>Sahithi Manne</v>
       </c>
+      <c r="B68" t="str">
+        <v/>
+      </c>
       <c r="C68" t="str">
         <v>Infosys</v>
       </c>
@@ -2145,6 +2374,9 @@
       </c>
       <c r="G68" t="str">
         <v>Billing &amp; Usage/Payment Programs | Energy Management</v>
+      </c>
+      <c r="H68" t="str">
+        <v/>
       </c>
       <c r="I68" t="str">
         <v>No</v>
@@ -2172,6 +2404,9 @@
       <c r="G69" t="str">
         <v>Billing &amp; Usage/Payment Programs</v>
       </c>
+      <c r="H69" t="str">
+        <v/>
+      </c>
       <c r="I69" t="str">
         <v>No</v>
       </c>
@@ -2198,6 +2433,9 @@
       <c r="G70" t="str">
         <v>Billing &amp; Usage/Payment Programs</v>
       </c>
+      <c r="H70" t="str">
+        <v/>
+      </c>
       <c r="I70" t="str">
         <v>No</v>
       </c>
@@ -2224,6 +2462,9 @@
       <c r="G71" t="str">
         <v>Billing &amp; Usage/Payment Programs</v>
       </c>
+      <c r="H71" t="str">
+        <v/>
+      </c>
       <c r="I71" t="str">
         <v>No</v>
       </c>
@@ -2232,6 +2473,9 @@
       <c r="A72" t="str">
         <v>Rohan Bandla</v>
       </c>
+      <c r="B72" t="str">
+        <v/>
+      </c>
       <c r="C72" t="str">
         <v>Senior Associate</v>
       </c>
@@ -2246,6 +2490,9 @@
       </c>
       <c r="G72" t="str">
         <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
+      </c>
+      <c r="H72" t="str">
+        <v/>
       </c>
       <c r="I72" t="str">
         <v>No</v>
@@ -2273,6 +2520,9 @@
       <c r="G73" t="str">
         <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
+      <c r="H73" t="str">
+        <v/>
+      </c>
       <c r="I73" t="str">
         <v>No</v>
       </c>
@@ -2299,6 +2549,9 @@
       <c r="G74" t="str">
         <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
+      <c r="H74" t="str">
+        <v/>
+      </c>
       <c r="I74" t="str">
         <v>No</v>
       </c>
@@ -2325,6 +2578,9 @@
       <c r="G75" t="str">
         <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
+      <c r="H75" t="str">
+        <v/>
+      </c>
       <c r="I75" t="str">
         <v>No</v>
       </c>
@@ -2351,6 +2607,9 @@
       <c r="G76" t="str">
         <v>Energy Management</v>
       </c>
+      <c r="H76" t="str">
+        <v/>
+      </c>
       <c r="I76" t="str">
         <v>No</v>
       </c>
@@ -2377,6 +2636,9 @@
       <c r="G77" t="str">
         <v>Energy Management</v>
       </c>
+      <c r="H77" t="str">
+        <v/>
+      </c>
       <c r="I77" t="str">
         <v>No</v>
       </c>
@@ -2403,6 +2665,9 @@
       <c r="G78" t="str">
         <v>Energy Management</v>
       </c>
+      <c r="H78" t="str">
+        <v/>
+      </c>
       <c r="I78" t="str">
         <v>No</v>
       </c>
@@ -2429,6 +2694,9 @@
       <c r="G79" t="str">
         <v>Energy Management</v>
       </c>
+      <c r="H79" t="str">
+        <v/>
+      </c>
       <c r="I79" t="str">
         <v>No</v>
       </c>
@@ -2455,6 +2723,9 @@
       <c r="G80" t="str">
         <v>Energy Management</v>
       </c>
+      <c r="H80" t="str">
+        <v/>
+      </c>
       <c r="I80" t="str">
         <v>No</v>
       </c>
@@ -2481,6 +2752,9 @@
       <c r="G81" t="str">
         <v>Energy Management</v>
       </c>
+      <c r="H81" t="str">
+        <v/>
+      </c>
       <c r="I81" t="str">
         <v>No</v>
       </c>
@@ -2507,6 +2781,9 @@
       <c r="G82" t="str">
         <v>Energy Management</v>
       </c>
+      <c r="H82" t="str">
+        <v/>
+      </c>
       <c r="I82" t="str">
         <v>No</v>
       </c>
@@ -2533,6 +2810,9 @@
       <c r="G83" t="str">
         <v>Energy Management</v>
       </c>
+      <c r="H83" t="str">
+        <v/>
+      </c>
       <c r="I83" t="str">
         <v>No</v>
       </c>
@@ -2559,6 +2839,9 @@
       <c r="G84" t="str">
         <v>Energy Management</v>
       </c>
+      <c r="H84" t="str">
+        <v/>
+      </c>
       <c r="I84" t="str">
         <v>No</v>
       </c>
@@ -2584,6 +2867,9 @@
       </c>
       <c r="G85" t="str">
         <v>Energy Management</v>
+      </c>
+      <c r="H85" t="str">
+        <v/>
       </c>
       <c r="I85" t="str">
         <v>No</v>
@@ -2594,942 +2880,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:I85"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D17"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Role</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Total</v>
-      </c>
-      <c r="C1" t="str">
-        <v>FPL</v>
-      </c>
-      <c r="D1" t="str">
-        <v>PwC</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>QA</v>
-      </c>
-      <c r="B2">
-        <v>26</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="B3">
-        <v>17</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Dev Lead</v>
-      </c>
-      <c r="B4">
-        <v>7</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Onshore SA</v>
-      </c>
-      <c r="B5">
-        <v>7</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>DevOps</v>
-      </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Engagement Lead</v>
-      </c>
-      <c r="B7">
-        <v>4</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>PMO</v>
-      </c>
-      <c r="B8">
-        <v>3</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Offshore SA</v>
-      </c>
-      <c r="B9">
-        <v>3</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Integration Lead</v>
-      </c>
-      <c r="B10">
-        <v>2</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Integration Dev</v>
-      </c>
-      <c r="B11">
-        <v>2</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>DevOps Lead</v>
-      </c>
-      <c r="B12">
-        <v>2</v>
-      </c>
-      <c r="C12">
-        <v>0</v>
-      </c>
-      <c r="D12">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Windsurf/Performance Dev</v>
-      </c>
-      <c r="B13">
-        <v>2</v>
-      </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Technical Architect</v>
-      </c>
-      <c r="B14">
-        <v>1</v>
-      </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Solution Architect</v>
-      </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="D15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Business Architect</v>
-      </c>
-      <c r="B16">
-        <v>1</v>
-      </c>
-      <c r="C16">
-        <v>0</v>
-      </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>QA Lead</v>
-      </c>
-      <c r="B17">
-        <v>1</v>
-      </c>
-      <c r="C17">
-        <v>0</v>
-      </c>
-      <c r="D17">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D17"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
-  <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Release</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Total</v>
-      </c>
-      <c r="C1" t="str">
-        <v>FPL</v>
-      </c>
-      <c r="D1" t="str">
-        <v>PwC</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>All</v>
-      </c>
-      <c r="B2">
-        <v>44</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>IR3.2</v>
-      </c>
-      <c r="B3">
-        <v>8</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>IR3.2/IR4</v>
-      </c>
-      <c r="B4">
-        <v>8</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>IR3.X</v>
-      </c>
-      <c r="B5">
-        <v>4</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>IR3.X/IR4</v>
-      </c>
-      <c r="B6">
-        <v>2</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>IR4</v>
-      </c>
-      <c r="B7">
-        <v>18</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>18</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D29"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Valuestream</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Total</v>
-      </c>
-      <c r="C1" t="str">
-        <v>FPL</v>
-      </c>
-      <c r="D1" t="str">
-        <v>PwC</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Account Maintenance</v>
-      </c>
-      <c r="B2">
-        <v>3</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Account Maintenance | Customer ID &amp; Fraud</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Architecture</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Billing &amp; Usage/Payment Programs</v>
-      </c>
-      <c r="B5">
-        <v>3</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Billing &amp; Usage/Payment Programs | Energy Management</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Billing Programs</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Case Management</v>
-      </c>
-      <c r="B8">
-        <v>4</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
-      </c>
-      <c r="B9">
-        <v>4</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>DevOps</v>
-      </c>
-      <c r="B10">
-        <v>7</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Energy Management</v>
-      </c>
-      <c r="B11">
-        <v>10</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Integration</v>
-      </c>
-      <c r="B12">
-        <v>4</v>
-      </c>
-      <c r="C12">
-        <v>0</v>
-      </c>
-      <c r="D12">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Interactions/Search</v>
-      </c>
-      <c r="B13">
-        <v>4</v>
-      </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Interactions/Search | Correspondence/360s/PEXT/Account Maintenance</v>
-      </c>
-      <c r="B14">
-        <v>1</v>
-      </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Move In</v>
-      </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="D15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>Move In/Move Out</v>
-      </c>
-      <c r="B16">
-        <v>3</v>
-      </c>
-      <c r="C16">
-        <v>0</v>
-      </c>
-      <c r="D16">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>Move In/Move Out/Transfer</v>
-      </c>
-      <c r="B17">
-        <v>4</v>
-      </c>
-      <c r="C17">
-        <v>0</v>
-      </c>
-      <c r="D17">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Move In/Move Out/Transfer | Multi Move In/Transfer/Amend</v>
-      </c>
-      <c r="B18">
-        <v>1</v>
-      </c>
-      <c r="C18">
-        <v>0</v>
-      </c>
-      <c r="D18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Move In/Transfer</v>
-      </c>
-      <c r="B19">
-        <v>2</v>
-      </c>
-      <c r="C19">
-        <v>0</v>
-      </c>
-      <c r="D19">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Move Out</v>
-      </c>
-      <c r="B20">
-        <v>1</v>
-      </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
-      <c r="D20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Move Out/Transfer</v>
-      </c>
-      <c r="B21">
-        <v>1</v>
-      </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-      <c r="D21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Outage</v>
-      </c>
-      <c r="B22">
-        <v>6</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-      <c r="D22">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>Payment &amp; Payment Options</v>
-      </c>
-      <c r="B23">
-        <v>2</v>
-      </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-      <c r="D23">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
-      </c>
-      <c r="B24">
-        <v>5</v>
-      </c>
-      <c r="C24">
-        <v>0</v>
-      </c>
-      <c r="D24">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>PMO</v>
-      </c>
-      <c r="B25">
-        <v>3</v>
-      </c>
-      <c r="C25">
-        <v>0</v>
-      </c>
-      <c r="D25">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>Program Leadership</v>
-      </c>
-      <c r="B26">
-        <v>4</v>
-      </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
-      <c r="D26">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>QA - All Value Streams</v>
-      </c>
-      <c r="B27">
-        <v>1</v>
-      </c>
-      <c r="C27">
-        <v>0</v>
-      </c>
-      <c r="D27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>Transfer</v>
-      </c>
-      <c r="B28">
-        <v>2</v>
-      </c>
-      <c r="C28">
-        <v>0</v>
-      </c>
-      <c r="D28">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>Windsurf/Performance</v>
-      </c>
-      <c r="B29">
-        <v>2</v>
-      </c>
-      <c r="C29">
-        <v>0</v>
-      </c>
-      <c r="D29">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D29"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="25.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-  </cols>
-  <sheetData/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B14"/>
-  <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Metric</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Count</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Total Team Members</v>
-      </c>
-      <c r="B2">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>FPL Members</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>PwC Members</v>
-      </c>
-      <c r="B4">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v/>
-      </c>
-      <c r="B5" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Total Devs</v>
-      </c>
-      <c r="B6">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>FPL Devs</v>
-      </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Total QAs</v>
-      </c>
-      <c r="B8">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>FPL QAs</v>
-      </c>
-      <c r="B9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Total Leads</v>
-      </c>
-      <c r="B10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Total Solution Analysts</v>
-      </c>
-      <c r="B11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v/>
-      </c>
-      <c r="B12" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Releases Covered</v>
-      </c>
-      <c r="B13">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Value Streams</v>
-      </c>
-      <c r="B14">
-        <v>28</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B14"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: enhance team member data extraction and XLSX generation
#VERCEL_SKIP
</commit_message>
<xml_diff>
--- a/public/Detailed Team View.xlsx
+++ b/public/Detailed Team View.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I85"/>
+  <dimension ref="A1:I143"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -2875,9 +2875,1691 @@
         <v>No</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>Nishi Jain</v>
+      </c>
+      <c r="B86" t="str">
+        <v/>
+      </c>
+      <c r="C86" t="str">
+        <v/>
+      </c>
+      <c r="D86" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
+      <c r="F86" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G86" t="str">
+        <v/>
+      </c>
+      <c r="H86" t="str">
+        <v/>
+      </c>
+      <c r="I86" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>FPL</v>
+      </c>
+      <c r="B87" t="str">
+        <v/>
+      </c>
+      <c r="C87" t="str">
+        <v/>
+      </c>
+      <c r="D87" t="str">
+        <v>Onshore Solution Analyst</v>
+      </c>
+      <c r="E87" t="str">
+        <v/>
+      </c>
+      <c r="F87" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G87" t="str">
+        <v/>
+      </c>
+      <c r="H87" t="str">
+        <v/>
+      </c>
+      <c r="I87" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>Sona Muthayala</v>
+      </c>
+      <c r="B88" t="str">
+        <v/>
+      </c>
+      <c r="C88" t="str">
+        <v/>
+      </c>
+      <c r="D88" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E88" t="str">
+        <v/>
+      </c>
+      <c r="F88" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G88" t="str">
+        <v/>
+      </c>
+      <c r="H88" t="str">
+        <v/>
+      </c>
+      <c r="I88" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>Sriharsha Sambaraj</v>
+      </c>
+      <c r="B89" t="str">
+        <v/>
+      </c>
+      <c r="C89" t="str">
+        <v/>
+      </c>
+      <c r="D89" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E89" t="str">
+        <v/>
+      </c>
+      <c r="F89" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G89" t="str">
+        <v/>
+      </c>
+      <c r="H89" t="str">
+        <v/>
+      </c>
+      <c r="I89" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>Russell Stein</v>
+      </c>
+      <c r="B90" t="str">
+        <v/>
+      </c>
+      <c r="C90" t="str">
+        <v/>
+      </c>
+      <c r="D90" t="str">
+        <v>Onshore Solution Analyst</v>
+      </c>
+      <c r="E90" t="str">
+        <v/>
+      </c>
+      <c r="F90" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G90" t="str">
+        <v/>
+      </c>
+      <c r="H90" t="str">
+        <v/>
+      </c>
+      <c r="I90" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>Namrata Bansode</v>
+      </c>
+      <c r="B91" t="str">
+        <v/>
+      </c>
+      <c r="C91" t="str">
+        <v/>
+      </c>
+      <c r="D91" t="str">
+        <v>Offshore Solution Analyst</v>
+      </c>
+      <c r="E91" t="str">
+        <v/>
+      </c>
+      <c r="F91" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G91" t="str">
+        <v/>
+      </c>
+      <c r="H91" t="str">
+        <v/>
+      </c>
+      <c r="I91" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>Shivam Shete</v>
+      </c>
+      <c r="B92" t="str">
+        <v/>
+      </c>
+      <c r="C92" t="str">
+        <v/>
+      </c>
+      <c r="D92" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E92" t="str">
+        <v/>
+      </c>
+      <c r="F92" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G92" t="str">
+        <v/>
+      </c>
+      <c r="H92" t="str">
+        <v/>
+      </c>
+      <c r="I92" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>Sahil Thadani</v>
+      </c>
+      <c r="B93" t="str">
+        <v/>
+      </c>
+      <c r="C93" t="str">
+        <v/>
+      </c>
+      <c r="D93" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E93" t="str">
+        <v/>
+      </c>
+      <c r="F93" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G93" t="str">
+        <v/>
+      </c>
+      <c r="H93" t="str">
+        <v/>
+      </c>
+      <c r="I93" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>Kankshitha Yalamuru</v>
+      </c>
+      <c r="B94" t="str">
+        <v/>
+      </c>
+      <c r="C94" t="str">
+        <v/>
+      </c>
+      <c r="D94" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E94" t="str">
+        <v/>
+      </c>
+      <c r="F94" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G94" t="str">
+        <v/>
+      </c>
+      <c r="H94" t="str">
+        <v/>
+      </c>
+      <c r="I94" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>Sahithi Chebrolu</v>
+      </c>
+      <c r="B95" t="str">
+        <v/>
+      </c>
+      <c r="C95" t="str">
+        <v/>
+      </c>
+      <c r="D95" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E95" t="str">
+        <v/>
+      </c>
+      <c r="F95" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G95" t="str">
+        <v/>
+      </c>
+      <c r="H95" t="str">
+        <v/>
+      </c>
+      <c r="I95" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>Prayas Abinash</v>
+      </c>
+      <c r="B96" t="str">
+        <v/>
+      </c>
+      <c r="C96" t="str">
+        <v/>
+      </c>
+      <c r="D96" t="str">
+        <v>Offshore Solution Analyst</v>
+      </c>
+      <c r="E96" t="str">
+        <v/>
+      </c>
+      <c r="F96" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G96" t="str">
+        <v/>
+      </c>
+      <c r="H96" t="str">
+        <v/>
+      </c>
+      <c r="I96" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>Pranay Reddy</v>
+      </c>
+      <c r="B97" t="str">
+        <v/>
+      </c>
+      <c r="C97" t="str">
+        <v/>
+      </c>
+      <c r="D97" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E97" t="str">
+        <v/>
+      </c>
+      <c r="F97" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G97" t="str">
+        <v/>
+      </c>
+      <c r="H97" t="str">
+        <v/>
+      </c>
+      <c r="I97" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>Manu Tyagi</v>
+      </c>
+      <c r="B98" t="str">
+        <v/>
+      </c>
+      <c r="C98" t="str">
+        <v/>
+      </c>
+      <c r="D98" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E98" t="str">
+        <v/>
+      </c>
+      <c r="F98" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G98" t="str">
+        <v/>
+      </c>
+      <c r="H98" t="str">
+        <v/>
+      </c>
+      <c r="I98" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>Sunandha Sanda</v>
+      </c>
+      <c r="B99" t="str">
+        <v/>
+      </c>
+      <c r="C99" t="str">
+        <v/>
+      </c>
+      <c r="D99" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E99" t="str">
+        <v/>
+      </c>
+      <c r="F99" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G99" t="str">
+        <v/>
+      </c>
+      <c r="H99" t="str">
+        <v/>
+      </c>
+      <c r="I99" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>Jason Pereira</v>
+      </c>
+      <c r="B100" t="str">
+        <v/>
+      </c>
+      <c r="C100" t="str">
+        <v/>
+      </c>
+      <c r="D100" t="str">
+        <v>Lead</v>
+      </c>
+      <c r="E100" t="str">
+        <v/>
+      </c>
+      <c r="F100" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G100" t="str">
+        <v/>
+      </c>
+      <c r="H100" t="str">
+        <v/>
+      </c>
+      <c r="I100" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>Akhil Palakeel</v>
+      </c>
+      <c r="B101" t="str">
+        <v/>
+      </c>
+      <c r="C101" t="str">
+        <v/>
+      </c>
+      <c r="D101" t="str">
+        <v>Offshore Solution Analyst</v>
+      </c>
+      <c r="E101" t="str">
+        <v/>
+      </c>
+      <c r="F101" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G101" t="str">
+        <v/>
+      </c>
+      <c r="H101" t="str">
+        <v/>
+      </c>
+      <c r="I101" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>Sridaran N M</v>
+      </c>
+      <c r="B102" t="str">
+        <v/>
+      </c>
+      <c r="C102" t="str">
+        <v/>
+      </c>
+      <c r="D102" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E102" t="str">
+        <v/>
+      </c>
+      <c r="F102" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G102" t="str">
+        <v/>
+      </c>
+      <c r="H102" t="str">
+        <v/>
+      </c>
+      <c r="I102" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>Prasad P</v>
+      </c>
+      <c r="B103" t="str">
+        <v/>
+      </c>
+      <c r="C103" t="str">
+        <v/>
+      </c>
+      <c r="D103" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E103" t="str">
+        <v/>
+      </c>
+      <c r="F103" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G103" t="str">
+        <v/>
+      </c>
+      <c r="H103" t="str">
+        <v/>
+      </c>
+      <c r="I103" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>Pradeep Lambu</v>
+      </c>
+      <c r="B104" t="str">
+        <v/>
+      </c>
+      <c r="C104" t="str">
+        <v/>
+      </c>
+      <c r="D104" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E104" t="str">
+        <v/>
+      </c>
+      <c r="F104" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G104" t="str">
+        <v/>
+      </c>
+      <c r="H104" t="str">
+        <v/>
+      </c>
+      <c r="I104" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>Nivetha Sudharsanam</v>
+      </c>
+      <c r="B105" t="str">
+        <v/>
+      </c>
+      <c r="C105" t="str">
+        <v/>
+      </c>
+      <c r="D105" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E105" t="str">
+        <v/>
+      </c>
+      <c r="F105" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G105" t="str">
+        <v/>
+      </c>
+      <c r="H105" t="str">
+        <v/>
+      </c>
+      <c r="I105" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>Sweta Sharma</v>
+      </c>
+      <c r="B106" t="str">
+        <v/>
+      </c>
+      <c r="C106" t="str">
+        <v/>
+      </c>
+      <c r="D106" t="str">
+        <v>Lead</v>
+      </c>
+      <c r="E106" t="str">
+        <v/>
+      </c>
+      <c r="F106" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G106" t="str">
+        <v/>
+      </c>
+      <c r="H106" t="str">
+        <v/>
+      </c>
+      <c r="I106" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>Shravya Nanjundaswamy</v>
+      </c>
+      <c r="B107" t="str">
+        <v/>
+      </c>
+      <c r="C107" t="str">
+        <v/>
+      </c>
+      <c r="D107" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E107" t="str">
+        <v/>
+      </c>
+      <c r="F107" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G107" t="str">
+        <v/>
+      </c>
+      <c r="H107" t="str">
+        <v/>
+      </c>
+      <c r="I107" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>Rida Maryam Mohammad</v>
+      </c>
+      <c r="B108" t="str">
+        <v/>
+      </c>
+      <c r="C108" t="str">
+        <v/>
+      </c>
+      <c r="D108" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E108" t="str">
+        <v/>
+      </c>
+      <c r="F108" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G108" t="str">
+        <v/>
+      </c>
+      <c r="H108" t="str">
+        <v/>
+      </c>
+      <c r="I108" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>Surya Teja Poka</v>
+      </c>
+      <c r="B109" t="str">
+        <v/>
+      </c>
+      <c r="C109" t="str">
+        <v/>
+      </c>
+      <c r="D109" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E109" t="str">
+        <v/>
+      </c>
+      <c r="F109" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G109" t="str">
+        <v/>
+      </c>
+      <c r="H109" t="str">
+        <v/>
+      </c>
+      <c r="I109" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>Kavita Jha</v>
+      </c>
+      <c r="B110" t="str">
+        <v/>
+      </c>
+      <c r="C110" t="str">
+        <v/>
+      </c>
+      <c r="D110" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E110" t="str">
+        <v/>
+      </c>
+      <c r="F110" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G110" t="str">
+        <v/>
+      </c>
+      <c r="H110" t="str">
+        <v/>
+      </c>
+      <c r="I110" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>Sanniboina Murali Krishna</v>
+      </c>
+      <c r="B111" t="str">
+        <v/>
+      </c>
+      <c r="C111" t="str">
+        <v/>
+      </c>
+      <c r="D111" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E111" t="str">
+        <v/>
+      </c>
+      <c r="F111" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G111" t="str">
+        <v/>
+      </c>
+      <c r="H111" t="str">
+        <v/>
+      </c>
+      <c r="I111" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>Tameka Robinson</v>
+      </c>
+      <c r="B112" t="str">
+        <v/>
+      </c>
+      <c r="C112" t="str">
+        <v/>
+      </c>
+      <c r="D112" t="str">
+        <v>Lead</v>
+      </c>
+      <c r="E112" t="str">
+        <v/>
+      </c>
+      <c r="F112" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G112" t="str">
+        <v/>
+      </c>
+      <c r="H112" t="str">
+        <v/>
+      </c>
+      <c r="I112" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>Maria Vidal Parra</v>
+      </c>
+      <c r="B113" t="str">
+        <v/>
+      </c>
+      <c r="C113" t="str">
+        <v/>
+      </c>
+      <c r="D113" t="str">
+        <v>Scrum Master</v>
+      </c>
+      <c r="E113" t="str">
+        <v/>
+      </c>
+      <c r="F113" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G113" t="str">
+        <v/>
+      </c>
+      <c r="H113" t="str">
+        <v/>
+      </c>
+      <c r="I113" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>Naveen Tayal</v>
+      </c>
+      <c r="B114" t="str">
+        <v/>
+      </c>
+      <c r="C114" t="str">
+        <v/>
+      </c>
+      <c r="D114" t="str">
+        <v>Onshore Solution Analyst</v>
+      </c>
+      <c r="E114" t="str">
+        <v/>
+      </c>
+      <c r="F114" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G114" t="str">
+        <v/>
+      </c>
+      <c r="H114" t="str">
+        <v/>
+      </c>
+      <c r="I114" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>Harsh Shah</v>
+      </c>
+      <c r="B115" t="str">
+        <v/>
+      </c>
+      <c r="C115" t="str">
+        <v/>
+      </c>
+      <c r="D115" t="str">
+        <v>Onshore Solution Analyst</v>
+      </c>
+      <c r="E115" t="str">
+        <v/>
+      </c>
+      <c r="F115" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G115" t="str">
+        <v/>
+      </c>
+      <c r="H115" t="str">
+        <v/>
+      </c>
+      <c r="I115" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>Sama Balayeva</v>
+      </c>
+      <c r="B116" t="str">
+        <v/>
+      </c>
+      <c r="C116" t="str">
+        <v/>
+      </c>
+      <c r="D116" t="str">
+        <v>Onshore Solution Analyst</v>
+      </c>
+      <c r="E116" t="str">
+        <v/>
+      </c>
+      <c r="F116" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G116" t="str">
+        <v/>
+      </c>
+      <c r="H116" t="str">
+        <v/>
+      </c>
+      <c r="I116" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>Jake Garrell</v>
+      </c>
+      <c r="B117" t="str">
+        <v/>
+      </c>
+      <c r="C117" t="str">
+        <v/>
+      </c>
+      <c r="D117" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E117" t="str">
+        <v/>
+      </c>
+      <c r="F117" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G117" t="str">
+        <v/>
+      </c>
+      <c r="H117" t="str">
+        <v/>
+      </c>
+      <c r="I117" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>John Harrison</v>
+      </c>
+      <c r="B118" t="str">
+        <v/>
+      </c>
+      <c r="C118" t="str">
+        <v/>
+      </c>
+      <c r="D118" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E118" t="str">
+        <v/>
+      </c>
+      <c r="F118" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G118" t="str">
+        <v/>
+      </c>
+      <c r="H118" t="str">
+        <v/>
+      </c>
+      <c r="I118" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>Shashank Satvai</v>
+      </c>
+      <c r="B119" t="str">
+        <v/>
+      </c>
+      <c r="C119" t="str">
+        <v/>
+      </c>
+      <c r="D119" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E119" t="str">
+        <v/>
+      </c>
+      <c r="F119" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G119" t="str">
+        <v/>
+      </c>
+      <c r="H119" t="str">
+        <v/>
+      </c>
+      <c r="I119" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>Bryan Camacho</v>
+      </c>
+      <c r="B120" t="str">
+        <v/>
+      </c>
+      <c r="C120" t="str">
+        <v/>
+      </c>
+      <c r="D120" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E120" t="str">
+        <v/>
+      </c>
+      <c r="F120" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G120" t="str">
+        <v/>
+      </c>
+      <c r="H120" t="str">
+        <v/>
+      </c>
+      <c r="I120" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>Yolanda Espinoza</v>
+      </c>
+      <c r="B121" t="str">
+        <v/>
+      </c>
+      <c r="C121" t="str">
+        <v/>
+      </c>
+      <c r="D121" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E121" t="str">
+        <v/>
+      </c>
+      <c r="F121" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G121" t="str">
+        <v/>
+      </c>
+      <c r="H121" t="str">
+        <v/>
+      </c>
+      <c r="I121" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>Santhosh Maduri</v>
+      </c>
+      <c r="B122" t="str">
+        <v/>
+      </c>
+      <c r="C122" t="str">
+        <v/>
+      </c>
+      <c r="D122" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E122" t="str">
+        <v/>
+      </c>
+      <c r="F122" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G122" t="str">
+        <v/>
+      </c>
+      <c r="H122" t="str">
+        <v/>
+      </c>
+      <c r="I122" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>Ankit Verma</v>
+      </c>
+      <c r="B123" t="str">
+        <v/>
+      </c>
+      <c r="C123" t="str">
+        <v/>
+      </c>
+      <c r="D123" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E123" t="str">
+        <v/>
+      </c>
+      <c r="F123" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G123" t="str">
+        <v/>
+      </c>
+      <c r="H123" t="str">
+        <v/>
+      </c>
+      <c r="I123" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>Sree Sowndarya Barani K</v>
+      </c>
+      <c r="B124" t="str">
+        <v/>
+      </c>
+      <c r="C124" t="str">
+        <v/>
+      </c>
+      <c r="D124" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E124" t="str">
+        <v/>
+      </c>
+      <c r="F124" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G124" t="str">
+        <v/>
+      </c>
+      <c r="H124" t="str">
+        <v/>
+      </c>
+      <c r="I124" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>John Jyothula</v>
+      </c>
+      <c r="B125" t="str">
+        <v/>
+      </c>
+      <c r="C125" t="str">
+        <v/>
+      </c>
+      <c r="D125" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E125" t="str">
+        <v/>
+      </c>
+      <c r="F125" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G125" t="str">
+        <v/>
+      </c>
+      <c r="H125" t="str">
+        <v/>
+      </c>
+      <c r="I125" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>Niket Saxena</v>
+      </c>
+      <c r="B126" t="str">
+        <v/>
+      </c>
+      <c r="C126" t="str">
+        <v/>
+      </c>
+      <c r="D126" t="str">
+        <v>Lead</v>
+      </c>
+      <c r="E126" t="str">
+        <v/>
+      </c>
+      <c r="F126" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G126" t="str">
+        <v/>
+      </c>
+      <c r="H126" t="str">
+        <v/>
+      </c>
+      <c r="I126" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>Ramya Kothuri</v>
+      </c>
+      <c r="B127" t="str">
+        <v/>
+      </c>
+      <c r="C127" t="str">
+        <v/>
+      </c>
+      <c r="D127" t="str">
+        <v>Scrum Master</v>
+      </c>
+      <c r="E127" t="str">
+        <v/>
+      </c>
+      <c r="F127" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G127" t="str">
+        <v/>
+      </c>
+      <c r="H127" t="str">
+        <v/>
+      </c>
+      <c r="I127" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>Chaitra Hanchinal</v>
+      </c>
+      <c r="B128" t="str">
+        <v/>
+      </c>
+      <c r="C128" t="str">
+        <v/>
+      </c>
+      <c r="D128" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E128" t="str">
+        <v/>
+      </c>
+      <c r="F128" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G128" t="str">
+        <v/>
+      </c>
+      <c r="H128" t="str">
+        <v/>
+      </c>
+      <c r="I128" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>Jaya Lakshmi Papolu</v>
+      </c>
+      <c r="B129" t="str">
+        <v/>
+      </c>
+      <c r="C129" t="str">
+        <v/>
+      </c>
+      <c r="D129" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E129" t="str">
+        <v/>
+      </c>
+      <c r="F129" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G129" t="str">
+        <v/>
+      </c>
+      <c r="H129" t="str">
+        <v/>
+      </c>
+      <c r="I129" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>Mrithika Kumaresan</v>
+      </c>
+      <c r="B130" t="str">
+        <v/>
+      </c>
+      <c r="C130" t="str">
+        <v/>
+      </c>
+      <c r="D130" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E130" t="str">
+        <v/>
+      </c>
+      <c r="F130" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G130" t="str">
+        <v/>
+      </c>
+      <c r="H130" t="str">
+        <v/>
+      </c>
+      <c r="I130" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>David Sotolongo</v>
+      </c>
+      <c r="B131" t="str">
+        <v/>
+      </c>
+      <c r="C131" t="str">
+        <v/>
+      </c>
+      <c r="D131" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E131" t="str">
+        <v/>
+      </c>
+      <c r="F131" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G131" t="str">
+        <v/>
+      </c>
+      <c r="H131" t="str">
+        <v/>
+      </c>
+      <c r="I131" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>Vamsi Papulo</v>
+      </c>
+      <c r="B132" t="str">
+        <v/>
+      </c>
+      <c r="C132" t="str">
+        <v/>
+      </c>
+      <c r="D132" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E132" t="str">
+        <v/>
+      </c>
+      <c r="F132" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G132" t="str">
+        <v/>
+      </c>
+      <c r="H132" t="str">
+        <v/>
+      </c>
+      <c r="I132" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>Tejaswini Pathade</v>
+      </c>
+      <c r="B133" t="str">
+        <v/>
+      </c>
+      <c r="C133" t="str">
+        <v/>
+      </c>
+      <c r="D133" t="str">
+        <v>Lead</v>
+      </c>
+      <c r="E133" t="str">
+        <v/>
+      </c>
+      <c r="F133" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G133" t="str">
+        <v/>
+      </c>
+      <c r="H133" t="str">
+        <v/>
+      </c>
+      <c r="I133" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>Andhy Gomez</v>
+      </c>
+      <c r="B134" t="str">
+        <v/>
+      </c>
+      <c r="C134" t="str">
+        <v/>
+      </c>
+      <c r="D134" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E134" t="str">
+        <v/>
+      </c>
+      <c r="F134" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G134" t="str">
+        <v/>
+      </c>
+      <c r="H134" t="str">
+        <v/>
+      </c>
+      <c r="I134" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>Kelvin Mobley</v>
+      </c>
+      <c r="B135" t="str">
+        <v/>
+      </c>
+      <c r="C135" t="str">
+        <v/>
+      </c>
+      <c r="D135" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E135" t="str">
+        <v/>
+      </c>
+      <c r="F135" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G135" t="str">
+        <v/>
+      </c>
+      <c r="H135" t="str">
+        <v/>
+      </c>
+      <c r="I135" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>Bharath Reddy Baddam</v>
+      </c>
+      <c r="B136" t="str">
+        <v/>
+      </c>
+      <c r="C136" t="str">
+        <v/>
+      </c>
+      <c r="D136" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E136" t="str">
+        <v/>
+      </c>
+      <c r="F136" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G136" t="str">
+        <v/>
+      </c>
+      <c r="H136" t="str">
+        <v/>
+      </c>
+      <c r="I136" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>Shweta Tiwari</v>
+      </c>
+      <c r="B137" t="str">
+        <v/>
+      </c>
+      <c r="C137" t="str">
+        <v/>
+      </c>
+      <c r="D137" t="str">
+        <v>Dev</v>
+      </c>
+      <c r="E137" t="str">
+        <v/>
+      </c>
+      <c r="F137" t="str">
+        <v>IR4</v>
+      </c>
+      <c r="G137" t="str">
+        <v/>
+      </c>
+      <c r="H137" t="str">
+        <v/>
+      </c>
+      <c r="I137" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>Rodolfo Duarte</v>
+      </c>
+      <c r="B138" t="str">
+        <v/>
+      </c>
+      <c r="C138" t="str">
+        <v/>
+      </c>
+      <c r="D138" t="str">
+        <v>Team</v>
+      </c>
+      <c r="E138" t="str">
+        <v>Cross-Functional</v>
+      </c>
+      <c r="F138" t="str">
+        <v>All</v>
+      </c>
+      <c r="G138" t="str">
+        <v>Cross-Functional</v>
+      </c>
+      <c r="H138" t="str">
+        <v/>
+      </c>
+      <c r="I138" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>Ziyad Auti</v>
+      </c>
+      <c r="B139" t="str">
+        <v/>
+      </c>
+      <c r="C139" t="str">
+        <v/>
+      </c>
+      <c r="D139" t="str">
+        <v>Intern</v>
+      </c>
+      <c r="E139" t="str">
+        <v>Cross-Functional</v>
+      </c>
+      <c r="F139" t="str">
+        <v>All</v>
+      </c>
+      <c r="G139" t="str">
+        <v>Cross-Functional</v>
+      </c>
+      <c r="H139" t="str">
+        <v/>
+      </c>
+      <c r="I139" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>Kishor S</v>
+      </c>
+      <c r="B140" t="str">
+        <v/>
+      </c>
+      <c r="C140" t="str">
+        <v/>
+      </c>
+      <c r="D140" t="str">
+        <v>Intern</v>
+      </c>
+      <c r="E140" t="str">
+        <v>Cross-Functional</v>
+      </c>
+      <c r="F140" t="str">
+        <v>All</v>
+      </c>
+      <c r="G140" t="str">
+        <v>Cross-Functional</v>
+      </c>
+      <c r="H140" t="str">
+        <v/>
+      </c>
+      <c r="I140" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>Krithika Harishchandra Shettigar</v>
+      </c>
+      <c r="B141" t="str">
+        <v/>
+      </c>
+      <c r="C141" t="str">
+        <v/>
+      </c>
+      <c r="D141" t="str">
+        <v>Intern</v>
+      </c>
+      <c r="E141" t="str">
+        <v>Cross-Functional</v>
+      </c>
+      <c r="F141" t="str">
+        <v>All</v>
+      </c>
+      <c r="G141" t="str">
+        <v>Cross-Functional</v>
+      </c>
+      <c r="H141" t="str">
+        <v/>
+      </c>
+      <c r="I141" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>Potumanchi Sree Yashana</v>
+      </c>
+      <c r="B142" t="str">
+        <v/>
+      </c>
+      <c r="C142" t="str">
+        <v/>
+      </c>
+      <c r="D142" t="str">
+        <v>Intern</v>
+      </c>
+      <c r="E142" t="str">
+        <v>Cross-Functional</v>
+      </c>
+      <c r="F142" t="str">
+        <v>All</v>
+      </c>
+      <c r="G142" t="str">
+        <v>Cross-Functional</v>
+      </c>
+      <c r="H142" t="str">
+        <v/>
+      </c>
+      <c r="I142" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>Adithya Sankar S</v>
+      </c>
+      <c r="B143" t="str">
+        <v/>
+      </c>
+      <c r="C143" t="str">
+        <v/>
+      </c>
+      <c r="D143" t="str">
+        <v>Intern</v>
+      </c>
+      <c r="E143" t="str">
+        <v>Cross-Functional</v>
+      </c>
+      <c r="F143" t="str">
+        <v>All</v>
+      </c>
+      <c r="G143" t="str">
+        <v>Cross-Functional</v>
+      </c>
+      <c r="H143" t="str">
+        <v/>
+      </c>
+      <c r="I143" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I85"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I143"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add script to update Detailed Team View Excel from team data
#VERCEL_SKIP
</commit_message>
<xml_diff>
--- a/public/Detailed Team View.xlsx
+++ b/public/Detailed Team View.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I143"/>
+  <dimension ref="A1:I125"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -441,405 +441,405 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Ted Capaldi</v>
+        <v>Andhy Gomez</v>
       </c>
       <c r="B2" t="str">
-        <v>theodore.capaldi@pwc.com</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>Partner</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>Engagement Lead</v>
+        <v>Dev</v>
       </c>
       <c r="E2" t="str">
-        <v>Leadership</v>
+        <v>IR4</v>
       </c>
       <c r="F2" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G2" t="str">
-        <v>Program Leadership</v>
+        <v>Release</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>FPL Case Management POD</v>
       </c>
       <c r="I2" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Matthew Rupas</v>
+        <v>Bharath Reddy Baddam</v>
       </c>
       <c r="B3" t="str">
-        <v>matthew.i.rupas@pwc.com</v>
+        <v/>
       </c>
       <c r="C3" t="str">
-        <v>Partner</v>
+        <v/>
       </c>
       <c r="D3" t="str">
-        <v>Engagement Lead</v>
+        <v>Dev</v>
       </c>
       <c r="E3" t="str">
-        <v>Leadership</v>
+        <v>IR4</v>
       </c>
       <c r="F3" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G3" t="str">
-        <v>Program Leadership</v>
+        <v>Release</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>FPL Case Management POD</v>
       </c>
       <c r="I3" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Sujith Pillai</v>
+        <v>Bryan Camacho</v>
       </c>
       <c r="B4" t="str">
-        <v>sujith.s.pillai@pwc.com</v>
+        <v/>
       </c>
       <c r="C4" t="str">
-        <v>Director</v>
+        <v/>
       </c>
       <c r="D4" t="str">
-        <v>Engagement Lead</v>
+        <v>Dev</v>
       </c>
       <c r="E4" t="str">
-        <v>Leadership</v>
+        <v>Hypercare</v>
       </c>
       <c r="F4" t="str">
-        <v>All</v>
+        <v>IR3.2-Hypercare</v>
       </c>
       <c r="G4" t="str">
-        <v>Program Leadership</v>
+        <v>Hypercare</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>IR3.2 Hypercare Support</v>
       </c>
       <c r="I4" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Anto Germans</v>
+        <v>David Sotolongo</v>
       </c>
       <c r="B5" t="str">
-        <v>anto.a.germans@pwc.com</v>
+        <v/>
       </c>
       <c r="C5" t="str">
-        <v>Director</v>
+        <v/>
       </c>
       <c r="D5" t="str">
-        <v>Engagement Lead</v>
+        <v>Dev</v>
       </c>
       <c r="E5" t="str">
-        <v>Leadership</v>
+        <v>IR4</v>
       </c>
       <c r="F5" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G5" t="str">
-        <v>Program Leadership</v>
+        <v>Release</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I5" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Hemant Jain</v>
+        <v>John Harrison</v>
       </c>
       <c r="B6" t="str">
-        <v>hemant.jain@pwc.com</v>
+        <v/>
       </c>
       <c r="C6" t="str">
-        <v>Senior Manager</v>
+        <v/>
       </c>
       <c r="D6" t="str">
-        <v>Technical Architect</v>
+        <v>Dev</v>
       </c>
       <c r="E6" t="str">
-        <v>Leadership</v>
+        <v>Hypercare</v>
       </c>
       <c r="F6" t="str">
-        <v>All</v>
+        <v>IR3.2-Hypercare</v>
       </c>
       <c r="G6" t="str">
-        <v>Architecture</v>
+        <v>Hypercare</v>
       </c>
       <c r="H6" t="str">
-        <v/>
+        <v>IR3.2 Hypercare Support</v>
       </c>
       <c r="I6" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Tyaga Pati</v>
+        <v>Kelvin Mobley</v>
       </c>
       <c r="B7" t="str">
-        <v>tyaga.pati@pwc.com</v>
+        <v/>
       </c>
       <c r="C7" t="str">
-        <v>Senior Manager</v>
+        <v/>
       </c>
       <c r="D7" t="str">
-        <v>Solution Architect</v>
+        <v>Dev</v>
       </c>
       <c r="E7" t="str">
-        <v>Leadership</v>
+        <v>IR4</v>
       </c>
       <c r="F7" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G7" t="str">
-        <v>Architecture</v>
+        <v>Release</v>
       </c>
       <c r="H7" t="str">
-        <v/>
+        <v>FPL Case Management POD</v>
       </c>
       <c r="I7" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Susan Matthews</v>
+        <v>Maria Vidal Parra</v>
       </c>
       <c r="B8" t="str">
-        <v>susan.m.mathew@pwc.com</v>
+        <v/>
       </c>
       <c r="C8" t="str">
-        <v>Senior Manager</v>
+        <v/>
       </c>
       <c r="D8" t="str">
-        <v>Business Architect</v>
+        <v>Scrum Master</v>
       </c>
       <c r="E8" t="str">
-        <v>Leadership</v>
+        <v>IR4</v>
       </c>
       <c r="F8" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G8" t="str">
-        <v>Architecture</v>
+        <v>Release</v>
       </c>
       <c r="H8" t="str">
-        <v/>
+        <v>FPL Dev POD</v>
       </c>
       <c r="I8" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Shanta Samlal</v>
+        <v>Ramya Kothuri</v>
       </c>
       <c r="B9" t="str">
-        <v>shanta.samlal@pwc.com</v>
+        <v/>
       </c>
       <c r="C9" t="str">
-        <v>Manager</v>
+        <v/>
       </c>
       <c r="D9" t="str">
-        <v>PMO</v>
+        <v>Scrum Master</v>
       </c>
       <c r="E9" t="str">
-        <v>Leadership</v>
+        <v>IR4</v>
       </c>
       <c r="F9" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G9" t="str">
-        <v>PMO</v>
+        <v>Release</v>
       </c>
       <c r="H9" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I9" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Paarth Sonwaney</v>
+        <v>Santhosh Maduri</v>
       </c>
       <c r="B10" t="str">
-        <v>paarth.sonwaney@pwc.com</v>
+        <v/>
       </c>
       <c r="C10" t="str">
-        <v>Manager</v>
+        <v/>
       </c>
       <c r="D10" t="str">
-        <v>PMO</v>
+        <v>Dev</v>
       </c>
       <c r="E10" t="str">
-        <v>Leadership</v>
+        <v>Hypercare</v>
       </c>
       <c r="F10" t="str">
-        <v>All</v>
+        <v>IR3.2-Hypercare</v>
       </c>
       <c r="G10" t="str">
-        <v>PMO</v>
+        <v>Hypercare</v>
       </c>
       <c r="H10" t="str">
-        <v/>
+        <v>IR3.2 Hypercare Support</v>
       </c>
       <c r="I10" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Courtney Hawkins</v>
+        <v>Shweta Tiwari</v>
       </c>
       <c r="B11" t="str">
-        <v>courtney.c.hawkins@pwc.com</v>
+        <v/>
       </c>
       <c r="C11" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D11" t="str">
-        <v>PMO</v>
+        <v>Dev</v>
       </c>
       <c r="E11" t="str">
-        <v>Leadership</v>
+        <v>IR4</v>
       </c>
       <c r="F11" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G11" t="str">
-        <v>PMO</v>
+        <v>Release</v>
       </c>
       <c r="H11" t="str">
-        <v/>
+        <v>FPL Case Management POD</v>
       </c>
       <c r="I11" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Kodi Elangovan</v>
+        <v>Tameka Robinson</v>
       </c>
       <c r="B12" t="str">
-        <v>kodiyarasan.elangovan@pwc.com</v>
+        <v/>
       </c>
       <c r="C12" t="str">
-        <v>Manager</v>
+        <v/>
       </c>
       <c r="D12" t="str">
-        <v>Integration Lead</v>
+        <v>Lead</v>
       </c>
       <c r="E12" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F12" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G12" t="str">
-        <v>Integration</v>
+        <v>Release</v>
       </c>
       <c r="H12" t="str">
-        <v/>
+        <v>FPL Dev POD</v>
       </c>
       <c r="I12" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Arun Kumar Krishnareddy Obannareddy</v>
+        <v>Tejaswini Pathade</v>
       </c>
       <c r="B13" t="str">
-        <v>arun.kumar.krishnareddy.obannareddy@pwc.com</v>
+        <v/>
       </c>
       <c r="C13" t="str">
-        <v>Manager</v>
+        <v/>
       </c>
       <c r="D13" t="str">
-        <v>Integration Lead</v>
+        <v>Lead</v>
       </c>
       <c r="E13" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F13" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G13" t="str">
-        <v>Integration</v>
+        <v>Release</v>
       </c>
       <c r="H13" t="str">
-        <v/>
+        <v>FPL Case Management POD</v>
       </c>
       <c r="I13" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Pranav Singh</v>
+        <v>Vamsi Papulo</v>
       </c>
       <c r="B14" t="str">
-        <v>pranav.s.singh@pwc.com</v>
+        <v/>
       </c>
       <c r="C14" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D14" t="str">
-        <v>Integration Dev</v>
+        <v>Dev</v>
       </c>
       <c r="E14" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F14" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G14" t="str">
-        <v>Integration</v>
+        <v>Release</v>
       </c>
       <c r="H14" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I14" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Vasudha Tandon</v>
+        <v>Aaditi Madhavan</v>
       </c>
       <c r="B15" t="str">
-        <v>vasudha.tandon@pwc.com</v>
+        <v>aaditi.madhavan@pwc.com</v>
       </c>
       <c r="C15" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D15" t="str">
-        <v>Integration Dev</v>
+        <v>Dev</v>
       </c>
       <c r="E15" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F15" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G15" t="str">
-        <v>Integration</v>
+        <v>Energy Management</v>
       </c>
       <c r="H15" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I15" t="str">
         <v>No</v>
@@ -847,28 +847,28 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Ritesh Nanda</v>
+        <v>Aakanksha</v>
       </c>
       <c r="B16" t="str">
-        <v>ritesh.nanda@pwc.com</v>
+        <v/>
       </c>
       <c r="C16" t="str">
-        <v>Manager</v>
+        <v>Infosys</v>
       </c>
       <c r="D16" t="str">
-        <v>DevOps Lead</v>
+        <v>QA</v>
       </c>
       <c r="E16" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.X</v>
       </c>
       <c r="F16" t="str">
-        <v>All</v>
+        <v>IR3.X</v>
       </c>
       <c r="G16" t="str">
-        <v>DevOps</v>
+        <v>Outage</v>
       </c>
       <c r="H16" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I16" t="str">
         <v>No</v>
@@ -876,16 +876,16 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Shabnam Nasreen</v>
+        <v>Adithya Sankar S</v>
       </c>
       <c r="B17" t="str">
-        <v>shabnam.nasreen@pwc.com</v>
+        <v/>
       </c>
       <c r="C17" t="str">
-        <v>Manager</v>
+        <v/>
       </c>
       <c r="D17" t="str">
-        <v>DevOps Lead</v>
+        <v>Intern</v>
       </c>
       <c r="E17" t="str">
         <v>Cross-Functional</v>
@@ -894,10 +894,10 @@
         <v>All</v>
       </c>
       <c r="G17" t="str">
-        <v>DevOps</v>
+        <v>Interns</v>
       </c>
       <c r="H17" t="str">
-        <v/>
+        <v>Interns</v>
       </c>
       <c r="I17" t="str">
         <v>No</v>
@@ -905,28 +905,28 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Santosh Kumar Jangam</v>
+        <v>Aditya Talwar</v>
       </c>
       <c r="B18" t="str">
-        <v>santosh.kumar.jangam@pwc.com</v>
+        <v>aditya.talwar@pwc.com</v>
       </c>
       <c r="C18" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D18" t="str">
-        <v>DevOps</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E18" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.2</v>
       </c>
       <c r="F18" t="str">
-        <v>All</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G18" t="str">
-        <v>DevOps</v>
+        <v>Account Maintenance | Customer ID &amp; Fraud</v>
       </c>
       <c r="H18" t="str">
-        <v/>
+        <v>Dev POD 6/Aditya</v>
       </c>
       <c r="I18" t="str">
         <v>No</v>
@@ -934,28 +934,28 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Rhitik Khanna</v>
+        <v>Akhil Palakeel</v>
       </c>
       <c r="B19" t="str">
-        <v>rhitik.khanna@pwc.com</v>
+        <v/>
       </c>
       <c r="C19" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D19" t="str">
-        <v>DevOps</v>
+        <v>Offshore Solution Analyst</v>
       </c>
       <c r="E19" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F19" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G19" t="str">
-        <v>DevOps</v>
+        <v>Release</v>
       </c>
       <c r="H19" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I19" t="str">
         <v>No</v>
@@ -963,25 +963,25 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Shatakshi Srivastava</v>
+        <v>Amarjeet Singh</v>
       </c>
       <c r="B20" t="str">
-        <v>shatakshi.s.srivastava@pwc.com</v>
+        <v>amarjeet.singh@pwc.com</v>
       </c>
       <c r="C20" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D20" t="str">
-        <v>DevOps</v>
+        <v>Dev</v>
       </c>
       <c r="E20" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F20" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G20" t="str">
-        <v>DevOps</v>
+        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
       <c r="H20" t="str">
         <v/>
@@ -992,25 +992,25 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Vinay Vadrevu</v>
+        <v>Ankit Mishra</v>
       </c>
       <c r="B21" t="str">
-        <v/>
+        <v>ankit.b.mishra@pwc.com</v>
       </c>
       <c r="C21" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D21" t="str">
-        <v>DevOps</v>
+        <v>Dev</v>
       </c>
       <c r="E21" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F21" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G21" t="str">
-        <v>DevOps</v>
+        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
       <c r="H21" t="str">
         <v/>
@@ -1021,28 +1021,28 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>B Rajkumar</v>
+        <v>Ankit Verma</v>
       </c>
       <c r="B22" t="str">
         <v/>
       </c>
       <c r="C22" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D22" t="str">
-        <v>DevOps</v>
+        <v>Dev</v>
       </c>
       <c r="E22" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F22" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G22" t="str">
-        <v>DevOps</v>
+        <v>Release</v>
       </c>
       <c r="H22" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I22" t="str">
         <v>No</v>
@@ -1050,25 +1050,25 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Harish Govindareddy</v>
+        <v>Anto Germans</v>
       </c>
       <c r="B23" t="str">
-        <v>harish.govindareddy@pwc.com</v>
+        <v>anto.a.germans@pwc.com</v>
       </c>
       <c r="C23" t="str">
-        <v>Senior Associate</v>
+        <v>Director</v>
       </c>
       <c r="D23" t="str">
-        <v>Windsurf/Performance Dev</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E23" t="str">
-        <v>Cross-Functional</v>
+        <v>Leadership</v>
       </c>
       <c r="F23" t="str">
         <v>All</v>
       </c>
       <c r="G23" t="str">
-        <v>Windsurf/Performance</v>
+        <v>Program Leadership</v>
       </c>
       <c r="H23" t="str">
         <v/>
@@ -1079,28 +1079,28 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Sanket Mundargi</v>
+        <v>Anurag Jakkal</v>
       </c>
       <c r="B24" t="str">
-        <v>sanket.mundargi@pwc.com</v>
+        <v>jakkal.anurag.surendra@pwc.com</v>
       </c>
       <c r="C24" t="str">
-        <v>Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D24" t="str">
-        <v>Windsurf/Performance Dev</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E24" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F24" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G24" t="str">
-        <v>Windsurf/Performance</v>
+        <v>Energy Management</v>
       </c>
       <c r="H24" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I24" t="str">
         <v>No</v>
@@ -1108,25 +1108,25 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Sneha Girigoudar</v>
+        <v>Argene M. Francisco</v>
       </c>
       <c r="B25" t="str">
-        <v>sneha.raosaheb.girigoudar@pwc.com</v>
+        <v>argene.francisco@pwc.com</v>
       </c>
       <c r="C25" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D25" t="str">
-        <v>Dev Lead</v>
+        <v>QA</v>
       </c>
       <c r="E25" t="str">
         <v>IR3.2</v>
       </c>
       <c r="F25" t="str">
-        <v>IR3.2/IR4</v>
+        <v>All</v>
       </c>
       <c r="G25" t="str">
-        <v>Interactions/Search | Correspondence/360s/PEXT/Account Maintenance</v>
+        <v>Move In/Transfer</v>
       </c>
       <c r="H25" t="str">
         <v/>
@@ -1137,25 +1137,25 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Michael O'shea</v>
+        <v>Arun Kumar Krishnareddy Obannareddy</v>
       </c>
       <c r="B26" t="str">
-        <v>michael.o.oshea@pwc.com</v>
+        <v>arun.kumar.krishnareddy.obannareddy@pwc.com</v>
       </c>
       <c r="C26" t="str">
-        <v>Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D26" t="str">
-        <v>Onshore SA</v>
+        <v>Integration Lead</v>
       </c>
       <c r="E26" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F26" t="str">
-        <v>IR3.2</v>
+        <v>All</v>
       </c>
       <c r="G26" t="str">
-        <v>Interactions/Search</v>
+        <v>Integration</v>
       </c>
       <c r="H26" t="str">
         <v/>
@@ -1166,28 +1166,28 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Madhumita Kodidela</v>
+        <v>Ashit Prashant Golwala</v>
       </c>
       <c r="B27" t="str">
-        <v>madhumitha.kodidela@pwc.com</v>
+        <v>ashit.prashant.golwala@pwc.com</v>
       </c>
       <c r="C27" t="str">
-        <v>Senior Associate</v>
+        <v>Associate</v>
       </c>
       <c r="D27" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E27" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F27" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G27" t="str">
-        <v>Interactions/Search</v>
+        <v>Energy Management</v>
       </c>
       <c r="H27" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I27" t="str">
         <v>No</v>
@@ -1195,25 +1195,25 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Suraj Ghodmare</v>
+        <v>B Rajkumar</v>
       </c>
       <c r="B28" t="str">
-        <v>suraj.ghodmare@pwc.com</v>
+        <v/>
       </c>
       <c r="C28" t="str">
-        <v>Manager</v>
+        <v>Associate</v>
       </c>
       <c r="D28" t="str">
-        <v>Dev Lead</v>
+        <v>DevOps</v>
       </c>
       <c r="E28" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F28" t="str">
-        <v>IR3.2</v>
+        <v>All</v>
       </c>
       <c r="G28" t="str">
-        <v>Move In/Move Out/Transfer</v>
+        <v>DevOps</v>
       </c>
       <c r="H28" t="str">
         <v/>
@@ -1224,25 +1224,25 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Gianna Caruso</v>
+        <v>Bhyravabhotla Naga Lakshmi Sirisha</v>
       </c>
       <c r="B29" t="str">
-        <v>gianna.caruso@pwc.com</v>
+        <v>bhyravabhotla.naga.lakshmi.sirisha@pwc.com</v>
       </c>
       <c r="C29" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D29" t="str">
-        <v>Onshore SA</v>
+        <v>QA</v>
       </c>
       <c r="E29" t="str">
         <v>IR3.2</v>
       </c>
       <c r="F29" t="str">
-        <v>IR3.2/IR4</v>
+        <v>All</v>
       </c>
       <c r="G29" t="str">
-        <v>Move In/Move Out/Transfer | Multi Move In/Transfer/Amend</v>
+        <v>Move In/Move Out</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -1253,28 +1253,28 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Piyush Singh</v>
+        <v>Chaitra Hanchinal</v>
       </c>
       <c r="B30" t="str">
-        <v>piyush.ss.singh@pwc.com</v>
+        <v/>
       </c>
       <c r="C30" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D30" t="str">
         <v>Dev</v>
       </c>
       <c r="E30" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F30" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G30" t="str">
-        <v>Move In/Move Out/Transfer</v>
+        <v>Release</v>
       </c>
       <c r="H30" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I30" t="str">
         <v>No</v>
@@ -1282,10 +1282,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Shikhar Sanjeev</v>
+        <v>Cheruku Pranay Reddy</v>
       </c>
       <c r="B31" t="str">
-        <v>shikhar.sanjeev@pwc.com</v>
+        <v>cheruku.pranay.reddy@pwc.com</v>
       </c>
       <c r="C31" t="str">
         <v>Senior Associate</v>
@@ -1294,13 +1294,13 @@
         <v>Dev</v>
       </c>
       <c r="E31" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F31" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G31" t="str">
-        <v>Move In/Move Out/Transfer</v>
+        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
       <c r="H31" t="str">
         <v/>
@@ -1311,16 +1311,16 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Aditya Talwar</v>
+        <v>Cicily Deng</v>
       </c>
       <c r="B32" t="str">
-        <v>aditya.talwar@pwc.com</v>
+        <v>cicily.deng@pwc.com</v>
       </c>
       <c r="C32" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D32" t="str">
-        <v>Dev Lead</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E32" t="str">
         <v>IR3.2</v>
@@ -1329,10 +1329,10 @@
         <v>IR3.2/IR4</v>
       </c>
       <c r="G32" t="str">
-        <v>Account Maintenance | Customer ID &amp; Fraud</v>
+        <v>Case Management</v>
       </c>
       <c r="H32" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I32" t="str">
         <v>No</v>
@@ -1340,25 +1340,25 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Nishi Narendra Jain</v>
+        <v>Courtney Hawkins</v>
       </c>
       <c r="B33" t="str">
-        <v>jain.u.nishi@pwc.com</v>
+        <v>courtney.c.hawkins@pwc.com</v>
       </c>
       <c r="C33" t="str">
         <v>Senior Associate</v>
       </c>
       <c r="D33" t="str">
-        <v>Dev</v>
+        <v>PMO</v>
       </c>
       <c r="E33" t="str">
-        <v>IR3.2</v>
+        <v>Leadership</v>
       </c>
       <c r="F33" t="str">
-        <v>IR3.2</v>
+        <v>All</v>
       </c>
       <c r="G33" t="str">
-        <v>Account Maintenance</v>
+        <v>PMO</v>
       </c>
       <c r="H33" t="str">
         <v/>
@@ -1369,16 +1369,16 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Shreya LNU</v>
+        <v>Deneys Van Der Merwe</v>
       </c>
       <c r="B34" t="str">
-        <v>shreya.l.lnu@pwc.com</v>
+        <v>deneys.van.der.merwe@pwc.com</v>
       </c>
       <c r="C34" t="str">
-        <v>Manager</v>
+        <v>Associate</v>
       </c>
       <c r="D34" t="str">
-        <v>Dev Lead</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E34" t="str">
         <v>IR3.2</v>
@@ -1387,10 +1387,10 @@
         <v>IR3.2/IR4</v>
       </c>
       <c r="G34" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v>Case Management</v>
       </c>
       <c r="H34" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I34" t="str">
         <v>No</v>
@@ -1398,28 +1398,28 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Mounika Depuri</v>
+        <v>Diksha</v>
       </c>
       <c r="B35" t="str">
-        <v>mounika.depuri@pwc.com</v>
+        <v/>
       </c>
       <c r="C35" t="str">
-        <v>Senior Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D35" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E35" t="str">
-        <v>IR3.2</v>
+        <v>IR3.X</v>
       </c>
       <c r="F35" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR3.X</v>
       </c>
       <c r="G35" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v>Outage</v>
       </c>
       <c r="H35" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I35" t="str">
         <v>No</v>
@@ -1427,25 +1427,25 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Sandesh Saravanan</v>
+        <v>Dnyanesh Prakash Painjane</v>
       </c>
       <c r="B36" t="str">
-        <v>sandesh.saravanan@pwc.com</v>
+        <v>dnyanesh.prakash.painjane@pwc.com</v>
       </c>
       <c r="C36" t="str">
-        <v>Intern</v>
+        <v>Associate</v>
       </c>
       <c r="D36" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E36" t="str">
         <v>IR3.2</v>
       </c>
       <c r="F36" t="str">
-        <v>IR3.2</v>
+        <v>All</v>
       </c>
       <c r="G36" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v>Move In/Transfer</v>
       </c>
       <c r="H36" t="str">
         <v/>
@@ -1456,16 +1456,16 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Rinky Chawla</v>
+        <v>Gianna Caruso</v>
       </c>
       <c r="B37" t="str">
-        <v>rinky.chawla@pwc.com</v>
+        <v>gianna.caruso@pwc.com</v>
       </c>
       <c r="C37" t="str">
-        <v>Manager</v>
+        <v>Associate</v>
       </c>
       <c r="D37" t="str">
-        <v>Dev Lead</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E37" t="str">
         <v>IR3.2</v>
@@ -1474,10 +1474,10 @@
         <v>IR3.2/IR4</v>
       </c>
       <c r="G37" t="str">
-        <v>Case Management</v>
+        <v>Move In/Move Out/Transfer | Multi Move In/Transfer/Amend</v>
       </c>
       <c r="H37" t="str">
-        <v/>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I37" t="str">
         <v>No</v>
@@ -1485,25 +1485,25 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Deneys Van Der Merwe</v>
+        <v>Girlee P. Alvarado</v>
       </c>
       <c r="B38" t="str">
-        <v>deneys.van.der.merwe@pwc.com</v>
+        <v>girlee.alvarado@pwc.com</v>
       </c>
       <c r="C38" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D38" t="str">
-        <v>Onshore SA</v>
+        <v>QA</v>
       </c>
       <c r="E38" t="str">
         <v>IR3.2</v>
       </c>
       <c r="F38" t="str">
-        <v>IR3.2/IR4</v>
+        <v>All</v>
       </c>
       <c r="G38" t="str">
-        <v>Case Management</v>
+        <v>Move Out/Transfer</v>
       </c>
       <c r="H38" t="str">
         <v/>
@@ -1514,25 +1514,25 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Cicily Deng</v>
+        <v>Harish Govindareddy</v>
       </c>
       <c r="B39" t="str">
-        <v>cicily.deng@pwc.com</v>
+        <v>harish.govindareddy@pwc.com</v>
       </c>
       <c r="C39" t="str">
         <v>Senior Associate</v>
       </c>
       <c r="D39" t="str">
-        <v>Onshore SA</v>
+        <v>Windsurf/Performance Dev</v>
       </c>
       <c r="E39" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F39" t="str">
-        <v>IR3.2/IR4</v>
+        <v>All</v>
       </c>
       <c r="G39" t="str">
-        <v>Case Management</v>
+        <v>Windsurf/Performance</v>
       </c>
       <c r="H39" t="str">
         <v/>
@@ -1543,25 +1543,25 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Pratik Kurdukar</v>
+        <v>Hemant Jain</v>
       </c>
       <c r="B40" t="str">
-        <v>pratik.k.kurdukar@pwc.com</v>
+        <v>hemant.jain@pwc.com</v>
       </c>
       <c r="C40" t="str">
-        <v>Associate</v>
+        <v>Senior Manager</v>
       </c>
       <c r="D40" t="str">
-        <v>Dev</v>
+        <v>Technical Architect</v>
       </c>
       <c r="E40" t="str">
-        <v>IR3.2</v>
+        <v>Leadership</v>
       </c>
       <c r="F40" t="str">
-        <v>IR3.2</v>
+        <v>All</v>
       </c>
       <c r="G40" t="str">
-        <v>Case Management</v>
+        <v>Architecture</v>
       </c>
       <c r="H40" t="str">
         <v/>
@@ -1572,16 +1572,16 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Rajaraman A</v>
+        <v>Israel L. Jacinto</v>
       </c>
       <c r="B41" t="str">
-        <v>rajaraman.a@pwc.com</v>
+        <v>israel.jacinto@pwc.com</v>
       </c>
       <c r="C41" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D41" t="str">
-        <v>QA Lead</v>
+        <v>QA</v>
       </c>
       <c r="E41" t="str">
         <v>IR3.2</v>
@@ -1590,7 +1590,7 @@
         <v>All</v>
       </c>
       <c r="G41" t="str">
-        <v>QA - All Value Streams</v>
+        <v>Move Out</v>
       </c>
       <c r="H41" t="str">
         <v/>
@@ -1601,28 +1601,28 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Maneesha</v>
+        <v>Jason Pereira</v>
       </c>
       <c r="B42" t="str">
         <v/>
       </c>
       <c r="C42" t="str">
-        <v>Infosys</v>
+        <v/>
       </c>
       <c r="D42" t="str">
-        <v>QA</v>
+        <v>Lead</v>
       </c>
       <c r="E42" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F42" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G42" t="str">
-        <v>Move In/Move Out/Transfer</v>
+        <v>Release</v>
       </c>
       <c r="H42" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I42" t="str">
         <v>No</v>
@@ -1630,28 +1630,28 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Bhyravabhotla Naga Lakshmi Sirisha</v>
+        <v>Jaya Lakshmi Papolu</v>
       </c>
       <c r="B43" t="str">
-        <v>bhyravabhotla.naga.lakshmi.sirisha@pwc.com</v>
+        <v/>
       </c>
       <c r="C43" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D43" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E43" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F43" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G43" t="str">
-        <v>Move In/Move Out</v>
+        <v>Release</v>
       </c>
       <c r="H43" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I43" t="str">
         <v>No</v>
@@ -1659,28 +1659,28 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Dnyanesh Prakash Painjane</v>
+        <v>Jayoti Chatterji</v>
       </c>
       <c r="B44" t="str">
-        <v>dnyanesh.prakash.painjane@pwc.com</v>
+        <v>jayoti.chatterji@pwc.com</v>
       </c>
       <c r="C44" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D44" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E44" t="str">
-        <v>IR3.2</v>
+        <v>IR3.X</v>
       </c>
       <c r="F44" t="str">
-        <v>All</v>
+        <v>IR3.X</v>
       </c>
       <c r="G44" t="str">
-        <v>Move In/Transfer</v>
+        <v>Outage</v>
       </c>
       <c r="H44" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I44" t="str">
         <v>No</v>
@@ -1688,28 +1688,28 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Girlee P. Alvarado</v>
+        <v>Jitain Mohun</v>
       </c>
       <c r="B45" t="str">
-        <v>girlee.alvarado@pwc.com</v>
+        <v/>
       </c>
       <c r="C45" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D45" t="str">
-        <v>QA</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E45" t="str">
-        <v>IR3.2</v>
+        <v>IR3.X</v>
       </c>
       <c r="F45" t="str">
-        <v>All</v>
+        <v>IR3.X/IR4</v>
       </c>
       <c r="G45" t="str">
-        <v>Move Out/Transfer</v>
+        <v>Outage</v>
       </c>
       <c r="H45" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I45" t="str">
         <v>No</v>
@@ -1717,28 +1717,28 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Venugopal Sinde</v>
+        <v>John Jyothula</v>
       </c>
       <c r="B46" t="str">
         <v/>
       </c>
       <c r="C46" t="str">
-        <v>Infosys</v>
+        <v/>
       </c>
       <c r="D46" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E46" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F46" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G46" t="str">
-        <v>Move In/Move Out</v>
+        <v>Release</v>
       </c>
       <c r="H46" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I46" t="str">
         <v>No</v>
@@ -1746,28 +1746,28 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Raveendra Reddy</v>
+        <v>Kavita Jha</v>
       </c>
       <c r="B47" t="str">
-        <v>raveendra.t.reddy@pwc.com</v>
+        <v/>
       </c>
       <c r="C47" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D47" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E47" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F47" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G47" t="str">
-        <v>Transfer</v>
+        <v>Release</v>
       </c>
       <c r="H47" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I47" t="str">
         <v>No</v>
@@ -1775,13 +1775,13 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Naga Srilekha Thummalacheruvu</v>
+        <v>Keerthana Manjunath</v>
       </c>
       <c r="B48" t="str">
-        <v>naga.t.thummalacheruvu@pwc.com</v>
+        <v/>
       </c>
       <c r="C48" t="str">
-        <v>Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D48" t="str">
         <v>QA</v>
@@ -1793,7 +1793,7 @@
         <v>All</v>
       </c>
       <c r="G48" t="str">
-        <v>Move In</v>
+        <v>Transfer</v>
       </c>
       <c r="H48" t="str">
         <v/>
@@ -1804,28 +1804,28 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Israel L. Jacinto</v>
+        <v>Kishor S</v>
       </c>
       <c r="B49" t="str">
-        <v>israel.jacinto@pwc.com</v>
+        <v/>
       </c>
       <c r="C49" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D49" t="str">
-        <v>QA</v>
+        <v>Intern</v>
       </c>
       <c r="E49" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F49" t="str">
         <v>All</v>
       </c>
       <c r="G49" t="str">
-        <v>Move Out</v>
+        <v>Interns</v>
       </c>
       <c r="H49" t="str">
-        <v/>
+        <v>Interns</v>
       </c>
       <c r="I49" t="str">
         <v>No</v>
@@ -1833,25 +1833,25 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Keerthana Manjunath</v>
+        <v>Kodi Elangovan</v>
       </c>
       <c r="B50" t="str">
-        <v/>
+        <v>kodiyarasan.elangovan@pwc.com</v>
       </c>
       <c r="C50" t="str">
-        <v>Infosys</v>
+        <v>Manager</v>
       </c>
       <c r="D50" t="str">
-        <v>QA</v>
+        <v>Integration Lead</v>
       </c>
       <c r="E50" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F50" t="str">
         <v>All</v>
       </c>
       <c r="G50" t="str">
-        <v>Transfer</v>
+        <v>Integration</v>
       </c>
       <c r="H50" t="str">
         <v/>
@@ -1862,28 +1862,28 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Sonal Yadav</v>
+        <v>Krithika Harishchandra Shettigar</v>
       </c>
       <c r="B51" t="str">
-        <v>sonal.y.yadav@pwc.com</v>
+        <v/>
       </c>
       <c r="C51" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D51" t="str">
-        <v>QA</v>
+        <v>Intern</v>
       </c>
       <c r="E51" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F51" t="str">
         <v>All</v>
       </c>
       <c r="G51" t="str">
-        <v>Move In/Move Out</v>
+        <v>Interns</v>
       </c>
       <c r="H51" t="str">
-        <v/>
+        <v>Interns</v>
       </c>
       <c r="I51" t="str">
         <v>No</v>
@@ -1891,28 +1891,28 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Argene M. Francisco</v>
+        <v>Lokesh Sai</v>
       </c>
       <c r="B52" t="str">
-        <v>argene.francisco@pwc.com</v>
+        <v>lokesh.sai@pwc.com</v>
       </c>
       <c r="C52" t="str">
-        <v>Senior Associate</v>
+        <v>Associate</v>
       </c>
       <c r="D52" t="str">
         <v>QA</v>
       </c>
       <c r="E52" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F52" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G52" t="str">
-        <v>Move In/Transfer</v>
+        <v>Energy Management</v>
       </c>
       <c r="H52" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I52" t="str">
         <v>No</v>
@@ -1920,28 +1920,28 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Sanjana</v>
+        <v>Madhumita Kodidela</v>
       </c>
       <c r="B53" t="str">
-        <v/>
+        <v>madhumitha.kodidela@pwc.com</v>
       </c>
       <c r="C53" t="str">
-        <v>Infosys</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D53" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E53" t="str">
         <v>IR3.2</v>
       </c>
       <c r="F53" t="str">
-        <v>All</v>
+        <v>IR3.2</v>
       </c>
       <c r="G53" t="str">
         <v>Interactions/Search</v>
       </c>
       <c r="H53" t="str">
-        <v/>
+        <v>Dev POD 2/Sneha G</v>
       </c>
       <c r="I53" t="str">
         <v>No</v>
@@ -1949,13 +1949,13 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Pratik Mahajan</v>
+        <v>Maneesha</v>
       </c>
       <c r="B54" t="str">
-        <v>pratik.sunil.mahajan@pwc.com</v>
+        <v/>
       </c>
       <c r="C54" t="str">
-        <v>Senior Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D54" t="str">
         <v>QA</v>
@@ -1967,7 +1967,7 @@
         <v>All</v>
       </c>
       <c r="G54" t="str">
-        <v>Interactions/Search</v>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H54" t="str">
         <v/>
@@ -1978,13 +1978,13 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Nilesh</v>
+        <v>Mary Grace Carinan Nazareno</v>
       </c>
       <c r="B55" t="str">
-        <v/>
+        <v>mary.grace.nazareno@pwc.com</v>
       </c>
       <c r="C55" t="str">
-        <v>Infosys</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D55" t="str">
         <v>QA</v>
@@ -1996,7 +1996,7 @@
         <v>All</v>
       </c>
       <c r="G55" t="str">
-        <v>Account Maintenance</v>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H55" t="str">
         <v/>
@@ -2007,25 +2007,25 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Pritam</v>
+        <v>Matthew Rupas</v>
       </c>
       <c r="B56" t="str">
-        <v/>
+        <v>matthew.i.rupas@pwc.com</v>
       </c>
       <c r="C56" t="str">
-        <v>Infosys</v>
+        <v>Partner</v>
       </c>
       <c r="D56" t="str">
-        <v>QA</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E56" t="str">
-        <v>IR3.2</v>
+        <v>Leadership</v>
       </c>
       <c r="F56" t="str">
         <v>All</v>
       </c>
       <c r="G56" t="str">
-        <v>Account Maintenance</v>
+        <v>Program Leadership</v>
       </c>
       <c r="H56" t="str">
         <v/>
@@ -2036,28 +2036,28 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Smita</v>
+        <v>Mayand Mani</v>
       </c>
       <c r="B57" t="str">
         <v/>
       </c>
       <c r="C57" t="str">
-        <v>Infosys</v>
+        <v>Associate</v>
       </c>
       <c r="D57" t="str">
         <v>QA</v>
       </c>
       <c r="E57" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F57" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G57" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v>Energy Management</v>
       </c>
       <c r="H57" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I57" t="str">
         <v>No</v>
@@ -2065,28 +2065,28 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Vidyashree S R</v>
+        <v>Mayur Kinhekar</v>
       </c>
       <c r="B58" t="str">
-        <v>vidyashree.s.r@pwc.com</v>
+        <v>mayur.murlidhar.kinhekar@pwc.com</v>
       </c>
       <c r="C58" t="str">
         <v>Senior Associate</v>
       </c>
       <c r="D58" t="str">
-        <v>QA</v>
+        <v>Offshore SA</v>
       </c>
       <c r="E58" t="str">
-        <v>IR3.2</v>
+        <v>IR3.X</v>
       </c>
       <c r="F58" t="str">
-        <v>All</v>
+        <v>IR3.X/IR4</v>
       </c>
       <c r="G58" t="str">
-        <v>Payment &amp; Payment Options</v>
+        <v>Outage</v>
       </c>
       <c r="H58" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I58" t="str">
         <v>No</v>
@@ -2094,28 +2094,28 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Prasanna Nangnure</v>
+        <v>Michael O'shea</v>
       </c>
       <c r="B59" t="str">
-        <v>prasanna.y.nangnure@pwc.com</v>
+        <v>michael.o.oshea@pwc.com</v>
       </c>
       <c r="C59" t="str">
         <v>Associate</v>
       </c>
       <c r="D59" t="str">
-        <v>QA</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E59" t="str">
         <v>IR3.2</v>
       </c>
       <c r="F59" t="str">
-        <v>All</v>
+        <v>IR3.2</v>
       </c>
       <c r="G59" t="str">
-        <v>Billing Programs</v>
+        <v>Interactions/Search</v>
       </c>
       <c r="H59" t="str">
-        <v/>
+        <v>Dev POD 2/Sneha G</v>
       </c>
       <c r="I59" t="str">
         <v>No</v>
@@ -2123,25 +2123,25 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Nikita</v>
+        <v>Mounika Depuri</v>
       </c>
       <c r="B60" t="str">
-        <v/>
+        <v>mounika.depuri@pwc.com</v>
       </c>
       <c r="C60" t="str">
-        <v>Infosys</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D60" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E60" t="str">
         <v>IR3.2</v>
       </c>
       <c r="F60" t="str">
-        <v>All</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G60" t="str">
-        <v>Payment &amp; Payment Options</v>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H60" t="str">
         <v/>
@@ -2152,28 +2152,28 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Mary Grace Carinan Nazareno</v>
+        <v>Mrithika Kumaresan</v>
       </c>
       <c r="B61" t="str">
-        <v>mary.grace.nazareno@pwc.com</v>
+        <v/>
       </c>
       <c r="C61" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D61" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E61" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F61" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G61" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v>Release</v>
       </c>
       <c r="H61" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I61" t="str">
         <v>No</v>
@@ -2181,28 +2181,28 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Pornima Rajguru</v>
+        <v>Mylavarapu V N R Saketh</v>
       </c>
       <c r="B62" t="str">
-        <v>Poornima.atul.rajguru@pwc.com</v>
+        <v>mylavarapu.v.n.r.saketh@pwc.com</v>
       </c>
       <c r="C62" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D62" t="str">
-        <v>Dev Lead</v>
+        <v>Dev</v>
       </c>
       <c r="E62" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="F62" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="G62" t="str">
-        <v>Outage</v>
+        <v>Energy Management</v>
       </c>
       <c r="H62" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I62" t="str">
         <v>No</v>
@@ -2210,25 +2210,25 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Jitain Mohun</v>
+        <v>Naga Srilekha Thummalacheruvu</v>
       </c>
       <c r="B63" t="str">
-        <v/>
+        <v>naga.t.thummalacheruvu@pwc.com</v>
       </c>
       <c r="C63" t="str">
-        <v>Manager</v>
+        <v>Associate</v>
       </c>
       <c r="D63" t="str">
-        <v>Onshore SA</v>
+        <v>QA</v>
       </c>
       <c r="E63" t="str">
-        <v>IR3.X</v>
+        <v>IR3.2</v>
       </c>
       <c r="F63" t="str">
-        <v>IR3.X/IR4</v>
+        <v>All</v>
       </c>
       <c r="G63" t="str">
-        <v>Outage</v>
+        <v>Move In</v>
       </c>
       <c r="H63" t="str">
         <v/>
@@ -2239,28 +2239,28 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Mayur Kinhekar</v>
+        <v>Naman Hiran</v>
       </c>
       <c r="B64" t="str">
-        <v>mayur.murlidhar.kinhekar@pwc.com</v>
+        <v>naman.hiran@pwc.com</v>
       </c>
       <c r="C64" t="str">
         <v>Senior Associate</v>
       </c>
       <c r="D64" t="str">
-        <v>Offshore SA</v>
+        <v>Dev</v>
       </c>
       <c r="E64" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="F64" t="str">
-        <v>IR3.X/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G64" t="str">
-        <v>Outage</v>
+        <v>Energy Management</v>
       </c>
       <c r="H64" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I64" t="str">
         <v>No</v>
@@ -2268,25 +2268,25 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Jayoti Chatterji</v>
+        <v>Namrata Uttareshwar Bansode</v>
       </c>
       <c r="B65" t="str">
-        <v>jayoti.chatterji@pwc.com</v>
+        <v>namrata.uttareshwar.bansode@pwc.com</v>
       </c>
       <c r="C65" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D65" t="str">
-        <v>Dev</v>
+        <v>Offshore SA</v>
       </c>
       <c r="E65" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="F65" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="G65" t="str">
-        <v>Outage</v>
+        <v>Billing &amp; Usage/Payment Programs</v>
       </c>
       <c r="H65" t="str">
         <v/>
@@ -2297,28 +2297,28 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Aakanksha</v>
+        <v>Niket Saxena</v>
       </c>
       <c r="B66" t="str">
         <v/>
       </c>
       <c r="C66" t="str">
-        <v>Infosys</v>
+        <v/>
       </c>
       <c r="D66" t="str">
-        <v>QA</v>
+        <v>Lead</v>
       </c>
       <c r="E66" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="F66" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="G66" t="str">
-        <v>Outage</v>
+        <v>Release</v>
       </c>
       <c r="H66" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I66" t="str">
         <v>No</v>
@@ -2326,7 +2326,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Diksha</v>
+        <v>Nikita</v>
       </c>
       <c r="B67" t="str">
         <v/>
@@ -2338,13 +2338,13 @@
         <v>QA</v>
       </c>
       <c r="E67" t="str">
-        <v>IR3.X</v>
+        <v>IR3.2</v>
       </c>
       <c r="F67" t="str">
-        <v>IR3.X</v>
+        <v>All</v>
       </c>
       <c r="G67" t="str">
-        <v>Outage</v>
+        <v>Payment &amp; Payment Options</v>
       </c>
       <c r="H67" t="str">
         <v/>
@@ -2355,7 +2355,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Sahithi Manne</v>
+        <v>Nilesh</v>
       </c>
       <c r="B68" t="str">
         <v/>
@@ -2364,16 +2364,16 @@
         <v>Infosys</v>
       </c>
       <c r="D68" t="str">
-        <v>Onshore SA</v>
+        <v>QA</v>
       </c>
       <c r="E68" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F68" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G68" t="str">
-        <v>Billing &amp; Usage/Payment Programs | Energy Management</v>
+        <v>Account Maintenance</v>
       </c>
       <c r="H68" t="str">
         <v/>
@@ -2384,28 +2384,28 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Namrata Uttareshwar Bansode</v>
+        <v>Nishi Jain</v>
       </c>
       <c r="B69" t="str">
-        <v>namrata.uttareshwar.bansode@pwc.com</v>
+        <v/>
       </c>
       <c r="C69" t="str">
-        <v>Manager</v>
+        <v/>
       </c>
       <c r="D69" t="str">
-        <v>Offshore SA</v>
+        <v>Dev</v>
       </c>
       <c r="E69" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F69" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G69" t="str">
-        <v>Billing &amp; Usage/Payment Programs</v>
+        <v>Release</v>
       </c>
       <c r="H69" t="str">
-        <v/>
+        <v>Dev POD 6/Aditya</v>
       </c>
       <c r="I69" t="str">
         <v>No</v>
@@ -2413,10 +2413,10 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Shivam Surendra Shete</v>
+        <v>Nishi Narendra Jain</v>
       </c>
       <c r="B70" t="str">
-        <v>shivam.surendra.shete@pwc.com</v>
+        <v>jain.u.nishi@pwc.com</v>
       </c>
       <c r="C70" t="str">
         <v>Senior Associate</v>
@@ -2425,13 +2425,13 @@
         <v>Dev</v>
       </c>
       <c r="E70" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F70" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G70" t="str">
-        <v>Billing &amp; Usage/Payment Programs</v>
+        <v>Account Maintenance</v>
       </c>
       <c r="H70" t="str">
         <v/>
@@ -2442,13 +2442,13 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Rubasri S</v>
+        <v>Nivetha Sudharsanam</v>
       </c>
       <c r="B71" t="str">
-        <v>rubasri.x.s@pwc.com</v>
+        <v/>
       </c>
       <c r="C71" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D71" t="str">
         <v>Dev</v>
@@ -2460,10 +2460,10 @@
         <v>IR4</v>
       </c>
       <c r="G71" t="str">
-        <v>Billing &amp; Usage/Payment Programs</v>
+        <v>Release</v>
       </c>
       <c r="H71" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I71" t="str">
         <v>No</v>
@@ -2471,25 +2471,25 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Rohan Bandla</v>
+        <v>Paarth Sonwaney</v>
       </c>
       <c r="B72" t="str">
-        <v/>
+        <v>paarth.sonwaney@pwc.com</v>
       </c>
       <c r="C72" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D72" t="str">
-        <v>Onshore SA</v>
+        <v>PMO</v>
       </c>
       <c r="E72" t="str">
-        <v>IR4</v>
+        <v>Leadership</v>
       </c>
       <c r="F72" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G72" t="str">
-        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
+        <v>PMO</v>
       </c>
       <c r="H72" t="str">
         <v/>
@@ -2500,16 +2500,16 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Amarjeet Singh</v>
+        <v>Parul Prasad</v>
       </c>
       <c r="B73" t="str">
-        <v>amarjeet.singh@pwc.com</v>
+        <v>parul.prasad@pwc.com</v>
       </c>
       <c r="C73" t="str">
         <v>Senior Associate</v>
       </c>
       <c r="D73" t="str">
-        <v>Dev</v>
+        <v>Offshore SA</v>
       </c>
       <c r="E73" t="str">
         <v>IR4</v>
@@ -2518,10 +2518,10 @@
         <v>IR4</v>
       </c>
       <c r="G73" t="str">
-        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
+        <v>Energy Management</v>
       </c>
       <c r="H73" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I73" t="str">
         <v>No</v>
@@ -2529,28 +2529,28 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Ankit Mishra</v>
+        <v>Piyush Singh</v>
       </c>
       <c r="B74" t="str">
-        <v>ankit.b.mishra@pwc.com</v>
+        <v>piyush.ss.singh@pwc.com</v>
       </c>
       <c r="C74" t="str">
-        <v>Senior Associate</v>
+        <v>Associate</v>
       </c>
       <c r="D74" t="str">
         <v>Dev</v>
       </c>
       <c r="E74" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F74" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G74" t="str">
-        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H74" t="str">
-        <v/>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I74" t="str">
         <v>No</v>
@@ -2558,28 +2558,28 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Cheruku Pranay Reddy</v>
+        <v>Pornima Rajguru</v>
       </c>
       <c r="B75" t="str">
-        <v>cheruku.pranay.reddy@pwc.com</v>
+        <v>Poornima.atul.rajguru@pwc.com</v>
       </c>
       <c r="C75" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D75" t="str">
-        <v>Dev</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E75" t="str">
-        <v>IR4</v>
+        <v>IR3.X</v>
       </c>
       <c r="F75" t="str">
-        <v>IR4</v>
+        <v>IR3.X</v>
       </c>
       <c r="G75" t="str">
-        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
+        <v>Outage</v>
       </c>
       <c r="H75" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I75" t="str">
         <v>No</v>
@@ -2587,28 +2587,28 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Anurag Jakkal</v>
+        <v>Potumanchi Sree Yashana</v>
       </c>
       <c r="B76" t="str">
-        <v>jakkal.anurag.surendra@pwc.com</v>
+        <v/>
       </c>
       <c r="C76" t="str">
-        <v>Manager</v>
+        <v/>
       </c>
       <c r="D76" t="str">
-        <v>Dev Lead</v>
+        <v>Intern</v>
       </c>
       <c r="E76" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F76" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G76" t="str">
-        <v>Energy Management</v>
+        <v>Interns</v>
       </c>
       <c r="H76" t="str">
-        <v/>
+        <v>Interns</v>
       </c>
       <c r="I76" t="str">
         <v>No</v>
@@ -2616,16 +2616,16 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Parul Prasad</v>
+        <v>Pradeep Lambu</v>
       </c>
       <c r="B77" t="str">
-        <v>parul.prasad@pwc.com</v>
+        <v/>
       </c>
       <c r="C77" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D77" t="str">
-        <v>Offshore SA</v>
+        <v>Dev</v>
       </c>
       <c r="E77" t="str">
         <v>IR4</v>
@@ -2634,10 +2634,10 @@
         <v>IR4</v>
       </c>
       <c r="G77" t="str">
-        <v>Energy Management</v>
+        <v>Release</v>
       </c>
       <c r="H77" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I77" t="str">
         <v>No</v>
@@ -2645,25 +2645,25 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Aaditi Madhavan</v>
+        <v>Pranav Singh</v>
       </c>
       <c r="B78" t="str">
-        <v>aaditi.madhavan@pwc.com</v>
+        <v>pranav.s.singh@pwc.com</v>
       </c>
       <c r="C78" t="str">
         <v>Senior Associate</v>
       </c>
       <c r="D78" t="str">
-        <v>Dev</v>
+        <v>Integration Dev</v>
       </c>
       <c r="E78" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F78" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G78" t="str">
-        <v>Energy Management</v>
+        <v>Integration</v>
       </c>
       <c r="H78" t="str">
         <v/>
@@ -2674,13 +2674,13 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Naman Hiran</v>
+        <v>Prasad P</v>
       </c>
       <c r="B79" t="str">
-        <v>naman.hiran@pwc.com</v>
+        <v/>
       </c>
       <c r="C79" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D79" t="str">
         <v>Dev</v>
@@ -2692,10 +2692,10 @@
         <v>IR4</v>
       </c>
       <c r="G79" t="str">
-        <v>Energy Management</v>
+        <v>Release</v>
       </c>
       <c r="H79" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I79" t="str">
         <v>No</v>
@@ -2703,25 +2703,25 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Mylavarapu V N R Saketh</v>
+        <v>Prasanna Nangnure</v>
       </c>
       <c r="B80" t="str">
-        <v>mylavarapu.v.n.r.saketh@pwc.com</v>
+        <v>prasanna.y.nangnure@pwc.com</v>
       </c>
       <c r="C80" t="str">
-        <v>Senior Associate</v>
+        <v>Associate</v>
       </c>
       <c r="D80" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E80" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F80" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G80" t="str">
-        <v>Energy Management</v>
+        <v>Billing Programs</v>
       </c>
       <c r="H80" t="str">
         <v/>
@@ -2732,10 +2732,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Venkata Sai Harika Ambati</v>
+        <v>Pratik Kurdukar</v>
       </c>
       <c r="B81" t="str">
-        <v>venkata.sai.harika.ambati@pwc.com</v>
+        <v>pratik.k.kurdukar@pwc.com</v>
       </c>
       <c r="C81" t="str">
         <v>Associate</v>
@@ -2744,16 +2744,16 @@
         <v>Dev</v>
       </c>
       <c r="E81" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F81" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G81" t="str">
-        <v>Energy Management</v>
+        <v>Case Management</v>
       </c>
       <c r="H81" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I81" t="str">
         <v>No</v>
@@ -2761,25 +2761,25 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Ashit Prashant Golwala</v>
+        <v>Pratik Mahajan</v>
       </c>
       <c r="B82" t="str">
-        <v>ashit.prashant.golwala@pwc.com</v>
+        <v>pratik.sunil.mahajan@pwc.com</v>
       </c>
       <c r="C82" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D82" t="str">
         <v>QA</v>
       </c>
       <c r="E82" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F82" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G82" t="str">
-        <v>Energy Management</v>
+        <v>Interactions/Search</v>
       </c>
       <c r="H82" t="str">
         <v/>
@@ -2790,25 +2790,25 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Sagnik Chakraborty</v>
+        <v>Pritam</v>
       </c>
       <c r="B83" t="str">
-        <v>sagnik.chakraborty@pwc.com</v>
+        <v/>
       </c>
       <c r="C83" t="str">
-        <v>Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D83" t="str">
         <v>QA</v>
       </c>
       <c r="E83" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F83" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G83" t="str">
-        <v>Energy Management</v>
+        <v>Account Maintenance</v>
       </c>
       <c r="H83" t="str">
         <v/>
@@ -2819,25 +2819,25 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>Lokesh Sai</v>
+        <v>Rajaraman A</v>
       </c>
       <c r="B84" t="str">
-        <v>lokesh.sai@pwc.com</v>
+        <v>rajaraman.a@pwc.com</v>
       </c>
       <c r="C84" t="str">
-        <v>Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D84" t="str">
-        <v>QA</v>
+        <v>QA Lead</v>
       </c>
       <c r="E84" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F84" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G84" t="str">
-        <v>Energy Management</v>
+        <v>QA - All Value Streams</v>
       </c>
       <c r="H84" t="str">
         <v/>
@@ -2848,25 +2848,25 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Mayand Mani</v>
+        <v>Raveendra Reddy</v>
       </c>
       <c r="B85" t="str">
-        <v/>
+        <v>raveendra.t.reddy@pwc.com</v>
       </c>
       <c r="C85" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D85" t="str">
         <v>QA</v>
       </c>
       <c r="E85" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F85" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G85" t="str">
-        <v>Energy Management</v>
+        <v>Transfer</v>
       </c>
       <c r="H85" t="str">
         <v/>
@@ -2877,25 +2877,25 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Nishi Jain</v>
+        <v>Rhitik Khanna</v>
       </c>
       <c r="B86" t="str">
-        <v/>
+        <v>rhitik.khanna@pwc.com</v>
       </c>
       <c r="C86" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D86" t="str">
-        <v>Dev</v>
+        <v>DevOps</v>
       </c>
       <c r="E86" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F86" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G86" t="str">
-        <v/>
+        <v>DevOps</v>
       </c>
       <c r="H86" t="str">
         <v/>
@@ -2906,7 +2906,7 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>FPL</v>
+        <v>Rida Maryam Mohammad</v>
       </c>
       <c r="B87" t="str">
         <v/>
@@ -2915,19 +2915,19 @@
         <v/>
       </c>
       <c r="D87" t="str">
-        <v>Onshore Solution Analyst</v>
+        <v>Dev</v>
       </c>
       <c r="E87" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F87" t="str">
         <v>IR4</v>
       </c>
       <c r="G87" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H87" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I87" t="str">
         <v>No</v>
@@ -2935,28 +2935,28 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Sona Muthayala</v>
+        <v>Rinky Chawla</v>
       </c>
       <c r="B88" t="str">
-        <v/>
+        <v>rinky.chawla@pwc.com</v>
       </c>
       <c r="C88" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D88" t="str">
-        <v>Dev</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E88" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F88" t="str">
-        <v>IR4</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G88" t="str">
-        <v/>
+        <v>Case Management</v>
       </c>
       <c r="H88" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I88" t="str">
         <v>No</v>
@@ -2964,25 +2964,25 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Sriharsha Sambaraj</v>
+        <v>Ritesh Nanda</v>
       </c>
       <c r="B89" t="str">
-        <v/>
+        <v>ritesh.nanda@pwc.com</v>
       </c>
       <c r="C89" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D89" t="str">
-        <v>Dev</v>
+        <v>DevOps Lead</v>
       </c>
       <c r="E89" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F89" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G89" t="str">
-        <v/>
+        <v>DevOps</v>
       </c>
       <c r="H89" t="str">
         <v/>
@@ -2993,7 +2993,7 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Russell Stein</v>
+        <v>Rodolfo Duarte</v>
       </c>
       <c r="B90" t="str">
         <v/>
@@ -3002,19 +3002,19 @@
         <v/>
       </c>
       <c r="D90" t="str">
-        <v>Onshore Solution Analyst</v>
+        <v>Team</v>
       </c>
       <c r="E90" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F90" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G90" t="str">
-        <v/>
+        <v>DevOps POD</v>
       </c>
       <c r="H90" t="str">
-        <v/>
+        <v>DevOps POD</v>
       </c>
       <c r="I90" t="str">
         <v>No</v>
@@ -3022,25 +3022,25 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Namrata Bansode</v>
+        <v>Rohan Bandla</v>
       </c>
       <c r="B91" t="str">
         <v/>
       </c>
       <c r="C91" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D91" t="str">
-        <v>Offshore Solution Analyst</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E91" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F91" t="str">
         <v>IR4</v>
       </c>
       <c r="G91" t="str">
-        <v/>
+        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
       <c r="H91" t="str">
         <v/>
@@ -3051,25 +3051,25 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Shivam Shete</v>
+        <v>Rubasri S</v>
       </c>
       <c r="B92" t="str">
-        <v/>
+        <v>rubasri.x.s@pwc.com</v>
       </c>
       <c r="C92" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D92" t="str">
         <v>Dev</v>
       </c>
       <c r="E92" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F92" t="str">
         <v>IR4</v>
       </c>
       <c r="G92" t="str">
-        <v/>
+        <v>Billing &amp; Usage/Payment Programs</v>
       </c>
       <c r="H92" t="str">
         <v/>
@@ -3080,28 +3080,28 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>Sahil Thadani</v>
+        <v>Sagnik Chakraborty</v>
       </c>
       <c r="B93" t="str">
-        <v/>
+        <v>sagnik.chakraborty@pwc.com</v>
       </c>
       <c r="C93" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D93" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E93" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F93" t="str">
         <v>IR4</v>
       </c>
       <c r="G93" t="str">
-        <v/>
+        <v>Energy Management</v>
       </c>
       <c r="H93" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I93" t="str">
         <v>No</v>
@@ -3109,28 +3109,28 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>Kankshitha Yalamuru</v>
+        <v>Sahithi Manne</v>
       </c>
       <c r="B94" t="str">
         <v/>
       </c>
       <c r="C94" t="str">
-        <v/>
+        <v>Infosys</v>
       </c>
       <c r="D94" t="str">
-        <v>Dev</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E94" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F94" t="str">
         <v>IR4</v>
       </c>
       <c r="G94" t="str">
-        <v/>
+        <v>Billing &amp; Usage/Payment Programs | Energy Management</v>
       </c>
       <c r="H94" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I94" t="str">
         <v>No</v>
@@ -3138,25 +3138,25 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>Sahithi Chebrolu</v>
+        <v>Sandesh Saravanan</v>
       </c>
       <c r="B95" t="str">
-        <v/>
+        <v>sandesh.saravanan@pwc.com</v>
       </c>
       <c r="C95" t="str">
-        <v/>
+        <v>Intern</v>
       </c>
       <c r="D95" t="str">
         <v>Dev</v>
       </c>
       <c r="E95" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F95" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G95" t="str">
-        <v/>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H95" t="str">
         <v/>
@@ -3167,25 +3167,25 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Prayas Abinash</v>
+        <v>Sanjana</v>
       </c>
       <c r="B96" t="str">
         <v/>
       </c>
       <c r="C96" t="str">
-        <v/>
+        <v>Infosys</v>
       </c>
       <c r="D96" t="str">
-        <v>Offshore Solution Analyst</v>
+        <v>QA</v>
       </c>
       <c r="E96" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F96" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G96" t="str">
-        <v/>
+        <v>Interactions/Search</v>
       </c>
       <c r="H96" t="str">
         <v/>
@@ -3196,25 +3196,25 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>Pranay Reddy</v>
+        <v>Sanket Mundargi</v>
       </c>
       <c r="B97" t="str">
-        <v/>
+        <v>sanket.mundargi@pwc.com</v>
       </c>
       <c r="C97" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D97" t="str">
-        <v>Dev</v>
+        <v>Windsurf/Performance Dev</v>
       </c>
       <c r="E97" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F97" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G97" t="str">
-        <v/>
+        <v>Windsurf/Performance</v>
       </c>
       <c r="H97" t="str">
         <v/>
@@ -3225,7 +3225,7 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>Manu Tyagi</v>
+        <v>Sanniboina Murali Krishna</v>
       </c>
       <c r="B98" t="str">
         <v/>
@@ -3237,16 +3237,16 @@
         <v>Dev</v>
       </c>
       <c r="E98" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F98" t="str">
         <v>IR4</v>
       </c>
       <c r="G98" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H98" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I98" t="str">
         <v>No</v>
@@ -3254,25 +3254,25 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Sunandha Sanda</v>
+        <v>Santosh Kumar Jangam</v>
       </c>
       <c r="B99" t="str">
-        <v/>
+        <v>santosh.kumar.jangam@pwc.com</v>
       </c>
       <c r="C99" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D99" t="str">
-        <v>Dev</v>
+        <v>DevOps</v>
       </c>
       <c r="E99" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F99" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G99" t="str">
-        <v/>
+        <v>DevOps</v>
       </c>
       <c r="H99" t="str">
         <v/>
@@ -3283,25 +3283,25 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>Jason Pereira</v>
+        <v>Shabnam Nasreen</v>
       </c>
       <c r="B100" t="str">
-        <v/>
+        <v>shabnam.nasreen@pwc.com</v>
       </c>
       <c r="C100" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D100" t="str">
-        <v>Lead</v>
+        <v>DevOps Lead</v>
       </c>
       <c r="E100" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F100" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G100" t="str">
-        <v/>
+        <v>DevOps</v>
       </c>
       <c r="H100" t="str">
         <v/>
@@ -3312,25 +3312,25 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Akhil Palakeel</v>
+        <v>Shanta Samlal</v>
       </c>
       <c r="B101" t="str">
-        <v/>
+        <v>shanta.samlal@pwc.com</v>
       </c>
       <c r="C101" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D101" t="str">
-        <v>Offshore Solution Analyst</v>
+        <v>PMO</v>
       </c>
       <c r="E101" t="str">
-        <v/>
+        <v>Leadership</v>
       </c>
       <c r="F101" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G101" t="str">
-        <v/>
+        <v>PMO</v>
       </c>
       <c r="H101" t="str">
         <v/>
@@ -3341,25 +3341,25 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>Sridaran N M</v>
+        <v>Shatakshi Srivastava</v>
       </c>
       <c r="B102" t="str">
-        <v/>
+        <v>shatakshi.s.srivastava@pwc.com</v>
       </c>
       <c r="C102" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D102" t="str">
-        <v>Dev</v>
+        <v>DevOps</v>
       </c>
       <c r="E102" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F102" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G102" t="str">
-        <v/>
+        <v>DevOps</v>
       </c>
       <c r="H102" t="str">
         <v/>
@@ -3370,28 +3370,28 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>Prasad P</v>
+        <v>Shikhar Sanjeev</v>
       </c>
       <c r="B103" t="str">
-        <v/>
+        <v>shikhar.sanjeev@pwc.com</v>
       </c>
       <c r="C103" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D103" t="str">
         <v>Dev</v>
       </c>
       <c r="E103" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F103" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G103" t="str">
-        <v/>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H103" t="str">
-        <v/>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I103" t="str">
         <v>No</v>
@@ -3399,25 +3399,25 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>Pradeep Lambu</v>
+        <v>Shivam Surendra Shete</v>
       </c>
       <c r="B104" t="str">
-        <v/>
+        <v>shivam.surendra.shete@pwc.com</v>
       </c>
       <c r="C104" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D104" t="str">
         <v>Dev</v>
       </c>
       <c r="E104" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F104" t="str">
         <v>IR4</v>
       </c>
       <c r="G104" t="str">
-        <v/>
+        <v>Billing &amp; Usage/Payment Programs</v>
       </c>
       <c r="H104" t="str">
         <v/>
@@ -3428,7 +3428,7 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>Nivetha Sudharsanam</v>
+        <v>Shravya Nanjundaswamy</v>
       </c>
       <c r="B105" t="str">
         <v/>
@@ -3440,16 +3440,16 @@
         <v>Dev</v>
       </c>
       <c r="E105" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F105" t="str">
         <v>IR4</v>
       </c>
       <c r="G105" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H105" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I105" t="str">
         <v>No</v>
@@ -3457,28 +3457,28 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>Sweta Sharma</v>
+        <v>Shreya LNU</v>
       </c>
       <c r="B106" t="str">
-        <v/>
+        <v>shreya.l.lnu@pwc.com</v>
       </c>
       <c r="C106" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D106" t="str">
-        <v>Lead</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E106" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F106" t="str">
-        <v>IR4</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G106" t="str">
-        <v/>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H106" t="str">
-        <v/>
+        <v>Dev POD 1/Shreya</v>
       </c>
       <c r="I106" t="str">
         <v>No</v>
@@ -3486,25 +3486,25 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>Shravya Nanjundaswamy</v>
+        <v>Smita</v>
       </c>
       <c r="B107" t="str">
         <v/>
       </c>
       <c r="C107" t="str">
-        <v/>
+        <v>Infosys</v>
       </c>
       <c r="D107" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E107" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F107" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G107" t="str">
-        <v/>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H107" t="str">
         <v/>
@@ -3515,28 +3515,28 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>Rida Maryam Mohammad</v>
+        <v>Sneha Girigoudar</v>
       </c>
       <c r="B108" t="str">
-        <v/>
+        <v>sneha.raosaheb.girigoudar@pwc.com</v>
       </c>
       <c r="C108" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D108" t="str">
-        <v>Dev</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E108" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F108" t="str">
-        <v>IR4</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G108" t="str">
-        <v/>
+        <v>Interactions/Search | Correspondence/360s/PEXT/Account Maintenance</v>
       </c>
       <c r="H108" t="str">
-        <v/>
+        <v>Dev POD 2/Sneha G</v>
       </c>
       <c r="I108" t="str">
         <v>No</v>
@@ -3544,25 +3544,25 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>Surya Teja Poka</v>
+        <v>Sonal Yadav</v>
       </c>
       <c r="B109" t="str">
-        <v/>
+        <v>sonal.y.yadav@pwc.com</v>
       </c>
       <c r="C109" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D109" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E109" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F109" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G109" t="str">
-        <v/>
+        <v>Move In/Move Out</v>
       </c>
       <c r="H109" t="str">
         <v/>
@@ -3573,7 +3573,7 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>Kavita Jha</v>
+        <v>Sree Sowndarya Barani K</v>
       </c>
       <c r="B110" t="str">
         <v/>
@@ -3585,16 +3585,16 @@
         <v>Dev</v>
       </c>
       <c r="E110" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F110" t="str">
         <v>IR4</v>
       </c>
       <c r="G110" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H110" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I110" t="str">
         <v>No</v>
@@ -3602,7 +3602,7 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>Sanniboina Murali Krishna</v>
+        <v>Sridaran N M</v>
       </c>
       <c r="B111" t="str">
         <v/>
@@ -3614,16 +3614,16 @@
         <v>Dev</v>
       </c>
       <c r="E111" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F111" t="str">
         <v>IR4</v>
       </c>
       <c r="G111" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H111" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I111" t="str">
         <v>No</v>
@@ -3631,65 +3631,65 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>Tameka Robinson</v>
+        <v>Sujith Pillai</v>
       </c>
       <c r="B112" t="str">
-        <v/>
+        <v>sujith.s.pillai@pwc.com</v>
       </c>
       <c r="C112" t="str">
-        <v/>
+        <v>Director</v>
       </c>
       <c r="D112" t="str">
-        <v>Lead</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E112" t="str">
-        <v/>
+        <v>Leadership</v>
       </c>
       <c r="F112" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G112" t="str">
-        <v/>
+        <v>Program Leadership</v>
       </c>
       <c r="H112" t="str">
         <v/>
       </c>
       <c r="I112" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>Maria Vidal Parra</v>
+        <v>Suraj Ghodmare</v>
       </c>
       <c r="B113" t="str">
-        <v/>
+        <v>suraj.ghodmare@pwc.com</v>
       </c>
       <c r="C113" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D113" t="str">
-        <v>Scrum Master</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E113" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F113" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G113" t="str">
-        <v/>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H113" t="str">
-        <v/>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I113" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>Naveen Tayal</v>
+        <v>Surya Teja Poka</v>
       </c>
       <c r="B114" t="str">
         <v/>
@@ -3698,19 +3698,19 @@
         <v/>
       </c>
       <c r="D114" t="str">
-        <v>Onshore Solution Analyst</v>
+        <v>Dev</v>
       </c>
       <c r="E114" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F114" t="str">
         <v>IR4</v>
       </c>
       <c r="G114" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H114" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I114" t="str">
         <v>No</v>
@@ -3718,25 +3718,25 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>Harsh Shah</v>
+        <v>Susan Matthews</v>
       </c>
       <c r="B115" t="str">
-        <v/>
+        <v>susan.m.mathew@pwc.com</v>
       </c>
       <c r="C115" t="str">
-        <v/>
+        <v>Senior Manager</v>
       </c>
       <c r="D115" t="str">
-        <v>Onshore Solution Analyst</v>
+        <v>Business Architect</v>
       </c>
       <c r="E115" t="str">
-        <v/>
+        <v>Leadership</v>
       </c>
       <c r="F115" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G115" t="str">
-        <v/>
+        <v>Architecture</v>
       </c>
       <c r="H115" t="str">
         <v/>
@@ -3747,7 +3747,7 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>Sama Balayeva</v>
+        <v>Sweta Sharma</v>
       </c>
       <c r="B116" t="str">
         <v/>
@@ -3756,19 +3756,19 @@
         <v/>
       </c>
       <c r="D116" t="str">
-        <v>Onshore Solution Analyst</v>
+        <v>Lead</v>
       </c>
       <c r="E116" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F116" t="str">
         <v>IR4</v>
       </c>
       <c r="G116" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H116" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I116" t="str">
         <v>No</v>
@@ -3776,7 +3776,7 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>Jake Garrell</v>
+        <v>TBD</v>
       </c>
       <c r="B117" t="str">
         <v/>
@@ -3788,16 +3788,16 @@
         <v>Dev</v>
       </c>
       <c r="E117" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F117" t="str">
         <v>IR4</v>
       </c>
       <c r="G117" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H117" t="str">
-        <v/>
+        <v>Dev POD 6/Aditya</v>
       </c>
       <c r="I117" t="str">
         <v>No</v>
@@ -3805,25 +3805,25 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>John Harrison</v>
+        <v>Ted Capaldi</v>
       </c>
       <c r="B118" t="str">
-        <v/>
+        <v>theodore.capaldi@pwc.com</v>
       </c>
       <c r="C118" t="str">
-        <v/>
+        <v>Partner</v>
       </c>
       <c r="D118" t="str">
-        <v>Dev</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E118" t="str">
-        <v/>
+        <v>Leadership</v>
       </c>
       <c r="F118" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G118" t="str">
-        <v/>
+        <v>Program Leadership</v>
       </c>
       <c r="H118" t="str">
         <v/>
@@ -3834,25 +3834,25 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>Shashank Satvai</v>
+        <v>Tyaga Pati</v>
       </c>
       <c r="B119" t="str">
-        <v/>
+        <v>tyaga.pati@pwc.com</v>
       </c>
       <c r="C119" t="str">
-        <v/>
+        <v>Senior Manager</v>
       </c>
       <c r="D119" t="str">
-        <v>Dev</v>
+        <v>Solution Architect</v>
       </c>
       <c r="E119" t="str">
-        <v/>
+        <v>Leadership</v>
       </c>
       <c r="F119" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G119" t="str">
-        <v/>
+        <v>Architecture</v>
       </c>
       <c r="H119" t="str">
         <v/>
@@ -3863,25 +3863,25 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>Bryan Camacho</v>
+        <v>Vasudha Tandon</v>
       </c>
       <c r="B120" t="str">
-        <v/>
+        <v>vasudha.tandon@pwc.com</v>
       </c>
       <c r="C120" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D120" t="str">
-        <v>Dev</v>
+        <v>Integration Dev</v>
       </c>
       <c r="E120" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F120" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G120" t="str">
-        <v/>
+        <v>Integration</v>
       </c>
       <c r="H120" t="str">
         <v/>
@@ -3892,28 +3892,28 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>Yolanda Espinoza</v>
+        <v>Venkata Sai Harika Ambati</v>
       </c>
       <c r="B121" t="str">
-        <v/>
+        <v>venkata.sai.harika.ambati@pwc.com</v>
       </c>
       <c r="C121" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D121" t="str">
         <v>Dev</v>
       </c>
       <c r="E121" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F121" t="str">
         <v>IR4</v>
       </c>
       <c r="G121" t="str">
-        <v/>
+        <v>Energy Management</v>
       </c>
       <c r="H121" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I121" t="str">
         <v>No</v>
@@ -3921,25 +3921,25 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>Santhosh Maduri</v>
+        <v>Venugopal Sinde</v>
       </c>
       <c r="B122" t="str">
         <v/>
       </c>
       <c r="C122" t="str">
-        <v/>
+        <v>Infosys</v>
       </c>
       <c r="D122" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E122" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F122" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G122" t="str">
-        <v/>
+        <v>Move In/Move Out</v>
       </c>
       <c r="H122" t="str">
         <v/>
@@ -3950,25 +3950,25 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>Ankit Verma</v>
+        <v>Vidyashree S R</v>
       </c>
       <c r="B123" t="str">
-        <v/>
+        <v>vidyashree.s.r@pwc.com</v>
       </c>
       <c r="C123" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D123" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E123" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F123" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G123" t="str">
-        <v/>
+        <v>Payment &amp; Payment Options</v>
       </c>
       <c r="H123" t="str">
         <v/>
@@ -3979,25 +3979,25 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>Sree Sowndarya Barani K</v>
+        <v>Vinay Vadrevu</v>
       </c>
       <c r="B124" t="str">
         <v/>
       </c>
       <c r="C124" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D124" t="str">
-        <v>Dev</v>
+        <v>DevOps</v>
       </c>
       <c r="E124" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F124" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G124" t="str">
-        <v/>
+        <v>DevOps</v>
       </c>
       <c r="H124" t="str">
         <v/>
@@ -4008,7 +4008,7 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>John Jyothula</v>
+        <v>Ziyad Auti</v>
       </c>
       <c r="B125" t="str">
         <v/>
@@ -4017,549 +4017,27 @@
         <v/>
       </c>
       <c r="D125" t="str">
-        <v>Dev</v>
+        <v>Intern</v>
       </c>
       <c r="E125" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F125" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G125" t="str">
-        <v/>
+        <v>Interns</v>
       </c>
       <c r="H125" t="str">
-        <v/>
+        <v>Interns</v>
       </c>
       <c r="I125" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="str">
-        <v>Niket Saxena</v>
-      </c>
-      <c r="B126" t="str">
-        <v/>
-      </c>
-      <c r="C126" t="str">
-        <v/>
-      </c>
-      <c r="D126" t="str">
-        <v>Lead</v>
-      </c>
-      <c r="E126" t="str">
-        <v/>
-      </c>
-      <c r="F126" t="str">
-        <v>IR4</v>
-      </c>
-      <c r="G126" t="str">
-        <v/>
-      </c>
-      <c r="H126" t="str">
-        <v/>
-      </c>
-      <c r="I126" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="str">
-        <v>Ramya Kothuri</v>
-      </c>
-      <c r="B127" t="str">
-        <v/>
-      </c>
-      <c r="C127" t="str">
-        <v/>
-      </c>
-      <c r="D127" t="str">
-        <v>Scrum Master</v>
-      </c>
-      <c r="E127" t="str">
-        <v/>
-      </c>
-      <c r="F127" t="str">
-        <v>IR4</v>
-      </c>
-      <c r="G127" t="str">
-        <v/>
-      </c>
-      <c r="H127" t="str">
-        <v/>
-      </c>
-      <c r="I127" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="str">
-        <v>Chaitra Hanchinal</v>
-      </c>
-      <c r="B128" t="str">
-        <v/>
-      </c>
-      <c r="C128" t="str">
-        <v/>
-      </c>
-      <c r="D128" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E128" t="str">
-        <v/>
-      </c>
-      <c r="F128" t="str">
-        <v>IR4</v>
-      </c>
-      <c r="G128" t="str">
-        <v/>
-      </c>
-      <c r="H128" t="str">
-        <v/>
-      </c>
-      <c r="I128" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="str">
-        <v>Jaya Lakshmi Papolu</v>
-      </c>
-      <c r="B129" t="str">
-        <v/>
-      </c>
-      <c r="C129" t="str">
-        <v/>
-      </c>
-      <c r="D129" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E129" t="str">
-        <v/>
-      </c>
-      <c r="F129" t="str">
-        <v>IR4</v>
-      </c>
-      <c r="G129" t="str">
-        <v/>
-      </c>
-      <c r="H129" t="str">
-        <v/>
-      </c>
-      <c r="I129" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="str">
-        <v>Mrithika Kumaresan</v>
-      </c>
-      <c r="B130" t="str">
-        <v/>
-      </c>
-      <c r="C130" t="str">
-        <v/>
-      </c>
-      <c r="D130" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E130" t="str">
-        <v/>
-      </c>
-      <c r="F130" t="str">
-        <v>IR4</v>
-      </c>
-      <c r="G130" t="str">
-        <v/>
-      </c>
-      <c r="H130" t="str">
-        <v/>
-      </c>
-      <c r="I130" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="str">
-        <v>David Sotolongo</v>
-      </c>
-      <c r="B131" t="str">
-        <v/>
-      </c>
-      <c r="C131" t="str">
-        <v/>
-      </c>
-      <c r="D131" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E131" t="str">
-        <v/>
-      </c>
-      <c r="F131" t="str">
-        <v>IR4</v>
-      </c>
-      <c r="G131" t="str">
-        <v/>
-      </c>
-      <c r="H131" t="str">
-        <v/>
-      </c>
-      <c r="I131" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="str">
-        <v>Vamsi Papulo</v>
-      </c>
-      <c r="B132" t="str">
-        <v/>
-      </c>
-      <c r="C132" t="str">
-        <v/>
-      </c>
-      <c r="D132" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E132" t="str">
-        <v/>
-      </c>
-      <c r="F132" t="str">
-        <v>IR4</v>
-      </c>
-      <c r="G132" t="str">
-        <v/>
-      </c>
-      <c r="H132" t="str">
-        <v/>
-      </c>
-      <c r="I132" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="str">
-        <v>Tejaswini Pathade</v>
-      </c>
-      <c r="B133" t="str">
-        <v/>
-      </c>
-      <c r="C133" t="str">
-        <v/>
-      </c>
-      <c r="D133" t="str">
-        <v>Lead</v>
-      </c>
-      <c r="E133" t="str">
-        <v/>
-      </c>
-      <c r="F133" t="str">
-        <v>IR4</v>
-      </c>
-      <c r="G133" t="str">
-        <v/>
-      </c>
-      <c r="H133" t="str">
-        <v/>
-      </c>
-      <c r="I133" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="str">
-        <v>Andhy Gomez</v>
-      </c>
-      <c r="B134" t="str">
-        <v/>
-      </c>
-      <c r="C134" t="str">
-        <v/>
-      </c>
-      <c r="D134" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E134" t="str">
-        <v/>
-      </c>
-      <c r="F134" t="str">
-        <v>IR4</v>
-      </c>
-      <c r="G134" t="str">
-        <v/>
-      </c>
-      <c r="H134" t="str">
-        <v/>
-      </c>
-      <c r="I134" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="str">
-        <v>Kelvin Mobley</v>
-      </c>
-      <c r="B135" t="str">
-        <v/>
-      </c>
-      <c r="C135" t="str">
-        <v/>
-      </c>
-      <c r="D135" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E135" t="str">
-        <v/>
-      </c>
-      <c r="F135" t="str">
-        <v>IR4</v>
-      </c>
-      <c r="G135" t="str">
-        <v/>
-      </c>
-      <c r="H135" t="str">
-        <v/>
-      </c>
-      <c r="I135" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="str">
-        <v>Bharath Reddy Baddam</v>
-      </c>
-      <c r="B136" t="str">
-        <v/>
-      </c>
-      <c r="C136" t="str">
-        <v/>
-      </c>
-      <c r="D136" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E136" t="str">
-        <v/>
-      </c>
-      <c r="F136" t="str">
-        <v>IR4</v>
-      </c>
-      <c r="G136" t="str">
-        <v/>
-      </c>
-      <c r="H136" t="str">
-        <v/>
-      </c>
-      <c r="I136" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="str">
-        <v>Shweta Tiwari</v>
-      </c>
-      <c r="B137" t="str">
-        <v/>
-      </c>
-      <c r="C137" t="str">
-        <v/>
-      </c>
-      <c r="D137" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E137" t="str">
-        <v/>
-      </c>
-      <c r="F137" t="str">
-        <v>IR4</v>
-      </c>
-      <c r="G137" t="str">
-        <v/>
-      </c>
-      <c r="H137" t="str">
-        <v/>
-      </c>
-      <c r="I137" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="str">
-        <v>Rodolfo Duarte</v>
-      </c>
-      <c r="B138" t="str">
-        <v/>
-      </c>
-      <c r="C138" t="str">
-        <v/>
-      </c>
-      <c r="D138" t="str">
-        <v>Team</v>
-      </c>
-      <c r="E138" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="F138" t="str">
-        <v>All</v>
-      </c>
-      <c r="G138" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="H138" t="str">
-        <v/>
-      </c>
-      <c r="I138" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="str">
-        <v>Ziyad Auti</v>
-      </c>
-      <c r="B139" t="str">
-        <v/>
-      </c>
-      <c r="C139" t="str">
-        <v/>
-      </c>
-      <c r="D139" t="str">
-        <v>Intern</v>
-      </c>
-      <c r="E139" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="F139" t="str">
-        <v>All</v>
-      </c>
-      <c r="G139" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="H139" t="str">
-        <v/>
-      </c>
-      <c r="I139" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="str">
-        <v>Kishor S</v>
-      </c>
-      <c r="B140" t="str">
-        <v/>
-      </c>
-      <c r="C140" t="str">
-        <v/>
-      </c>
-      <c r="D140" t="str">
-        <v>Intern</v>
-      </c>
-      <c r="E140" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="F140" t="str">
-        <v>All</v>
-      </c>
-      <c r="G140" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="H140" t="str">
-        <v/>
-      </c>
-      <c r="I140" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="str">
-        <v>Krithika Harishchandra Shettigar</v>
-      </c>
-      <c r="B141" t="str">
-        <v/>
-      </c>
-      <c r="C141" t="str">
-        <v/>
-      </c>
-      <c r="D141" t="str">
-        <v>Intern</v>
-      </c>
-      <c r="E141" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="F141" t="str">
-        <v>All</v>
-      </c>
-      <c r="G141" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="H141" t="str">
-        <v/>
-      </c>
-      <c r="I141" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="str">
-        <v>Potumanchi Sree Yashana</v>
-      </c>
-      <c r="B142" t="str">
-        <v/>
-      </c>
-      <c r="C142" t="str">
-        <v/>
-      </c>
-      <c r="D142" t="str">
-        <v>Intern</v>
-      </c>
-      <c r="E142" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="F142" t="str">
-        <v>All</v>
-      </c>
-      <c r="G142" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="H142" t="str">
-        <v/>
-      </c>
-      <c r="I142" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="str">
-        <v>Adithya Sankar S</v>
-      </c>
-      <c r="B143" t="str">
-        <v/>
-      </c>
-      <c r="C143" t="str">
-        <v/>
-      </c>
-      <c r="D143" t="str">
-        <v>Intern</v>
-      </c>
-      <c r="E143" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="F143" t="str">
-        <v>All</v>
-      </c>
-      <c r="G143" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="H143" t="str">
-        <v/>
-      </c>
-      <c r="I143" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I143"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I125"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Restored v223: feat: add script to update Detailed Team View Excel from team data
</commit_message>
<xml_diff>
--- a/public/Detailed Team View.xlsx
+++ b/public/Detailed Team View.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I153"/>
+  <dimension ref="A1:I125"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="30.83203125" customWidth="1"/>
@@ -441,13 +441,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Aaditi Madhavan</v>
+        <v>Andhy Gomez</v>
       </c>
       <c r="B2" t="str">
-        <v>aaditi.madhavan@pwc.com</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D2" t="str">
         <v>Dev</v>
@@ -459,47 +459,47 @@
         <v>IR4</v>
       </c>
       <c r="G2" t="str">
-        <v>Energy Management</v>
+        <v>Release</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>FPL Case Management POD</v>
       </c>
       <c r="I2" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Aakanksha</v>
+        <v>Bharath Reddy Baddam</v>
       </c>
       <c r="B3" t="str">
         <v/>
       </c>
       <c r="C3" t="str">
-        <v>Infosys</v>
+        <v/>
       </c>
       <c r="D3" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E3" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="F3" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="G3" t="str">
-        <v>Outage</v>
+        <v>Release</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>FPL Case Management POD</v>
       </c>
       <c r="I3" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Adithya Sankar S</v>
+        <v>Bryan Camacho</v>
       </c>
       <c r="B4" t="str">
         <v/>
@@ -508,56 +508,56 @@
         <v/>
       </c>
       <c r="D4" t="str">
-        <v>Intern</v>
+        <v>Dev</v>
       </c>
       <c r="E4" t="str">
-        <v/>
+        <v>Hypercare</v>
       </c>
       <c r="F4" t="str">
-        <v/>
+        <v>IR3.2-Hypercare</v>
       </c>
       <c r="G4" t="str">
-        <v/>
+        <v>Hypercare</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>IR3.2 Hypercare Support</v>
       </c>
       <c r="I4" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Aditya Talwar</v>
+        <v>David Sotolongo</v>
       </c>
       <c r="B5" t="str">
-        <v>aditya.talwar@pwc.com</v>
+        <v/>
       </c>
       <c r="C5" t="str">
-        <v>Manager</v>
+        <v/>
       </c>
       <c r="D5" t="str">
-        <v>Dev Lead</v>
+        <v>Dev</v>
       </c>
       <c r="E5" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F5" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G5" t="str">
-        <v>Account Maintenance | Customer ID &amp; Fraud</v>
+        <v>Release</v>
       </c>
       <c r="H5" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I5" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Akhil Palakeel</v>
+        <v>John Harrison</v>
       </c>
       <c r="B6" t="str">
         <v/>
@@ -566,33 +566,33 @@
         <v/>
       </c>
       <c r="D6" t="str">
-        <v>Offshore Solution Analyst</v>
+        <v>Dev</v>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>Hypercare</v>
       </c>
       <c r="F6" t="str">
-        <v/>
+        <v>IR3.2-Hypercare</v>
       </c>
       <c r="G6" t="str">
-        <v/>
+        <v>Hypercare</v>
       </c>
       <c r="H6" t="str">
-        <v/>
+        <v>IR3.2 Hypercare Support</v>
       </c>
       <c r="I6" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Amarjeet Singh</v>
+        <v>Kelvin Mobley</v>
       </c>
       <c r="B7" t="str">
-        <v>amarjeet.singh@pwc.com</v>
+        <v/>
       </c>
       <c r="C7" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D7" t="str">
         <v>Dev</v>
@@ -604,18 +604,18 @@
         <v>IR4</v>
       </c>
       <c r="G7" t="str">
-        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
+        <v>Release</v>
       </c>
       <c r="H7" t="str">
-        <v/>
+        <v>FPL Case Management POD</v>
       </c>
       <c r="I7" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Andhy Gomez</v>
+        <v>Maria Vidal Parra</v>
       </c>
       <c r="B8" t="str">
         <v/>
@@ -624,36 +624,36 @@
         <v/>
       </c>
       <c r="D8" t="str">
-        <v>Dev</v>
+        <v>Scrum Master</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F8" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="G8" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H8" t="str">
-        <v/>
+        <v>FPL Dev POD</v>
       </c>
       <c r="I8" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Ankit Mishra</v>
+        <v>Ramya Kothuri</v>
       </c>
       <c r="B9" t="str">
-        <v>ankit.b.mishra@pwc.com</v>
+        <v/>
       </c>
       <c r="C9" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D9" t="str">
-        <v>Dev</v>
+        <v>Scrum Master</v>
       </c>
       <c r="E9" t="str">
         <v>IR4</v>
@@ -662,18 +662,18 @@
         <v>IR4</v>
       </c>
       <c r="G9" t="str">
-        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
+        <v>Release</v>
       </c>
       <c r="H9" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I9" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Ankit Verma</v>
+        <v>Santhosh Maduri</v>
       </c>
       <c r="B10" t="str">
         <v/>
@@ -685,62 +685,62 @@
         <v>Dev</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>Hypercare</v>
       </c>
       <c r="F10" t="str">
-        <v/>
+        <v>IR3.2-Hypercare</v>
       </c>
       <c r="G10" t="str">
-        <v/>
+        <v>Hypercare</v>
       </c>
       <c r="H10" t="str">
-        <v/>
+        <v>IR3.2 Hypercare Support</v>
       </c>
       <c r="I10" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Anto Germans</v>
+        <v>Shweta Tiwari</v>
       </c>
       <c r="B11" t="str">
-        <v>anto.a.germans@pwc.com</v>
+        <v/>
       </c>
       <c r="C11" t="str">
-        <v>Director</v>
+        <v/>
       </c>
       <c r="D11" t="str">
-        <v>Engagement Lead</v>
+        <v>Dev</v>
       </c>
       <c r="E11" t="str">
-        <v>Leadership</v>
+        <v>IR4</v>
       </c>
       <c r="F11" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G11" t="str">
-        <v>Program Leadership</v>
+        <v>Release</v>
       </c>
       <c r="H11" t="str">
-        <v/>
+        <v>FPL Case Management POD</v>
       </c>
       <c r="I11" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Anurag Jakkal</v>
+        <v>Tameka Robinson</v>
       </c>
       <c r="B12" t="str">
-        <v>jakkal.anurag.surendra@pwc.com</v>
+        <v/>
       </c>
       <c r="C12" t="str">
-        <v>Manager</v>
+        <v/>
       </c>
       <c r="D12" t="str">
-        <v>Dev Lead</v>
+        <v>Lead</v>
       </c>
       <c r="E12" t="str">
         <v>IR4</v>
@@ -749,18 +749,18 @@
         <v>IR4</v>
       </c>
       <c r="G12" t="str">
-        <v>Energy Management</v>
+        <v>Release</v>
       </c>
       <c r="H12" t="str">
-        <v/>
+        <v>FPL Dev POD</v>
       </c>
       <c r="I12" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Argene Francisco</v>
+        <v>Tejaswini Pathade</v>
       </c>
       <c r="B13" t="str">
         <v/>
@@ -769,77 +769,77 @@
         <v/>
       </c>
       <c r="D13" t="str">
-        <v>QA</v>
+        <v>Lead</v>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F13" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="G13" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H13" t="str">
-        <v/>
+        <v>FPL Case Management POD</v>
       </c>
       <c r="I13" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Argene M. Francisco</v>
+        <v>Vamsi Papulo</v>
       </c>
       <c r="B14" t="str">
-        <v>argene.francisco@pwc.com</v>
+        <v/>
       </c>
       <c r="C14" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D14" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E14" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F14" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G14" t="str">
-        <v>Move In/Transfer</v>
+        <v>Release</v>
       </c>
       <c r="H14" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I14" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Arun Kumar Krishnareddy Obannareddy</v>
+        <v>Aaditi Madhavan</v>
       </c>
       <c r="B15" t="str">
-        <v>arun.kumar.krishnareddy.obannareddy@pwc.com</v>
+        <v>aaditi.madhavan@pwc.com</v>
       </c>
       <c r="C15" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D15" t="str">
-        <v>Integration Lead</v>
+        <v>Dev</v>
       </c>
       <c r="E15" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F15" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G15" t="str">
-        <v>Integration</v>
+        <v>Energy Management</v>
       </c>
       <c r="H15" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I15" t="str">
         <v>No</v>
@@ -847,28 +847,28 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Ashit Prashant Golwala</v>
+        <v>Aakanksha</v>
       </c>
       <c r="B16" t="str">
-        <v>ashit.prashant.golwala@pwc.com</v>
+        <v/>
       </c>
       <c r="C16" t="str">
-        <v>Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D16" t="str">
         <v>QA</v>
       </c>
       <c r="E16" t="str">
-        <v>IR4</v>
+        <v>IR3.X</v>
       </c>
       <c r="F16" t="str">
-        <v>IR4</v>
+        <v>IR3.X</v>
       </c>
       <c r="G16" t="str">
-        <v>Energy Management</v>
+        <v>Outage</v>
       </c>
       <c r="H16" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I16" t="str">
         <v>No</v>
@@ -876,16 +876,16 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>B Rajkumar</v>
+        <v>Adithya Sankar S</v>
       </c>
       <c r="B17" t="str">
         <v/>
       </c>
       <c r="C17" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D17" t="str">
-        <v>DevOps</v>
+        <v>Intern</v>
       </c>
       <c r="E17" t="str">
         <v>Cross-Functional</v>
@@ -894,10 +894,10 @@
         <v>All</v>
       </c>
       <c r="G17" t="str">
-        <v>DevOps</v>
+        <v>Interns</v>
       </c>
       <c r="H17" t="str">
-        <v/>
+        <v>Interns</v>
       </c>
       <c r="I17" t="str">
         <v>No</v>
@@ -905,28 +905,28 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Bharath Reddy Baddam</v>
+        <v>Aditya Talwar</v>
       </c>
       <c r="B18" t="str">
-        <v/>
+        <v>aditya.talwar@pwc.com</v>
       </c>
       <c r="C18" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D18" t="str">
-        <v>Dev</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E18" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F18" t="str">
-        <v/>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G18" t="str">
-        <v/>
+        <v>Account Maintenance | Customer ID &amp; Fraud</v>
       </c>
       <c r="H18" t="str">
-        <v/>
+        <v>Dev POD 6/Aditya</v>
       </c>
       <c r="I18" t="str">
         <v>No</v>
@@ -934,28 +934,28 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Bhyravabhotla Naga Lakshmi Sirisha</v>
+        <v>Akhil Palakeel</v>
       </c>
       <c r="B19" t="str">
-        <v>bhyravabhotla.naga.lakshmi.sirisha@pwc.com</v>
+        <v/>
       </c>
       <c r="C19" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D19" t="str">
-        <v>QA</v>
+        <v>Offshore Solution Analyst</v>
       </c>
       <c r="E19" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F19" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G19" t="str">
-        <v>Move In/Move Out</v>
+        <v>Release</v>
       </c>
       <c r="H19" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I19" t="str">
         <v>No</v>
@@ -963,25 +963,25 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Bryan Camacho</v>
+        <v>Amarjeet Singh</v>
       </c>
       <c r="B20" t="str">
-        <v/>
+        <v>amarjeet.singh@pwc.com</v>
       </c>
       <c r="C20" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D20" t="str">
         <v>Dev</v>
       </c>
       <c r="E20" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F20" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="G20" t="str">
-        <v/>
+        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
       <c r="H20" t="str">
         <v/>
@@ -992,25 +992,25 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Chaitra Hanchinal</v>
+        <v>Ankit Mishra</v>
       </c>
       <c r="B21" t="str">
-        <v/>
+        <v>ankit.b.mishra@pwc.com</v>
       </c>
       <c r="C21" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D21" t="str">
         <v>Dev</v>
       </c>
       <c r="E21" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F21" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="G21" t="str">
-        <v/>
+        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
       <c r="H21" t="str">
         <v/>
@@ -1021,7 +1021,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Charlie Martinez</v>
+        <v>Ankit Verma</v>
       </c>
       <c r="B22" t="str">
         <v/>
@@ -1030,19 +1030,19 @@
         <v/>
       </c>
       <c r="D22" t="str">
-        <v>Lead</v>
+        <v>Dev</v>
       </c>
       <c r="E22" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F22" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="G22" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H22" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I22" t="str">
         <v>No</v>
@@ -1050,25 +1050,25 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Cheruku Pranay Reddy</v>
+        <v>Anto Germans</v>
       </c>
       <c r="B23" t="str">
-        <v>cheruku.pranay.reddy@pwc.com</v>
+        <v>anto.a.germans@pwc.com</v>
       </c>
       <c r="C23" t="str">
-        <v>Senior Associate</v>
+        <v>Director</v>
       </c>
       <c r="D23" t="str">
-        <v>Dev</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E23" t="str">
-        <v>IR4</v>
+        <v>Leadership</v>
       </c>
       <c r="F23" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G23" t="str">
-        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
+        <v>Program Leadership</v>
       </c>
       <c r="H23" t="str">
         <v/>
@@ -1079,28 +1079,28 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Cicily Deng</v>
+        <v>Anurag Jakkal</v>
       </c>
       <c r="B24" t="str">
-        <v>cicily.deng@pwc.com</v>
+        <v>jakkal.anurag.surendra@pwc.com</v>
       </c>
       <c r="C24" t="str">
-        <v>Senior Associate</v>
+        <v>Manager</v>
       </c>
       <c r="D24" t="str">
-        <v>Onshore SA</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E24" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F24" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G24" t="str">
-        <v>Case Management</v>
+        <v>Energy Management</v>
       </c>
       <c r="H24" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I24" t="str">
         <v>No</v>
@@ -1108,25 +1108,25 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Courtney Hawkins</v>
+        <v>Argene M. Francisco</v>
       </c>
       <c r="B25" t="str">
-        <v>courtney.c.hawkins@pwc.com</v>
+        <v>argene.francisco@pwc.com</v>
       </c>
       <c r="C25" t="str">
         <v>Senior Associate</v>
       </c>
       <c r="D25" t="str">
-        <v>PMO</v>
+        <v>QA</v>
       </c>
       <c r="E25" t="str">
-        <v>Leadership</v>
+        <v>IR3.2</v>
       </c>
       <c r="F25" t="str">
         <v>All</v>
       </c>
       <c r="G25" t="str">
-        <v>PMO</v>
+        <v>Move In/Transfer</v>
       </c>
       <c r="H25" t="str">
         <v/>
@@ -1137,25 +1137,25 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>David Sotolongo</v>
+        <v>Arun Kumar Krishnareddy Obannareddy</v>
       </c>
       <c r="B26" t="str">
-        <v/>
+        <v>arun.kumar.krishnareddy.obannareddy@pwc.com</v>
       </c>
       <c r="C26" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D26" t="str">
-        <v>Dev</v>
+        <v>Integration Lead</v>
       </c>
       <c r="E26" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F26" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G26" t="str">
-        <v/>
+        <v>Integration</v>
       </c>
       <c r="H26" t="str">
         <v/>
@@ -1166,28 +1166,28 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Deneys Van Der Merwe</v>
+        <v>Ashit Prashant Golwala</v>
       </c>
       <c r="B27" t="str">
-        <v>deneys.van.der.merwe@pwc.com</v>
+        <v>ashit.prashant.golwala@pwc.com</v>
       </c>
       <c r="C27" t="str">
         <v>Associate</v>
       </c>
       <c r="D27" t="str">
-        <v>Onshore SA</v>
+        <v>QA</v>
       </c>
       <c r="E27" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F27" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G27" t="str">
-        <v>Case Management</v>
+        <v>Energy Management</v>
       </c>
       <c r="H27" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I27" t="str">
         <v>No</v>
@@ -1195,25 +1195,25 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Diksha</v>
+        <v>B Rajkumar</v>
       </c>
       <c r="B28" t="str">
         <v/>
       </c>
       <c r="C28" t="str">
-        <v>Infosys</v>
+        <v>Associate</v>
       </c>
       <c r="D28" t="str">
-        <v>QA</v>
+        <v>DevOps</v>
       </c>
       <c r="E28" t="str">
-        <v>IR3.X</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F28" t="str">
-        <v>IR3.X</v>
+        <v>All</v>
       </c>
       <c r="G28" t="str">
-        <v>Outage</v>
+        <v>DevOps</v>
       </c>
       <c r="H28" t="str">
         <v/>
@@ -1224,25 +1224,25 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Dnyanesh Prakash Painjan</v>
+        <v>Bhyravabhotla Naga Lakshmi Sirisha</v>
       </c>
       <c r="B29" t="str">
-        <v/>
+        <v>bhyravabhotla.naga.lakshmi.sirisha@pwc.com</v>
       </c>
       <c r="C29" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D29" t="str">
         <v>QA</v>
       </c>
       <c r="E29" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F29" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G29" t="str">
-        <v/>
+        <v>Move In/Move Out</v>
       </c>
       <c r="H29" t="str">
         <v/>
@@ -1253,28 +1253,28 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Dnyanesh Prakash Painjane</v>
+        <v>Chaitra Hanchinal</v>
       </c>
       <c r="B30" t="str">
-        <v>dnyanesh.prakash.painjane@pwc.com</v>
+        <v/>
       </c>
       <c r="C30" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D30" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E30" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F30" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G30" t="str">
-        <v>Move In/Transfer</v>
+        <v>Release</v>
       </c>
       <c r="H30" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I30" t="str">
         <v>No</v>
@@ -1282,25 +1282,25 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Gianna Caruso</v>
+        <v>Cheruku Pranay Reddy</v>
       </c>
       <c r="B31" t="str">
-        <v>gianna.caruso@pwc.com</v>
+        <v>cheruku.pranay.reddy@pwc.com</v>
       </c>
       <c r="C31" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D31" t="str">
-        <v>Onshore SA</v>
+        <v>Dev</v>
       </c>
       <c r="E31" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F31" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G31" t="str">
-        <v>Move In/Move Out/Transfer | Multi Move In/Transfer/Amend</v>
+        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
       <c r="H31" t="str">
         <v/>
@@ -1311,28 +1311,28 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Girlee Alvarado</v>
+        <v>Cicily Deng</v>
       </c>
       <c r="B32" t="str">
-        <v/>
+        <v>cicily.deng@pwc.com</v>
       </c>
       <c r="C32" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D32" t="str">
-        <v>QA</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E32" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F32" t="str">
-        <v/>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G32" t="str">
-        <v/>
+        <v>Case Management</v>
       </c>
       <c r="H32" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I32" t="str">
         <v>No</v>
@@ -1340,25 +1340,25 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Girlee P. Alvarado</v>
+        <v>Courtney Hawkins</v>
       </c>
       <c r="B33" t="str">
-        <v>girlee.alvarado@pwc.com</v>
+        <v>courtney.c.hawkins@pwc.com</v>
       </c>
       <c r="C33" t="str">
         <v>Senior Associate</v>
       </c>
       <c r="D33" t="str">
-        <v>QA</v>
+        <v>PMO</v>
       </c>
       <c r="E33" t="str">
-        <v>IR3.2</v>
+        <v>Leadership</v>
       </c>
       <c r="F33" t="str">
         <v>All</v>
       </c>
       <c r="G33" t="str">
-        <v>Move Out/Transfer</v>
+        <v>PMO</v>
       </c>
       <c r="H33" t="str">
         <v/>
@@ -1369,28 +1369,28 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Grace Nazareno</v>
+        <v>Deneys Van Der Merwe</v>
       </c>
       <c r="B34" t="str">
-        <v/>
+        <v>deneys.van.der.merwe@pwc.com</v>
       </c>
       <c r="C34" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D34" t="str">
-        <v>QA</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E34" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F34" t="str">
-        <v/>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G34" t="str">
-        <v/>
+        <v>Case Management</v>
       </c>
       <c r="H34" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I34" t="str">
         <v>No</v>
@@ -1398,28 +1398,28 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Harish Govindareddy</v>
+        <v>Diksha</v>
       </c>
       <c r="B35" t="str">
-        <v>harish.govindareddy@pwc.com</v>
+        <v/>
       </c>
       <c r="C35" t="str">
-        <v>Senior Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D35" t="str">
-        <v>Windsurf/Performance Dev</v>
+        <v>QA</v>
       </c>
       <c r="E35" t="str">
-        <v>Cross-Functional</v>
+        <v>IR3.X</v>
       </c>
       <c r="F35" t="str">
-        <v>All</v>
+        <v>IR3.X</v>
       </c>
       <c r="G35" t="str">
-        <v>Windsurf/Performance</v>
+        <v>Outage</v>
       </c>
       <c r="H35" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I35" t="str">
         <v>No</v>
@@ -1427,25 +1427,25 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Harsh Shah</v>
+        <v>Dnyanesh Prakash Painjane</v>
       </c>
       <c r="B36" t="str">
-        <v/>
+        <v>dnyanesh.prakash.painjane@pwc.com</v>
       </c>
       <c r="C36" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D36" t="str">
-        <v>Onshore Solution Analyst</v>
+        <v>QA</v>
       </c>
       <c r="E36" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F36" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G36" t="str">
-        <v/>
+        <v>Move In/Transfer</v>
       </c>
       <c r="H36" t="str">
         <v/>
@@ -1456,28 +1456,28 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Hemant Jain</v>
+        <v>Gianna Caruso</v>
       </c>
       <c r="B37" t="str">
-        <v>hemant.jain@pwc.com</v>
+        <v>gianna.caruso@pwc.com</v>
       </c>
       <c r="C37" t="str">
-        <v>Senior Manager</v>
+        <v>Associate</v>
       </c>
       <c r="D37" t="str">
-        <v>Technical Architect</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E37" t="str">
-        <v>Leadership</v>
+        <v>IR3.2</v>
       </c>
       <c r="F37" t="str">
-        <v>All</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G37" t="str">
-        <v>Architecture</v>
+        <v>Move In/Move Out/Transfer | Multi Move In/Transfer/Amend</v>
       </c>
       <c r="H37" t="str">
-        <v/>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I37" t="str">
         <v>No</v>
@@ -1485,25 +1485,25 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ISH Jacinto</v>
+        <v>Girlee P. Alvarado</v>
       </c>
       <c r="B38" t="str">
-        <v/>
+        <v>girlee.alvarado@pwc.com</v>
       </c>
       <c r="C38" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D38" t="str">
         <v>QA</v>
       </c>
       <c r="E38" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F38" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G38" t="str">
-        <v/>
+        <v>Move Out/Transfer</v>
       </c>
       <c r="H38" t="str">
         <v/>
@@ -1514,25 +1514,25 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Israel L. Jacinto</v>
+        <v>Harish Govindareddy</v>
       </c>
       <c r="B39" t="str">
-        <v>israel.jacinto@pwc.com</v>
+        <v>harish.govindareddy@pwc.com</v>
       </c>
       <c r="C39" t="str">
         <v>Senior Associate</v>
       </c>
       <c r="D39" t="str">
-        <v>QA</v>
+        <v>Windsurf/Performance Dev</v>
       </c>
       <c r="E39" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F39" t="str">
         <v>All</v>
       </c>
       <c r="G39" t="str">
-        <v>Move Out</v>
+        <v>Windsurf/Performance</v>
       </c>
       <c r="H39" t="str">
         <v/>
@@ -1543,25 +1543,25 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Jake Garrell</v>
+        <v>Hemant Jain</v>
       </c>
       <c r="B40" t="str">
-        <v/>
+        <v>hemant.jain@pwc.com</v>
       </c>
       <c r="C40" t="str">
-        <v/>
+        <v>Senior Manager</v>
       </c>
       <c r="D40" t="str">
-        <v>Dev</v>
+        <v>Technical Architect</v>
       </c>
       <c r="E40" t="str">
-        <v/>
+        <v>Leadership</v>
       </c>
       <c r="F40" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G40" t="str">
-        <v/>
+        <v>Architecture</v>
       </c>
       <c r="H40" t="str">
         <v/>
@@ -1572,25 +1572,25 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Jason Pereira</v>
+        <v>Israel L. Jacinto</v>
       </c>
       <c r="B41" t="str">
-        <v/>
+        <v>israel.jacinto@pwc.com</v>
       </c>
       <c r="C41" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D41" t="str">
-        <v>Lead</v>
+        <v>QA</v>
       </c>
       <c r="E41" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F41" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G41" t="str">
-        <v/>
+        <v>Move Out</v>
       </c>
       <c r="H41" t="str">
         <v/>
@@ -1601,7 +1601,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Jaya Lakshmi Papolu</v>
+        <v>Jason Pereira</v>
       </c>
       <c r="B42" t="str">
         <v/>
@@ -1610,19 +1610,19 @@
         <v/>
       </c>
       <c r="D42" t="str">
-        <v>Dev</v>
+        <v>Lead</v>
       </c>
       <c r="E42" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F42" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="G42" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H42" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I42" t="str">
         <v>No</v>
@@ -1630,28 +1630,28 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Jayoti Chatterji</v>
+        <v>Jaya Lakshmi Papolu</v>
       </c>
       <c r="B43" t="str">
-        <v>jayoti.chatterji@pwc.com</v>
+        <v/>
       </c>
       <c r="C43" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D43" t="str">
         <v>Dev</v>
       </c>
       <c r="E43" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="F43" t="str">
-        <v>IR3.X</v>
+        <v>IR4</v>
       </c>
       <c r="G43" t="str">
-        <v>Outage</v>
+        <v>Release</v>
       </c>
       <c r="H43" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I43" t="str">
         <v>No</v>
@@ -1659,28 +1659,28 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Jitain Mohun</v>
+        <v>Jayoti Chatterji</v>
       </c>
       <c r="B44" t="str">
-        <v/>
+        <v>jayoti.chatterji@pwc.com</v>
       </c>
       <c r="C44" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D44" t="str">
-        <v>Onshore SA</v>
+        <v>Dev</v>
       </c>
       <c r="E44" t="str">
         <v>IR3.X</v>
       </c>
       <c r="F44" t="str">
-        <v>IR3.X/IR4</v>
+        <v>IR3.X</v>
       </c>
       <c r="G44" t="str">
         <v>Outage</v>
       </c>
       <c r="H44" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I44" t="str">
         <v>No</v>
@@ -1688,28 +1688,28 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>John Harrison</v>
+        <v>Jitain Mohun</v>
       </c>
       <c r="B45" t="str">
         <v/>
       </c>
       <c r="C45" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D45" t="str">
-        <v>Dev</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E45" t="str">
-        <v/>
+        <v>IR3.X</v>
       </c>
       <c r="F45" t="str">
-        <v/>
+        <v>IR3.X/IR4</v>
       </c>
       <c r="G45" t="str">
-        <v/>
+        <v>Outage</v>
       </c>
       <c r="H45" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I45" t="str">
         <v>No</v>
@@ -1729,16 +1729,16 @@
         <v>Dev</v>
       </c>
       <c r="E46" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F46" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="G46" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H46" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I46" t="str">
         <v>No</v>
@@ -1746,7 +1746,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Kankshitha Yalamuru</v>
+        <v>Kavita Jha</v>
       </c>
       <c r="B47" t="str">
         <v/>
@@ -1758,16 +1758,16 @@
         <v>Dev</v>
       </c>
       <c r="E47" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F47" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="G47" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H47" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I47" t="str">
         <v>No</v>
@@ -1775,25 +1775,25 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Kavita Jha</v>
+        <v>Keerthana Manjunath</v>
       </c>
       <c r="B48" t="str">
         <v/>
       </c>
       <c r="C48" t="str">
-        <v/>
+        <v>Infosys</v>
       </c>
       <c r="D48" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E48" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F48" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G48" t="str">
-        <v/>
+        <v>Transfer</v>
       </c>
       <c r="H48" t="str">
         <v/>
@@ -1804,28 +1804,28 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Keerthana Manjunath</v>
+        <v>Kishor S</v>
       </c>
       <c r="B49" t="str">
         <v/>
       </c>
       <c r="C49" t="str">
-        <v>Infosys</v>
+        <v/>
       </c>
       <c r="D49" t="str">
-        <v>QA</v>
+        <v>Intern</v>
       </c>
       <c r="E49" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F49" t="str">
         <v>All</v>
       </c>
       <c r="G49" t="str">
-        <v>Transfer</v>
+        <v>Interns</v>
       </c>
       <c r="H49" t="str">
-        <v/>
+        <v>Interns</v>
       </c>
       <c r="I49" t="str">
         <v>No</v>
@@ -1833,25 +1833,25 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Kelvin Mobley</v>
+        <v>Kodi Elangovan</v>
       </c>
       <c r="B50" t="str">
-        <v/>
+        <v>kodiyarasan.elangovan@pwc.com</v>
       </c>
       <c r="C50" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D50" t="str">
-        <v>Dev</v>
+        <v>Integration Lead</v>
       </c>
       <c r="E50" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F50" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G50" t="str">
-        <v/>
+        <v>Integration</v>
       </c>
       <c r="H50" t="str">
         <v/>
@@ -1862,7 +1862,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Kishor S</v>
+        <v>Krithika Harishchandra Shettigar</v>
       </c>
       <c r="B51" t="str">
         <v/>
@@ -1874,16 +1874,16 @@
         <v>Intern</v>
       </c>
       <c r="E51" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F51" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G51" t="str">
-        <v/>
+        <v>Interns</v>
       </c>
       <c r="H51" t="str">
-        <v/>
+        <v>Interns</v>
       </c>
       <c r="I51" t="str">
         <v>No</v>
@@ -1891,28 +1891,28 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Kodi Elangovan</v>
+        <v>Lokesh Sai</v>
       </c>
       <c r="B52" t="str">
-        <v>kodiyarasan.elangovan@pwc.com</v>
+        <v>lokesh.sai@pwc.com</v>
       </c>
       <c r="C52" t="str">
-        <v>Manager</v>
+        <v>Associate</v>
       </c>
       <c r="D52" t="str">
-        <v>Integration Lead</v>
+        <v>QA</v>
       </c>
       <c r="E52" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F52" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G52" t="str">
-        <v>Integration</v>
+        <v>Energy Management</v>
       </c>
       <c r="H52" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I52" t="str">
         <v>No</v>
@@ -1920,28 +1920,28 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Krithika Harishchandra Shettigar</v>
+        <v>Madhumita Kodidela</v>
       </c>
       <c r="B53" t="str">
-        <v/>
+        <v>madhumitha.kodidela@pwc.com</v>
       </c>
       <c r="C53" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D53" t="str">
-        <v>Intern</v>
+        <v>Dev</v>
       </c>
       <c r="E53" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F53" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="G53" t="str">
-        <v/>
+        <v>Interactions/Search</v>
       </c>
       <c r="H53" t="str">
-        <v/>
+        <v>Dev POD 2/Sneha G</v>
       </c>
       <c r="I53" t="str">
         <v>No</v>
@@ -1949,25 +1949,25 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Lisa Pell</v>
+        <v>Maneesha</v>
       </c>
       <c r="B54" t="str">
         <v/>
       </c>
       <c r="C54" t="str">
-        <v/>
+        <v>Infosys</v>
       </c>
       <c r="D54" t="str">
-        <v>Architect</v>
+        <v>QA</v>
       </c>
       <c r="E54" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F54" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G54" t="str">
-        <v/>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H54" t="str">
         <v/>
@@ -1978,25 +1978,25 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Lokesh Sai</v>
+        <v>Mary Grace Carinan Nazareno</v>
       </c>
       <c r="B55" t="str">
-        <v>lokesh.sai@pwc.com</v>
+        <v>mary.grace.nazareno@pwc.com</v>
       </c>
       <c r="C55" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D55" t="str">
         <v>QA</v>
       </c>
       <c r="E55" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F55" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G55" t="str">
-        <v>Energy Management</v>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H55" t="str">
         <v/>
@@ -2007,25 +2007,25 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Madhumita Kodidela</v>
+        <v>Matthew Rupas</v>
       </c>
       <c r="B56" t="str">
-        <v>madhumitha.kodidela@pwc.com</v>
+        <v>matthew.i.rupas@pwc.com</v>
       </c>
       <c r="C56" t="str">
-        <v>Senior Associate</v>
+        <v>Partner</v>
       </c>
       <c r="D56" t="str">
-        <v>Dev</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E56" t="str">
-        <v>IR3.2</v>
+        <v>Leadership</v>
       </c>
       <c r="F56" t="str">
-        <v>IR3.2</v>
+        <v>All</v>
       </c>
       <c r="G56" t="str">
-        <v>Interactions/Search</v>
+        <v>Program Leadership</v>
       </c>
       <c r="H56" t="str">
         <v/>
@@ -2036,28 +2036,28 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Maneesha</v>
+        <v>Mayand Mani</v>
       </c>
       <c r="B57" t="str">
         <v/>
       </c>
       <c r="C57" t="str">
-        <v>Infosys</v>
+        <v>Associate</v>
       </c>
       <c r="D57" t="str">
         <v>QA</v>
       </c>
       <c r="E57" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F57" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G57" t="str">
-        <v>Move In/Move Out/Transfer</v>
+        <v>Energy Management</v>
       </c>
       <c r="H57" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I57" t="str">
         <v>No</v>
@@ -2065,28 +2065,28 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Manu Tyagi</v>
+        <v>Mayur Kinhekar</v>
       </c>
       <c r="B58" t="str">
-        <v/>
+        <v>mayur.murlidhar.kinhekar@pwc.com</v>
       </c>
       <c r="C58" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D58" t="str">
-        <v>Dev</v>
+        <v>Offshore SA</v>
       </c>
       <c r="E58" t="str">
-        <v/>
+        <v>IR3.X</v>
       </c>
       <c r="F58" t="str">
-        <v/>
+        <v>IR3.X/IR4</v>
       </c>
       <c r="G58" t="str">
-        <v/>
+        <v>Outage</v>
       </c>
       <c r="H58" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I58" t="str">
         <v>No</v>
@@ -2094,28 +2094,28 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Maria Vidal Parra</v>
+        <v>Michael O'shea</v>
       </c>
       <c r="B59" t="str">
-        <v/>
+        <v>michael.o.oshea@pwc.com</v>
       </c>
       <c r="C59" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D59" t="str">
-        <v>Scrum Master</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E59" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F59" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="G59" t="str">
-        <v/>
+        <v>Interactions/Search</v>
       </c>
       <c r="H59" t="str">
-        <v/>
+        <v>Dev POD 2/Sneha G</v>
       </c>
       <c r="I59" t="str">
         <v>No</v>
@@ -2123,22 +2123,22 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Mary Grace Carinan Nazareno</v>
+        <v>Mounika Depuri</v>
       </c>
       <c r="B60" t="str">
-        <v>mary.grace.nazareno@pwc.com</v>
+        <v>mounika.depuri@pwc.com</v>
       </c>
       <c r="C60" t="str">
         <v>Senior Associate</v>
       </c>
       <c r="D60" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E60" t="str">
         <v>IR3.2</v>
       </c>
       <c r="F60" t="str">
-        <v>All</v>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G60" t="str">
         <v>Payment &amp; Payment Options/Billing Programs</v>
@@ -2152,28 +2152,28 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>Matthew Rupas</v>
+        <v>Mrithika Kumaresan</v>
       </c>
       <c r="B61" t="str">
-        <v>matthew.i.rupas@pwc.com</v>
+        <v/>
       </c>
       <c r="C61" t="str">
-        <v>Partner</v>
+        <v/>
       </c>
       <c r="D61" t="str">
-        <v>Engagement Lead</v>
+        <v>Dev</v>
       </c>
       <c r="E61" t="str">
-        <v>Leadership</v>
+        <v>IR4</v>
       </c>
       <c r="F61" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G61" t="str">
-        <v>Program Leadership</v>
+        <v>Release</v>
       </c>
       <c r="H61" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I61" t="str">
         <v>No</v>
@@ -2181,16 +2181,16 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>Mayand Mani</v>
+        <v>Mylavarapu V N R Saketh</v>
       </c>
       <c r="B62" t="str">
-        <v/>
+        <v>mylavarapu.v.n.r.saketh@pwc.com</v>
       </c>
       <c r="C62" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D62" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E62" t="str">
         <v>IR4</v>
@@ -2202,7 +2202,7 @@
         <v>Energy Management</v>
       </c>
       <c r="H62" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I62" t="str">
         <v>No</v>
@@ -2210,25 +2210,25 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>Mayur Kinhekar</v>
+        <v>Naga Srilekha Thummalacheruvu</v>
       </c>
       <c r="B63" t="str">
-        <v>mayur.murlidhar.kinhekar@pwc.com</v>
+        <v>naga.t.thummalacheruvu@pwc.com</v>
       </c>
       <c r="C63" t="str">
-        <v>Senior Associate</v>
+        <v>Associate</v>
       </c>
       <c r="D63" t="str">
-        <v>Offshore SA</v>
+        <v>QA</v>
       </c>
       <c r="E63" t="str">
-        <v>IR3.X</v>
+        <v>IR3.2</v>
       </c>
       <c r="F63" t="str">
-        <v>IR3.X/IR4</v>
+        <v>All</v>
       </c>
       <c r="G63" t="str">
-        <v>Outage</v>
+        <v>Move In</v>
       </c>
       <c r="H63" t="str">
         <v/>
@@ -2239,28 +2239,28 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Michael O'shea</v>
+        <v>Naman Hiran</v>
       </c>
       <c r="B64" t="str">
-        <v>michael.o.oshea@pwc.com</v>
+        <v>naman.hiran@pwc.com</v>
       </c>
       <c r="C64" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D64" t="str">
-        <v>Onshore SA</v>
+        <v>Dev</v>
       </c>
       <c r="E64" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F64" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G64" t="str">
-        <v>Interactions/Search</v>
+        <v>Energy Management</v>
       </c>
       <c r="H64" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I64" t="str">
         <v>No</v>
@@ -2268,25 +2268,25 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Mindi Sai Bhavana</v>
+        <v>Namrata Uttareshwar Bansode</v>
       </c>
       <c r="B65" t="str">
-        <v/>
+        <v>namrata.uttareshwar.bansode@pwc.com</v>
       </c>
       <c r="C65" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D65" t="str">
-        <v>QA</v>
+        <v>Offshore SA</v>
       </c>
       <c r="E65" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F65" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="G65" t="str">
-        <v/>
+        <v>Billing &amp; Usage/Payment Programs</v>
       </c>
       <c r="H65" t="str">
         <v/>
@@ -2297,28 +2297,28 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Mounika Depuri</v>
+        <v>Niket Saxena</v>
       </c>
       <c r="B66" t="str">
-        <v>mounika.depuri@pwc.com</v>
+        <v/>
       </c>
       <c r="C66" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D66" t="str">
-        <v>Dev</v>
+        <v>Lead</v>
       </c>
       <c r="E66" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F66" t="str">
-        <v>IR3.2/IR4</v>
+        <v>IR4</v>
       </c>
       <c r="G66" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v>Release</v>
       </c>
       <c r="H66" t="str">
-        <v/>
+        <v>Field Management POD</v>
       </c>
       <c r="I66" t="str">
         <v>No</v>
@@ -2326,25 +2326,25 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Mrithika Kumaresan</v>
+        <v>Nikita</v>
       </c>
       <c r="B67" t="str">
         <v/>
       </c>
       <c r="C67" t="str">
-        <v/>
+        <v>Infosys</v>
       </c>
       <c r="D67" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E67" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F67" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G67" t="str">
-        <v/>
+        <v>Payment &amp; Payment Options</v>
       </c>
       <c r="H67" t="str">
         <v/>
@@ -2355,25 +2355,25 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Mukul Sagar</v>
+        <v>Nilesh</v>
       </c>
       <c r="B68" t="str">
         <v/>
       </c>
       <c r="C68" t="str">
-        <v/>
+        <v>Infosys</v>
       </c>
       <c r="D68" t="str">
-        <v>Architect</v>
+        <v>QA</v>
       </c>
       <c r="E68" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F68" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G68" t="str">
-        <v/>
+        <v>Account Maintenance</v>
       </c>
       <c r="H68" t="str">
         <v/>
@@ -2384,28 +2384,28 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>Mylavarapu V N R Saketh</v>
+        <v>Nishi Jain</v>
       </c>
       <c r="B69" t="str">
-        <v>mylavarapu.v.n.r.saketh@pwc.com</v>
+        <v/>
       </c>
       <c r="C69" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D69" t="str">
         <v>Dev</v>
       </c>
       <c r="E69" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F69" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="G69" t="str">
-        <v>Energy Management</v>
+        <v>Release</v>
       </c>
       <c r="H69" t="str">
-        <v/>
+        <v>Dev POD 6/Aditya</v>
       </c>
       <c r="I69" t="str">
         <v>No</v>
@@ -2413,25 +2413,25 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>Naga Srilekha Thummalacheruvu</v>
+        <v>Nishi Narendra Jain</v>
       </c>
       <c r="B70" t="str">
-        <v>naga.t.thummalacheruvu@pwc.com</v>
+        <v>jain.u.nishi@pwc.com</v>
       </c>
       <c r="C70" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D70" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E70" t="str">
         <v>IR3.2</v>
       </c>
       <c r="F70" t="str">
-        <v>All</v>
+        <v>IR3.2</v>
       </c>
       <c r="G70" t="str">
-        <v>Move In</v>
+        <v>Account Maintenance</v>
       </c>
       <c r="H70" t="str">
         <v/>
@@ -2442,13 +2442,13 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>Naman Hiran</v>
+        <v>Nivetha Sudharsanam</v>
       </c>
       <c r="B71" t="str">
-        <v>naman.hiran@pwc.com</v>
+        <v/>
       </c>
       <c r="C71" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D71" t="str">
         <v>Dev</v>
@@ -2460,10 +2460,10 @@
         <v>IR4</v>
       </c>
       <c r="G71" t="str">
-        <v>Energy Management</v>
+        <v>Release</v>
       </c>
       <c r="H71" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I71" t="str">
         <v>No</v>
@@ -2471,25 +2471,25 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>Namrata Bansode</v>
+        <v>Paarth Sonwaney</v>
       </c>
       <c r="B72" t="str">
-        <v/>
+        <v>paarth.sonwaney@pwc.com</v>
       </c>
       <c r="C72" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D72" t="str">
-        <v>Offshore Solution Analyst</v>
+        <v>PMO</v>
       </c>
       <c r="E72" t="str">
-        <v/>
+        <v>Leadership</v>
       </c>
       <c r="F72" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G72" t="str">
-        <v/>
+        <v>PMO</v>
       </c>
       <c r="H72" t="str">
         <v/>
@@ -2500,13 +2500,13 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>Namrata Uttareshwar Bansode</v>
+        <v>Parul Prasad</v>
       </c>
       <c r="B73" t="str">
-        <v>namrata.uttareshwar.bansode@pwc.com</v>
+        <v>parul.prasad@pwc.com</v>
       </c>
       <c r="C73" t="str">
-        <v>Manager</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D73" t="str">
         <v>Offshore SA</v>
@@ -2518,10 +2518,10 @@
         <v>IR4</v>
       </c>
       <c r="G73" t="str">
-        <v>Billing &amp; Usage/Payment Programs</v>
+        <v>Energy Management</v>
       </c>
       <c r="H73" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I73" t="str">
         <v>No</v>
@@ -2529,28 +2529,28 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>Naveen Tayal</v>
+        <v>Piyush Singh</v>
       </c>
       <c r="B74" t="str">
-        <v/>
+        <v>piyush.ss.singh@pwc.com</v>
       </c>
       <c r="C74" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D74" t="str">
-        <v>Onshore Solution Analyst</v>
+        <v>Dev</v>
       </c>
       <c r="E74" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F74" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="G74" t="str">
-        <v/>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H74" t="str">
-        <v/>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I74" t="str">
         <v>No</v>
@@ -2558,28 +2558,28 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>Niket Saxena</v>
+        <v>Pornima Rajguru</v>
       </c>
       <c r="B75" t="str">
-        <v/>
+        <v>Poornima.atul.rajguru@pwc.com</v>
       </c>
       <c r="C75" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D75" t="str">
-        <v>Lead</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E75" t="str">
-        <v/>
+        <v>IR3.X</v>
       </c>
       <c r="F75" t="str">
-        <v/>
+        <v>IR3.X</v>
       </c>
       <c r="G75" t="str">
-        <v/>
+        <v>Outage</v>
       </c>
       <c r="H75" t="str">
-        <v/>
+        <v>Dev POD 5/Pornima</v>
       </c>
       <c r="I75" t="str">
         <v>No</v>
@@ -2587,28 +2587,28 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>Nikita</v>
+        <v>Potumanchi Sree Yashana</v>
       </c>
       <c r="B76" t="str">
         <v/>
       </c>
       <c r="C76" t="str">
-        <v>Infosys</v>
+        <v/>
       </c>
       <c r="D76" t="str">
-        <v>QA</v>
+        <v>Intern</v>
       </c>
       <c r="E76" t="str">
-        <v>IR3.2</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F76" t="str">
         <v>All</v>
       </c>
       <c r="G76" t="str">
-        <v>Payment &amp; Payment Options</v>
+        <v>Interns</v>
       </c>
       <c r="H76" t="str">
-        <v/>
+        <v>Interns</v>
       </c>
       <c r="I76" t="str">
         <v>No</v>
@@ -2616,28 +2616,28 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>Nilesh</v>
+        <v>Pradeep Lambu</v>
       </c>
       <c r="B77" t="str">
         <v/>
       </c>
       <c r="C77" t="str">
-        <v>Infosys</v>
+        <v/>
       </c>
       <c r="D77" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E77" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F77" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G77" t="str">
-        <v>Account Maintenance</v>
+        <v>Release</v>
       </c>
       <c r="H77" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I77" t="str">
         <v>No</v>
@@ -2645,25 +2645,25 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>Nishi Jain</v>
+        <v>Pranav Singh</v>
       </c>
       <c r="B78" t="str">
-        <v/>
+        <v>pranav.s.singh@pwc.com</v>
       </c>
       <c r="C78" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D78" t="str">
-        <v>Dev</v>
+        <v>Integration Dev</v>
       </c>
       <c r="E78" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F78" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G78" t="str">
-        <v/>
+        <v>Integration</v>
       </c>
       <c r="H78" t="str">
         <v/>
@@ -2674,28 +2674,28 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>Nishi Narendra Jain</v>
+        <v>Prasad P</v>
       </c>
       <c r="B79" t="str">
-        <v>jain.u.nishi@pwc.com</v>
+        <v/>
       </c>
       <c r="C79" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D79" t="str">
         <v>Dev</v>
       </c>
       <c r="E79" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F79" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G79" t="str">
-        <v>Account Maintenance</v>
+        <v>Release</v>
       </c>
       <c r="H79" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I79" t="str">
         <v>No</v>
@@ -2703,25 +2703,25 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Nivetha Sudharsanam</v>
+        <v>Prasanna Nangnure</v>
       </c>
       <c r="B80" t="str">
-        <v/>
+        <v>prasanna.y.nangnure@pwc.com</v>
       </c>
       <c r="C80" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D80" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E80" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F80" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G80" t="str">
-        <v/>
+        <v>Billing Programs</v>
       </c>
       <c r="H80" t="str">
         <v/>
@@ -2732,28 +2732,28 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Paarth Sonwaney</v>
+        <v>Pratik Kurdukar</v>
       </c>
       <c r="B81" t="str">
-        <v>paarth.sonwaney@pwc.com</v>
+        <v>pratik.k.kurdukar@pwc.com</v>
       </c>
       <c r="C81" t="str">
-        <v>Manager</v>
+        <v>Associate</v>
       </c>
       <c r="D81" t="str">
-        <v>PMO</v>
+        <v>Dev</v>
       </c>
       <c r="E81" t="str">
-        <v>Leadership</v>
+        <v>IR3.2</v>
       </c>
       <c r="F81" t="str">
-        <v>All</v>
+        <v>IR3.2</v>
       </c>
       <c r="G81" t="str">
-        <v>PMO</v>
+        <v>Case Management</v>
       </c>
       <c r="H81" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I81" t="str">
         <v>No</v>
@@ -2761,25 +2761,25 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>Parul Prasad</v>
+        <v>Pratik Mahajan</v>
       </c>
       <c r="B82" t="str">
-        <v>parul.prasad@pwc.com</v>
+        <v>pratik.sunil.mahajan@pwc.com</v>
       </c>
       <c r="C82" t="str">
         <v>Senior Associate</v>
       </c>
       <c r="D82" t="str">
-        <v>Offshore SA</v>
+        <v>QA</v>
       </c>
       <c r="E82" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F82" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G82" t="str">
-        <v>Energy Management</v>
+        <v>Interactions/Search</v>
       </c>
       <c r="H82" t="str">
         <v/>
@@ -2790,25 +2790,25 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>Piyush Singh</v>
+        <v>Pritam</v>
       </c>
       <c r="B83" t="str">
-        <v>piyush.ss.singh@pwc.com</v>
+        <v/>
       </c>
       <c r="C83" t="str">
-        <v>Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D83" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E83" t="str">
         <v>IR3.2</v>
       </c>
       <c r="F83" t="str">
-        <v>IR3.2</v>
+        <v>All</v>
       </c>
       <c r="G83" t="str">
-        <v>Move In/Move Out/Transfer</v>
+        <v>Account Maintenance</v>
       </c>
       <c r="H83" t="str">
         <v/>
@@ -2819,25 +2819,25 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>Pornima Rajguru</v>
+        <v>Rajaraman A</v>
       </c>
       <c r="B84" t="str">
-        <v>Poornima.atul.rajguru@pwc.com</v>
+        <v>rajaraman.a@pwc.com</v>
       </c>
       <c r="C84" t="str">
         <v>Manager</v>
       </c>
       <c r="D84" t="str">
-        <v>Dev Lead</v>
+        <v>QA Lead</v>
       </c>
       <c r="E84" t="str">
-        <v>IR3.X</v>
+        <v>IR3.2</v>
       </c>
       <c r="F84" t="str">
-        <v>IR3.X</v>
+        <v>All</v>
       </c>
       <c r="G84" t="str">
-        <v>Outage</v>
+        <v>QA - All Value Streams</v>
       </c>
       <c r="H84" t="str">
         <v/>
@@ -2848,25 +2848,25 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>Potumanchi Sree Yashana</v>
+        <v>Raveendra Reddy</v>
       </c>
       <c r="B85" t="str">
-        <v/>
+        <v>raveendra.t.reddy@pwc.com</v>
       </c>
       <c r="C85" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D85" t="str">
-        <v>Intern</v>
+        <v>QA</v>
       </c>
       <c r="E85" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F85" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G85" t="str">
-        <v/>
+        <v>Transfer</v>
       </c>
       <c r="H85" t="str">
         <v/>
@@ -2877,25 +2877,25 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>Pradeep Lambu</v>
+        <v>Rhitik Khanna</v>
       </c>
       <c r="B86" t="str">
-        <v/>
+        <v>rhitik.khanna@pwc.com</v>
       </c>
       <c r="C86" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D86" t="str">
-        <v>Dev</v>
+        <v>DevOps</v>
       </c>
       <c r="E86" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F86" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G86" t="str">
-        <v/>
+        <v>DevOps</v>
       </c>
       <c r="H86" t="str">
         <v/>
@@ -2906,28 +2906,28 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>Pranav Singh</v>
+        <v>Rida Maryam Mohammad</v>
       </c>
       <c r="B87" t="str">
-        <v>pranav.s.singh@pwc.com</v>
+        <v/>
       </c>
       <c r="C87" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D87" t="str">
-        <v>Integration Dev</v>
+        <v>Dev</v>
       </c>
       <c r="E87" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F87" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G87" t="str">
-        <v>Integration</v>
+        <v>Release</v>
       </c>
       <c r="H87" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I87" t="str">
         <v>No</v>
@@ -2935,28 +2935,28 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>Pranay Reddy</v>
+        <v>Rinky Chawla</v>
       </c>
       <c r="B88" t="str">
-        <v/>
+        <v>rinky.chawla@pwc.com</v>
       </c>
       <c r="C88" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D88" t="str">
-        <v>Dev</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E88" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F88" t="str">
-        <v/>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G88" t="str">
-        <v/>
+        <v>Case Management</v>
       </c>
       <c r="H88" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I88" t="str">
         <v>No</v>
@@ -2964,25 +2964,25 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>Prasad P</v>
+        <v>Ritesh Nanda</v>
       </c>
       <c r="B89" t="str">
-        <v/>
+        <v>ritesh.nanda@pwc.com</v>
       </c>
       <c r="C89" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D89" t="str">
-        <v>Dev</v>
+        <v>DevOps Lead</v>
       </c>
       <c r="E89" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F89" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G89" t="str">
-        <v/>
+        <v>DevOps</v>
       </c>
       <c r="H89" t="str">
         <v/>
@@ -2993,7 +2993,7 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>Prasanna</v>
+        <v>Rodolfo Duarte</v>
       </c>
       <c r="B90" t="str">
         <v/>
@@ -3002,19 +3002,19 @@
         <v/>
       </c>
       <c r="D90" t="str">
-        <v>QA</v>
+        <v>Team</v>
       </c>
       <c r="E90" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F90" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G90" t="str">
-        <v/>
+        <v>DevOps POD</v>
       </c>
       <c r="H90" t="str">
-        <v/>
+        <v>DevOps POD</v>
       </c>
       <c r="I90" t="str">
         <v>No</v>
@@ -3022,25 +3022,25 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>Prasanna Nangnure</v>
+        <v>Rohan Bandla</v>
       </c>
       <c r="B91" t="str">
-        <v>prasanna.y.nangnure@pwc.com</v>
+        <v/>
       </c>
       <c r="C91" t="str">
-        <v>Associate</v>
+        <v>Senior Associate</v>
       </c>
       <c r="D91" t="str">
-        <v>QA</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E91" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F91" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G91" t="str">
-        <v>Billing Programs</v>
+        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
       </c>
       <c r="H91" t="str">
         <v/>
@@ -3051,10 +3051,10 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>Pratik Kurdukar</v>
+        <v>Rubasri S</v>
       </c>
       <c r="B92" t="str">
-        <v>pratik.k.kurdukar@pwc.com</v>
+        <v>rubasri.x.s@pwc.com</v>
       </c>
       <c r="C92" t="str">
         <v>Associate</v>
@@ -3063,13 +3063,13 @@
         <v>Dev</v>
       </c>
       <c r="E92" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F92" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="G92" t="str">
-        <v>Case Management</v>
+        <v>Billing &amp; Usage/Payment Programs</v>
       </c>
       <c r="H92" t="str">
         <v/>
@@ -3080,28 +3080,28 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>Pratik Mahajan</v>
+        <v>Sagnik Chakraborty</v>
       </c>
       <c r="B93" t="str">
-        <v>pratik.sunil.mahajan@pwc.com</v>
+        <v>sagnik.chakraborty@pwc.com</v>
       </c>
       <c r="C93" t="str">
-        <v>Senior Associate</v>
+        <v>Associate</v>
       </c>
       <c r="D93" t="str">
         <v>QA</v>
       </c>
       <c r="E93" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F93" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G93" t="str">
-        <v>Interactions/Search</v>
+        <v>Energy Management</v>
       </c>
       <c r="H93" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I93" t="str">
         <v>No</v>
@@ -3109,28 +3109,28 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>Prayas Abinash</v>
+        <v>Sahithi Manne</v>
       </c>
       <c r="B94" t="str">
         <v/>
       </c>
       <c r="C94" t="str">
-        <v/>
+        <v>Infosys</v>
       </c>
       <c r="D94" t="str">
-        <v>Offshore Solution Analyst</v>
+        <v>Onshore SA</v>
       </c>
       <c r="E94" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F94" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="G94" t="str">
-        <v/>
+        <v>Billing &amp; Usage/Payment Programs | Energy Management</v>
       </c>
       <c r="H94" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I94" t="str">
         <v>No</v>
@@ -3138,25 +3138,25 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>Pritam</v>
+        <v>Sandesh Saravanan</v>
       </c>
       <c r="B95" t="str">
-        <v/>
+        <v>sandesh.saravanan@pwc.com</v>
       </c>
       <c r="C95" t="str">
-        <v>Infosys</v>
+        <v>Intern</v>
       </c>
       <c r="D95" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E95" t="str">
         <v>IR3.2</v>
       </c>
       <c r="F95" t="str">
-        <v>All</v>
+        <v>IR3.2</v>
       </c>
       <c r="G95" t="str">
-        <v>Account Maintenance</v>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H95" t="str">
         <v/>
@@ -3167,16 +3167,16 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>Rajaraman A</v>
+        <v>Sanjana</v>
       </c>
       <c r="B96" t="str">
-        <v>rajaraman.a@pwc.com</v>
+        <v/>
       </c>
       <c r="C96" t="str">
-        <v>Manager</v>
+        <v>Infosys</v>
       </c>
       <c r="D96" t="str">
-        <v>QA Lead</v>
+        <v>QA</v>
       </c>
       <c r="E96" t="str">
         <v>IR3.2</v>
@@ -3185,7 +3185,7 @@
         <v>All</v>
       </c>
       <c r="G96" t="str">
-        <v>QA - All Value Streams</v>
+        <v>Interactions/Search</v>
       </c>
       <c r="H96" t="str">
         <v/>
@@ -3196,25 +3196,25 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>Ramya Kothuri</v>
+        <v>Sanket Mundargi</v>
       </c>
       <c r="B97" t="str">
-        <v/>
+        <v>sanket.mundargi@pwc.com</v>
       </c>
       <c r="C97" t="str">
-        <v/>
+        <v>Associate</v>
       </c>
       <c r="D97" t="str">
-        <v>Scrum Master</v>
+        <v>Windsurf/Performance Dev</v>
       </c>
       <c r="E97" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F97" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G97" t="str">
-        <v/>
+        <v>Windsurf/Performance</v>
       </c>
       <c r="H97" t="str">
         <v/>
@@ -3225,28 +3225,28 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>Raveendra Reddy</v>
+        <v>Sanniboina Murali Krishna</v>
       </c>
       <c r="B98" t="str">
-        <v>raveendra.t.reddy@pwc.com</v>
+        <v/>
       </c>
       <c r="C98" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D98" t="str">
-        <v>QA</v>
+        <v>Dev</v>
       </c>
       <c r="E98" t="str">
-        <v>IR3.2</v>
+        <v>IR4</v>
       </c>
       <c r="F98" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G98" t="str">
-        <v>Transfer</v>
+        <v>Release</v>
       </c>
       <c r="H98" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I98" t="str">
         <v>No</v>
@@ -3254,10 +3254,10 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>Rhitik Khanna</v>
+        <v>Santosh Kumar Jangam</v>
       </c>
       <c r="B99" t="str">
-        <v>rhitik.khanna@pwc.com</v>
+        <v>santosh.kumar.jangam@pwc.com</v>
       </c>
       <c r="C99" t="str">
         <v>Senior Associate</v>
@@ -3283,25 +3283,25 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>Rida Maryam Mohammad</v>
+        <v>Shabnam Nasreen</v>
       </c>
       <c r="B100" t="str">
-        <v/>
+        <v>shabnam.nasreen@pwc.com</v>
       </c>
       <c r="C100" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D100" t="str">
-        <v>Dev</v>
+        <v>DevOps Lead</v>
       </c>
       <c r="E100" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F100" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G100" t="str">
-        <v/>
+        <v>DevOps</v>
       </c>
       <c r="H100" t="str">
         <v/>
@@ -3312,25 +3312,25 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>Rinky Chawla</v>
+        <v>Shanta Samlal</v>
       </c>
       <c r="B101" t="str">
-        <v>rinky.chawla@pwc.com</v>
+        <v>shanta.samlal@pwc.com</v>
       </c>
       <c r="C101" t="str">
         <v>Manager</v>
       </c>
       <c r="D101" t="str">
-        <v>Dev Lead</v>
+        <v>PMO</v>
       </c>
       <c r="E101" t="str">
-        <v>IR3.2</v>
+        <v>Leadership</v>
       </c>
       <c r="F101" t="str">
-        <v>IR3.2/IR4</v>
+        <v>All</v>
       </c>
       <c r="G101" t="str">
-        <v>Case Management</v>
+        <v>PMO</v>
       </c>
       <c r="H101" t="str">
         <v/>
@@ -3341,16 +3341,16 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>Ritesh Nanda</v>
+        <v>Shatakshi Srivastava</v>
       </c>
       <c r="B102" t="str">
-        <v>ritesh.nanda@pwc.com</v>
+        <v>shatakshi.s.srivastava@pwc.com</v>
       </c>
       <c r="C102" t="str">
         <v>Manager</v>
       </c>
       <c r="D102" t="str">
-        <v>DevOps Lead</v>
+        <v>DevOps</v>
       </c>
       <c r="E102" t="str">
         <v>Cross-Functional</v>
@@ -3370,28 +3370,28 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>Rodolfo Duarte</v>
+        <v>Shikhar Sanjeev</v>
       </c>
       <c r="B103" t="str">
-        <v/>
+        <v>shikhar.sanjeev@pwc.com</v>
       </c>
       <c r="C103" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D103" t="str">
-        <v>Team</v>
+        <v>Dev</v>
       </c>
       <c r="E103" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F103" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="G103" t="str">
-        <v/>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H103" t="str">
-        <v/>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I103" t="str">
         <v>No</v>
@@ -3399,16 +3399,16 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>Rohan Bandla</v>
+        <v>Shivam Surendra Shete</v>
       </c>
       <c r="B104" t="str">
-        <v/>
+        <v>shivam.surendra.shete@pwc.com</v>
       </c>
       <c r="C104" t="str">
         <v>Senior Associate</v>
       </c>
       <c r="D104" t="str">
-        <v>Onshore SA</v>
+        <v>Dev</v>
       </c>
       <c r="E104" t="str">
         <v>IR4</v>
@@ -3417,7 +3417,7 @@
         <v>IR4</v>
       </c>
       <c r="G104" t="str">
-        <v>Correspondence/360s/PEXT/Customer Auth/Account Maintenance</v>
+        <v>Billing &amp; Usage/Payment Programs</v>
       </c>
       <c r="H104" t="str">
         <v/>
@@ -3428,13 +3428,13 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>Rubasri S</v>
+        <v>Shravya Nanjundaswamy</v>
       </c>
       <c r="B105" t="str">
-        <v>rubasri.x.s@pwc.com</v>
+        <v/>
       </c>
       <c r="C105" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D105" t="str">
         <v>Dev</v>
@@ -3446,10 +3446,10 @@
         <v>IR4</v>
       </c>
       <c r="G105" t="str">
-        <v>Billing &amp; Usage/Payment Programs</v>
+        <v>Release</v>
       </c>
       <c r="H105" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I105" t="str">
         <v>No</v>
@@ -3457,28 +3457,28 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>Russell Stein</v>
+        <v>Shreya LNU</v>
       </c>
       <c r="B106" t="str">
-        <v/>
+        <v>shreya.l.lnu@pwc.com</v>
       </c>
       <c r="C106" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D106" t="str">
-        <v>Onshore Solution Analyst</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E106" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F106" t="str">
-        <v/>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G106" t="str">
-        <v/>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H106" t="str">
-        <v/>
+        <v>Dev POD 1/Shreya</v>
       </c>
       <c r="I106" t="str">
         <v>No</v>
@@ -3486,25 +3486,25 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>Sagnik Chakraborty</v>
+        <v>Smita</v>
       </c>
       <c r="B107" t="str">
-        <v>sagnik.chakraborty@pwc.com</v>
+        <v/>
       </c>
       <c r="C107" t="str">
-        <v>Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D107" t="str">
         <v>QA</v>
       </c>
       <c r="E107" t="str">
-        <v>IR4</v>
+        <v>IR3.2</v>
       </c>
       <c r="F107" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G107" t="str">
-        <v>Energy Management</v>
+        <v>Payment &amp; Payment Options/Billing Programs</v>
       </c>
       <c r="H107" t="str">
         <v/>
@@ -3515,28 +3515,28 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>Sahil Thadani</v>
+        <v>Sneha Girigoudar</v>
       </c>
       <c r="B108" t="str">
-        <v/>
+        <v>sneha.raosaheb.girigoudar@pwc.com</v>
       </c>
       <c r="C108" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D108" t="str">
-        <v>Dev</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E108" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F108" t="str">
-        <v/>
+        <v>IR3.2/IR4</v>
       </c>
       <c r="G108" t="str">
-        <v/>
+        <v>Interactions/Search | Correspondence/360s/PEXT/Account Maintenance</v>
       </c>
       <c r="H108" t="str">
-        <v/>
+        <v>Dev POD 2/Sneha G</v>
       </c>
       <c r="I108" t="str">
         <v>No</v>
@@ -3544,25 +3544,25 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>Sahithi Chebrolu</v>
+        <v>Sonal Yadav</v>
       </c>
       <c r="B109" t="str">
-        <v/>
+        <v>sonal.y.yadav@pwc.com</v>
       </c>
       <c r="C109" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D109" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E109" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F109" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G109" t="str">
-        <v/>
+        <v>Move In/Move Out</v>
       </c>
       <c r="H109" t="str">
         <v/>
@@ -3573,16 +3573,16 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>Sahithi Manne</v>
+        <v>Sree Sowndarya Barani K</v>
       </c>
       <c r="B110" t="str">
         <v/>
       </c>
       <c r="C110" t="str">
-        <v>Infosys</v>
+        <v/>
       </c>
       <c r="D110" t="str">
-        <v>Onshore SA</v>
+        <v>Dev</v>
       </c>
       <c r="E110" t="str">
         <v>IR4</v>
@@ -3591,10 +3591,10 @@
         <v>IR4</v>
       </c>
       <c r="G110" t="str">
-        <v>Billing &amp; Usage/Payment Programs | Energy Management</v>
+        <v>Release</v>
       </c>
       <c r="H110" t="str">
-        <v/>
+        <v>Case Management POD</v>
       </c>
       <c r="I110" t="str">
         <v>No</v>
@@ -3602,7 +3602,7 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>Sama Balayeva</v>
+        <v>Sridaran N M</v>
       </c>
       <c r="B111" t="str">
         <v/>
@@ -3611,19 +3611,19 @@
         <v/>
       </c>
       <c r="D111" t="str">
-        <v>Onshore Solution Analyst</v>
+        <v>Dev</v>
       </c>
       <c r="E111" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F111" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="G111" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H111" t="str">
-        <v/>
+        <v>Dev POD 4/Jason</v>
       </c>
       <c r="I111" t="str">
         <v>No</v>
@@ -3631,25 +3631,25 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>Sandesh Saravanan</v>
+        <v>Sujith Pillai</v>
       </c>
       <c r="B112" t="str">
-        <v>sandesh.saravanan@pwc.com</v>
+        <v>sujith.s.pillai@pwc.com</v>
       </c>
       <c r="C112" t="str">
-        <v>Intern</v>
+        <v>Director</v>
       </c>
       <c r="D112" t="str">
-        <v>Dev</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E112" t="str">
-        <v>IR3.2</v>
+        <v>Leadership</v>
       </c>
       <c r="F112" t="str">
-        <v>IR3.2</v>
+        <v>All</v>
       </c>
       <c r="G112" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
+        <v>Program Leadership</v>
       </c>
       <c r="H112" t="str">
         <v/>
@@ -3660,28 +3660,28 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>Sanjana</v>
+        <v>Suraj Ghodmare</v>
       </c>
       <c r="B113" t="str">
-        <v/>
+        <v>suraj.ghodmare@pwc.com</v>
       </c>
       <c r="C113" t="str">
-        <v>Infosys</v>
+        <v>Manager</v>
       </c>
       <c r="D113" t="str">
-        <v>QA</v>
+        <v>Dev Lead</v>
       </c>
       <c r="E113" t="str">
         <v>IR3.2</v>
       </c>
       <c r="F113" t="str">
-        <v>All</v>
+        <v>IR3.2</v>
       </c>
       <c r="G113" t="str">
-        <v>Interactions/Search</v>
+        <v>Move In/Move Out/Transfer</v>
       </c>
       <c r="H113" t="str">
-        <v/>
+        <v>Dev POD 4/Suraj</v>
       </c>
       <c r="I113" t="str">
         <v>No</v>
@@ -3689,28 +3689,28 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>Sanket Mundargi</v>
+        <v>Surya Teja Poka</v>
       </c>
       <c r="B114" t="str">
-        <v>sanket.mundargi@pwc.com</v>
+        <v/>
       </c>
       <c r="C114" t="str">
-        <v>Associate</v>
+        <v/>
       </c>
       <c r="D114" t="str">
-        <v>Windsurf/Performance Dev</v>
+        <v>Dev</v>
       </c>
       <c r="E114" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F114" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G114" t="str">
-        <v>Windsurf/Performance</v>
+        <v>Release</v>
       </c>
       <c r="H114" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I114" t="str">
         <v>No</v>
@@ -3718,25 +3718,25 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>Sanniboina Murali Krishna</v>
+        <v>Susan Matthews</v>
       </c>
       <c r="B115" t="str">
-        <v/>
+        <v>susan.m.mathew@pwc.com</v>
       </c>
       <c r="C115" t="str">
-        <v/>
+        <v>Senior Manager</v>
       </c>
       <c r="D115" t="str">
-        <v>Dev</v>
+        <v>Business Architect</v>
       </c>
       <c r="E115" t="str">
-        <v/>
+        <v>Leadership</v>
       </c>
       <c r="F115" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G115" t="str">
-        <v/>
+        <v>Architecture</v>
       </c>
       <c r="H115" t="str">
         <v/>
@@ -3747,7 +3747,7 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>Santhosh Maduri</v>
+        <v>Sweta Sharma</v>
       </c>
       <c r="B116" t="str">
         <v/>
@@ -3756,19 +3756,19 @@
         <v/>
       </c>
       <c r="D116" t="str">
-        <v>Dev</v>
+        <v>Lead</v>
       </c>
       <c r="E116" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="F116" t="str">
-        <v/>
+        <v>IR4</v>
       </c>
       <c r="G116" t="str">
-        <v/>
+        <v>Release</v>
       </c>
       <c r="H116" t="str">
-        <v/>
+        <v>Dev POD 5/Sweta</v>
       </c>
       <c r="I116" t="str">
         <v>No</v>
@@ -3776,28 +3776,28 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>Santosh Kumar Jangam</v>
+        <v>TBD</v>
       </c>
       <c r="B117" t="str">
-        <v>santosh.kumar.jangam@pwc.com</v>
+        <v/>
       </c>
       <c r="C117" t="str">
-        <v>Senior Associate</v>
+        <v/>
       </c>
       <c r="D117" t="str">
-        <v>DevOps</v>
+        <v>Dev</v>
       </c>
       <c r="E117" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F117" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G117" t="str">
-        <v>DevOps</v>
+        <v>Release</v>
       </c>
       <c r="H117" t="str">
-        <v/>
+        <v>Dev POD 6/Aditya</v>
       </c>
       <c r="I117" t="str">
         <v>No</v>
@@ -3805,25 +3805,25 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>Shabnam Nasreen</v>
+        <v>Ted Capaldi</v>
       </c>
       <c r="B118" t="str">
-        <v>shabnam.nasreen@pwc.com</v>
+        <v>theodore.capaldi@pwc.com</v>
       </c>
       <c r="C118" t="str">
-        <v>Manager</v>
+        <v>Partner</v>
       </c>
       <c r="D118" t="str">
-        <v>DevOps Lead</v>
+        <v>Engagement Lead</v>
       </c>
       <c r="E118" t="str">
-        <v>Cross-Functional</v>
+        <v>Leadership</v>
       </c>
       <c r="F118" t="str">
         <v>All</v>
       </c>
       <c r="G118" t="str">
-        <v>DevOps</v>
+        <v>Program Leadership</v>
       </c>
       <c r="H118" t="str">
         <v/>
@@ -3834,16 +3834,16 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>Shanta Samlal</v>
+        <v>Tyaga Pati</v>
       </c>
       <c r="B119" t="str">
-        <v>shanta.samlal@pwc.com</v>
+        <v>tyaga.pati@pwc.com</v>
       </c>
       <c r="C119" t="str">
-        <v>Manager</v>
+        <v>Senior Manager</v>
       </c>
       <c r="D119" t="str">
-        <v>PMO</v>
+        <v>Solution Architect</v>
       </c>
       <c r="E119" t="str">
         <v>Leadership</v>
@@ -3852,7 +3852,7 @@
         <v>All</v>
       </c>
       <c r="G119" t="str">
-        <v>PMO</v>
+        <v>Architecture</v>
       </c>
       <c r="H119" t="str">
         <v/>
@@ -3863,25 +3863,25 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>Shashank Satvai</v>
+        <v>Vasudha Tandon</v>
       </c>
       <c r="B120" t="str">
-        <v/>
+        <v>vasudha.tandon@pwc.com</v>
       </c>
       <c r="C120" t="str">
-        <v/>
+        <v>Manager</v>
       </c>
       <c r="D120" t="str">
-        <v>Dev</v>
+        <v>Integration Dev</v>
       </c>
       <c r="E120" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F120" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G120" t="str">
-        <v/>
+        <v>Integration</v>
       </c>
       <c r="H120" t="str">
         <v/>
@@ -3892,28 +3892,28 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>Shatakshi Srivastava</v>
+        <v>Venkata Sai Harika Ambati</v>
       </c>
       <c r="B121" t="str">
-        <v>shatakshi.s.srivastava@pwc.com</v>
+        <v>venkata.sai.harika.ambati@pwc.com</v>
       </c>
       <c r="C121" t="str">
-        <v>Manager</v>
+        <v>Associate</v>
       </c>
       <c r="D121" t="str">
-        <v>DevOps</v>
+        <v>Dev</v>
       </c>
       <c r="E121" t="str">
-        <v>Cross-Functional</v>
+        <v>IR4</v>
       </c>
       <c r="F121" t="str">
-        <v>All</v>
+        <v>IR4</v>
       </c>
       <c r="G121" t="str">
-        <v>DevOps</v>
+        <v>Energy Management</v>
       </c>
       <c r="H121" t="str">
-        <v/>
+        <v>Dev POD 3/Anurag</v>
       </c>
       <c r="I121" t="str">
         <v>No</v>
@@ -3921,25 +3921,25 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>Shikhar Sanjeev</v>
+        <v>Venugopal Sinde</v>
       </c>
       <c r="B122" t="str">
-        <v>shikhar.sanjeev@pwc.com</v>
+        <v/>
       </c>
       <c r="C122" t="str">
-        <v>Senior Associate</v>
+        <v>Infosys</v>
       </c>
       <c r="D122" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E122" t="str">
         <v>IR3.2</v>
       </c>
       <c r="F122" t="str">
-        <v>IR3.2</v>
+        <v>All</v>
       </c>
       <c r="G122" t="str">
-        <v>Move In/Move Out/Transfer</v>
+        <v>Move In/Move Out</v>
       </c>
       <c r="H122" t="str">
         <v/>
@@ -3950,25 +3950,25 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>Shivam Shete</v>
+        <v>Vidyashree S R</v>
       </c>
       <c r="B123" t="str">
-        <v/>
+        <v>vidyashree.s.r@pwc.com</v>
       </c>
       <c r="C123" t="str">
-        <v/>
+        <v>Senior Associate</v>
       </c>
       <c r="D123" t="str">
-        <v>Dev</v>
+        <v>QA</v>
       </c>
       <c r="E123" t="str">
-        <v/>
+        <v>IR3.2</v>
       </c>
       <c r="F123" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G123" t="str">
-        <v/>
+        <v>Payment &amp; Payment Options</v>
       </c>
       <c r="H123" t="str">
         <v/>
@@ -3979,25 +3979,25 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>Shivam Surendra Shete</v>
+        <v>Vinay Vadrevu</v>
       </c>
       <c r="B124" t="str">
-        <v>shivam.surendra.shete@pwc.com</v>
+        <v/>
       </c>
       <c r="C124" t="str">
-        <v>Senior Associate</v>
+        <v>Associate</v>
       </c>
       <c r="D124" t="str">
-        <v>Dev</v>
+        <v>DevOps</v>
       </c>
       <c r="E124" t="str">
-        <v>IR4</v>
+        <v>Cross-Functional</v>
       </c>
       <c r="F124" t="str">
-        <v>IR4</v>
+        <v>All</v>
       </c>
       <c r="G124" t="str">
-        <v>Billing &amp; Usage/Payment Programs</v>
+        <v>DevOps</v>
       </c>
       <c r="H124" t="str">
         <v/>
@@ -4008,7 +4008,7 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>Shravya Nanjundaswamy</v>
+        <v>Ziyad Auti</v>
       </c>
       <c r="B125" t="str">
         <v/>
@@ -4017,839 +4017,27 @@
         <v/>
       </c>
       <c r="D125" t="str">
-        <v>Dev</v>
+        <v>Intern</v>
       </c>
       <c r="E125" t="str">
-        <v/>
+        <v>Cross-Functional</v>
       </c>
       <c r="F125" t="str">
-        <v/>
+        <v>All</v>
       </c>
       <c r="G125" t="str">
-        <v/>
+        <v>Interns</v>
       </c>
       <c r="H125" t="str">
-        <v/>
+        <v>Interns</v>
       </c>
       <c r="I125" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="str">
-        <v>Shreya LNU</v>
-      </c>
-      <c r="B126" t="str">
-        <v>shreya.l.lnu@pwc.com</v>
-      </c>
-      <c r="C126" t="str">
-        <v>Manager</v>
-      </c>
-      <c r="D126" t="str">
-        <v>Dev Lead</v>
-      </c>
-      <c r="E126" t="str">
-        <v>IR3.2</v>
-      </c>
-      <c r="F126" t="str">
-        <v>IR3.2/IR4</v>
-      </c>
-      <c r="G126" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
-      </c>
-      <c r="H126" t="str">
-        <v/>
-      </c>
-      <c r="I126" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="str">
-        <v>Shweta Tiwari</v>
-      </c>
-      <c r="B127" t="str">
-        <v/>
-      </c>
-      <c r="C127" t="str">
-        <v/>
-      </c>
-      <c r="D127" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E127" t="str">
-        <v/>
-      </c>
-      <c r="F127" t="str">
-        <v/>
-      </c>
-      <c r="G127" t="str">
-        <v/>
-      </c>
-      <c r="H127" t="str">
-        <v/>
-      </c>
-      <c r="I127" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="str">
-        <v>Smita</v>
-      </c>
-      <c r="B128" t="str">
-        <v/>
-      </c>
-      <c r="C128" t="str">
-        <v>Infosys</v>
-      </c>
-      <c r="D128" t="str">
-        <v>QA</v>
-      </c>
-      <c r="E128" t="str">
-        <v>IR3.2</v>
-      </c>
-      <c r="F128" t="str">
-        <v>All</v>
-      </c>
-      <c r="G128" t="str">
-        <v>Payment &amp; Payment Options/Billing Programs</v>
-      </c>
-      <c r="H128" t="str">
-        <v/>
-      </c>
-      <c r="I128" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="str">
-        <v>Sneha Girigoudar</v>
-      </c>
-      <c r="B129" t="str">
-        <v>sneha.raosaheb.girigoudar@pwc.com</v>
-      </c>
-      <c r="C129" t="str">
-        <v>Manager</v>
-      </c>
-      <c r="D129" t="str">
-        <v>Dev Lead</v>
-      </c>
-      <c r="E129" t="str">
-        <v>IR3.2</v>
-      </c>
-      <c r="F129" t="str">
-        <v>IR3.2/IR4</v>
-      </c>
-      <c r="G129" t="str">
-        <v>Interactions/Search | Correspondence/360s/PEXT/Account Maintenance</v>
-      </c>
-      <c r="H129" t="str">
-        <v/>
-      </c>
-      <c r="I129" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="str">
-        <v>Sona Muthayala</v>
-      </c>
-      <c r="B130" t="str">
-        <v/>
-      </c>
-      <c r="C130" t="str">
-        <v/>
-      </c>
-      <c r="D130" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E130" t="str">
-        <v/>
-      </c>
-      <c r="F130" t="str">
-        <v/>
-      </c>
-      <c r="G130" t="str">
-        <v/>
-      </c>
-      <c r="H130" t="str">
-        <v/>
-      </c>
-      <c r="I130" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="str">
-        <v>Sonal Yadav</v>
-      </c>
-      <c r="B131" t="str">
-        <v>sonal.y.yadav@pwc.com</v>
-      </c>
-      <c r="C131" t="str">
-        <v>Senior Associate</v>
-      </c>
-      <c r="D131" t="str">
-        <v>QA</v>
-      </c>
-      <c r="E131" t="str">
-        <v>IR3.2</v>
-      </c>
-      <c r="F131" t="str">
-        <v>All</v>
-      </c>
-      <c r="G131" t="str">
-        <v>Move In/Move Out</v>
-      </c>
-      <c r="H131" t="str">
-        <v/>
-      </c>
-      <c r="I131" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="str">
-        <v>Sree Sowndarya Barani K</v>
-      </c>
-      <c r="B132" t="str">
-        <v/>
-      </c>
-      <c r="C132" t="str">
-        <v/>
-      </c>
-      <c r="D132" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E132" t="str">
-        <v/>
-      </c>
-      <c r="F132" t="str">
-        <v/>
-      </c>
-      <c r="G132" t="str">
-        <v/>
-      </c>
-      <c r="H132" t="str">
-        <v/>
-      </c>
-      <c r="I132" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="str">
-        <v>Sridaran N M</v>
-      </c>
-      <c r="B133" t="str">
-        <v/>
-      </c>
-      <c r="C133" t="str">
-        <v/>
-      </c>
-      <c r="D133" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E133" t="str">
-        <v/>
-      </c>
-      <c r="F133" t="str">
-        <v/>
-      </c>
-      <c r="G133" t="str">
-        <v/>
-      </c>
-      <c r="H133" t="str">
-        <v/>
-      </c>
-      <c r="I133" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="str">
-        <v>Sriharsha Sambaraj</v>
-      </c>
-      <c r="B134" t="str">
-        <v/>
-      </c>
-      <c r="C134" t="str">
-        <v/>
-      </c>
-      <c r="D134" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E134" t="str">
-        <v/>
-      </c>
-      <c r="F134" t="str">
-        <v/>
-      </c>
-      <c r="G134" t="str">
-        <v/>
-      </c>
-      <c r="H134" t="str">
-        <v/>
-      </c>
-      <c r="I134" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="str">
-        <v>Sujith Pillai</v>
-      </c>
-      <c r="B135" t="str">
-        <v>sujith.s.pillai@pwc.com</v>
-      </c>
-      <c r="C135" t="str">
-        <v>Director</v>
-      </c>
-      <c r="D135" t="str">
-        <v>Engagement Lead</v>
-      </c>
-      <c r="E135" t="str">
-        <v>Leadership</v>
-      </c>
-      <c r="F135" t="str">
-        <v>All</v>
-      </c>
-      <c r="G135" t="str">
-        <v>Program Leadership</v>
-      </c>
-      <c r="H135" t="str">
-        <v/>
-      </c>
-      <c r="I135" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="str">
-        <v>Sunandha Sanda</v>
-      </c>
-      <c r="B136" t="str">
-        <v/>
-      </c>
-      <c r="C136" t="str">
-        <v/>
-      </c>
-      <c r="D136" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E136" t="str">
-        <v/>
-      </c>
-      <c r="F136" t="str">
-        <v/>
-      </c>
-      <c r="G136" t="str">
-        <v/>
-      </c>
-      <c r="H136" t="str">
-        <v/>
-      </c>
-      <c r="I136" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="str">
-        <v>Suraj Ghodmare</v>
-      </c>
-      <c r="B137" t="str">
-        <v>suraj.ghodmare@pwc.com</v>
-      </c>
-      <c r="C137" t="str">
-        <v>Manager</v>
-      </c>
-      <c r="D137" t="str">
-        <v>Dev Lead</v>
-      </c>
-      <c r="E137" t="str">
-        <v>IR3.2</v>
-      </c>
-      <c r="F137" t="str">
-        <v>IR3.2</v>
-      </c>
-      <c r="G137" t="str">
-        <v>Move In/Move Out/Transfer</v>
-      </c>
-      <c r="H137" t="str">
-        <v/>
-      </c>
-      <c r="I137" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="str">
-        <v>Surya Teja Poka</v>
-      </c>
-      <c r="B138" t="str">
-        <v/>
-      </c>
-      <c r="C138" t="str">
-        <v/>
-      </c>
-      <c r="D138" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E138" t="str">
-        <v/>
-      </c>
-      <c r="F138" t="str">
-        <v/>
-      </c>
-      <c r="G138" t="str">
-        <v/>
-      </c>
-      <c r="H138" t="str">
-        <v/>
-      </c>
-      <c r="I138" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="str">
-        <v>Susan Matthews</v>
-      </c>
-      <c r="B139" t="str">
-        <v>susan.m.mathew@pwc.com</v>
-      </c>
-      <c r="C139" t="str">
-        <v>Senior Manager</v>
-      </c>
-      <c r="D139" t="str">
-        <v>Business Architect</v>
-      </c>
-      <c r="E139" t="str">
-        <v>Leadership</v>
-      </c>
-      <c r="F139" t="str">
-        <v>All</v>
-      </c>
-      <c r="G139" t="str">
-        <v>Architecture</v>
-      </c>
-      <c r="H139" t="str">
-        <v/>
-      </c>
-      <c r="I139" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="str">
-        <v>Sweta Sharma</v>
-      </c>
-      <c r="B140" t="str">
-        <v/>
-      </c>
-      <c r="C140" t="str">
-        <v/>
-      </c>
-      <c r="D140" t="str">
-        <v>Lead</v>
-      </c>
-      <c r="E140" t="str">
-        <v/>
-      </c>
-      <c r="F140" t="str">
-        <v/>
-      </c>
-      <c r="G140" t="str">
-        <v/>
-      </c>
-      <c r="H140" t="str">
-        <v/>
-      </c>
-      <c r="I140" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="str">
-        <v>Tameka Robinson</v>
-      </c>
-      <c r="B141" t="str">
-        <v/>
-      </c>
-      <c r="C141" t="str">
-        <v/>
-      </c>
-      <c r="D141" t="str">
-        <v>Lead</v>
-      </c>
-      <c r="E141" t="str">
-        <v/>
-      </c>
-      <c r="F141" t="str">
-        <v/>
-      </c>
-      <c r="G141" t="str">
-        <v/>
-      </c>
-      <c r="H141" t="str">
-        <v/>
-      </c>
-      <c r="I141" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="str">
-        <v>Ted Capaldi</v>
-      </c>
-      <c r="B142" t="str">
-        <v>theodore.capaldi@pwc.com</v>
-      </c>
-      <c r="C142" t="str">
-        <v>Partner</v>
-      </c>
-      <c r="D142" t="str">
-        <v>Engagement Lead</v>
-      </c>
-      <c r="E142" t="str">
-        <v>Leadership</v>
-      </c>
-      <c r="F142" t="str">
-        <v>All</v>
-      </c>
-      <c r="G142" t="str">
-        <v>Program Leadership</v>
-      </c>
-      <c r="H142" t="str">
-        <v/>
-      </c>
-      <c r="I142" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="str">
-        <v>Tejaswini Pathade</v>
-      </c>
-      <c r="B143" t="str">
-        <v/>
-      </c>
-      <c r="C143" t="str">
-        <v/>
-      </c>
-      <c r="D143" t="str">
-        <v>Lead</v>
-      </c>
-      <c r="E143" t="str">
-        <v/>
-      </c>
-      <c r="F143" t="str">
-        <v/>
-      </c>
-      <c r="G143" t="str">
-        <v/>
-      </c>
-      <c r="H143" t="str">
-        <v/>
-      </c>
-      <c r="I143" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="str">
-        <v>Tyaga Pati</v>
-      </c>
-      <c r="B144" t="str">
-        <v>tyaga.pati@pwc.com</v>
-      </c>
-      <c r="C144" t="str">
-        <v>Senior Manager</v>
-      </c>
-      <c r="D144" t="str">
-        <v>Solution Architect</v>
-      </c>
-      <c r="E144" t="str">
-        <v>Leadership</v>
-      </c>
-      <c r="F144" t="str">
-        <v>All</v>
-      </c>
-      <c r="G144" t="str">
-        <v>Architecture</v>
-      </c>
-      <c r="H144" t="str">
-        <v/>
-      </c>
-      <c r="I144" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="str">
-        <v>Vamsi Papulo</v>
-      </c>
-      <c r="B145" t="str">
-        <v/>
-      </c>
-      <c r="C145" t="str">
-        <v/>
-      </c>
-      <c r="D145" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E145" t="str">
-        <v/>
-      </c>
-      <c r="F145" t="str">
-        <v/>
-      </c>
-      <c r="G145" t="str">
-        <v/>
-      </c>
-      <c r="H145" t="str">
-        <v/>
-      </c>
-      <c r="I145" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="str">
-        <v>Vasudha Tandon</v>
-      </c>
-      <c r="B146" t="str">
-        <v>vasudha.tandon@pwc.com</v>
-      </c>
-      <c r="C146" t="str">
-        <v>Manager</v>
-      </c>
-      <c r="D146" t="str">
-        <v>Integration Dev</v>
-      </c>
-      <c r="E146" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="F146" t="str">
-        <v>All</v>
-      </c>
-      <c r="G146" t="str">
-        <v>Integration</v>
-      </c>
-      <c r="H146" t="str">
-        <v/>
-      </c>
-      <c r="I146" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="str">
-        <v>Venkata Sai Harika Ambati</v>
-      </c>
-      <c r="B147" t="str">
-        <v>venkata.sai.harika.ambati@pwc.com</v>
-      </c>
-      <c r="C147" t="str">
-        <v>Associate</v>
-      </c>
-      <c r="D147" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E147" t="str">
-        <v>IR4</v>
-      </c>
-      <c r="F147" t="str">
-        <v>IR4</v>
-      </c>
-      <c r="G147" t="str">
-        <v>Energy Management</v>
-      </c>
-      <c r="H147" t="str">
-        <v/>
-      </c>
-      <c r="I147" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="str">
-        <v>Venugopal Sinde</v>
-      </c>
-      <c r="B148" t="str">
-        <v/>
-      </c>
-      <c r="C148" t="str">
-        <v>Infosys</v>
-      </c>
-      <c r="D148" t="str">
-        <v>QA</v>
-      </c>
-      <c r="E148" t="str">
-        <v>IR3.2</v>
-      </c>
-      <c r="F148" t="str">
-        <v>All</v>
-      </c>
-      <c r="G148" t="str">
-        <v>Move In/Move Out</v>
-      </c>
-      <c r="H148" t="str">
-        <v/>
-      </c>
-      <c r="I148" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="str">
-        <v>Vidyashree</v>
-      </c>
-      <c r="B149" t="str">
-        <v/>
-      </c>
-      <c r="C149" t="str">
-        <v/>
-      </c>
-      <c r="D149" t="str">
-        <v>QA</v>
-      </c>
-      <c r="E149" t="str">
-        <v/>
-      </c>
-      <c r="F149" t="str">
-        <v/>
-      </c>
-      <c r="G149" t="str">
-        <v/>
-      </c>
-      <c r="H149" t="str">
-        <v/>
-      </c>
-      <c r="I149" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="str">
-        <v>Vidyashree S R</v>
-      </c>
-      <c r="B150" t="str">
-        <v>vidyashree.s.r@pwc.com</v>
-      </c>
-      <c r="C150" t="str">
-        <v>Senior Associate</v>
-      </c>
-      <c r="D150" t="str">
-        <v>QA</v>
-      </c>
-      <c r="E150" t="str">
-        <v>IR3.2</v>
-      </c>
-      <c r="F150" t="str">
-        <v>All</v>
-      </c>
-      <c r="G150" t="str">
-        <v>Payment &amp; Payment Options</v>
-      </c>
-      <c r="H150" t="str">
-        <v/>
-      </c>
-      <c r="I150" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="str">
-        <v>Vinay Vadrevu</v>
-      </c>
-      <c r="B151" t="str">
-        <v/>
-      </c>
-      <c r="C151" t="str">
-        <v>Associate</v>
-      </c>
-      <c r="D151" t="str">
-        <v>DevOps</v>
-      </c>
-      <c r="E151" t="str">
-        <v>Cross-Functional</v>
-      </c>
-      <c r="F151" t="str">
-        <v>All</v>
-      </c>
-      <c r="G151" t="str">
-        <v>DevOps</v>
-      </c>
-      <c r="H151" t="str">
-        <v/>
-      </c>
-      <c r="I151" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="str">
-        <v>Yolanda Espinoza</v>
-      </c>
-      <c r="B152" t="str">
-        <v/>
-      </c>
-      <c r="C152" t="str">
-        <v/>
-      </c>
-      <c r="D152" t="str">
-        <v>Dev</v>
-      </c>
-      <c r="E152" t="str">
-        <v/>
-      </c>
-      <c r="F152" t="str">
-        <v/>
-      </c>
-      <c r="G152" t="str">
-        <v/>
-      </c>
-      <c r="H152" t="str">
-        <v/>
-      </c>
-      <c r="I152" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="str">
-        <v>Ziyad Auti</v>
-      </c>
-      <c r="B153" t="str">
-        <v/>
-      </c>
-      <c r="C153" t="str">
-        <v/>
-      </c>
-      <c r="D153" t="str">
-        <v>Intern</v>
-      </c>
-      <c r="E153" t="str">
-        <v/>
-      </c>
-      <c r="F153" t="str">
-        <v/>
-      </c>
-      <c r="G153" t="str">
-        <v/>
-      </c>
-      <c r="H153" t="str">
-        <v/>
-      </c>
-      <c r="I153" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I153"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I125"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>